<commit_message>
Indonesia: verified profile, partnerships tracker records and map
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ChEN58PbdXFZmwUoBZYBRb
</commit_message>
<xml_diff>
--- a/output/Partnerships_Tracker.xlsx
+++ b/output/Partnerships_Tracker.xlsx
@@ -231,8 +231,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tracker" displayName="Tracker" ref="A1:L59" headerRowCount="1">
-  <autoFilter ref="A1:L59"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tracker" displayName="Tracker" ref="A1:L96" headerRowCount="1">
+  <autoFilter ref="A1:L96"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Status"/>
     <tableColumn id="2" name="Country"/>
@@ -558,7 +558,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Scope: partnerships that are active, or ended or last active within the past five years. Last checked 2026-10-05.</t>
+          <t>Scope: partnerships that are active, or ended or last active within the past five years. Last checked 2026-10-07.</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Tracker!$A$2:$A$59,A5)</f>
+        <f>COUNTIF(Tracker!$A$2:$A$96,A5)</f>
         <v/>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF(Tracker!$A$2:$A$59,A6)</f>
+        <f>COUNTIF(Tracker!$A$2:$A$96,A6)</f>
         <v/>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Tracker!$A$2:$A$59,A7)</f>
+        <f>COUNTIF(Tracker!$A$2:$A$96,A7)</f>
         <v/>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -670,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4098,6 +4098,2140 @@
       <c r="L59" s="14" t="inlineStr">
         <is>
           <t>MD Anderson Cancer Center, undated</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C60" s="13" t="inlineStr">
+        <is>
+          <t>Cedars-Sinai</t>
+        </is>
+      </c>
+      <c r="D60" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E60" s="12" t="inlineStr">
+        <is>
+          <t>Eka Hospital Group</t>
+        </is>
+      </c>
+      <c r="F60" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G60" s="12" t="inlineStr">
+        <is>
+          <t>Cedars-Sinai and Eka Hospital Group signed a three-year memorandum of understanding in August 2022, starting with advisory services in emergency medicine and trauma care. Under the agreement, two Cedars-Sinai emergency nurses led a two-week teaching mission for nurses from Eka's seven hospitals in Jakarta.</t>
+        </is>
+      </c>
+      <c r="H60" s="12" t="inlineStr">
+        <is>
+          <t>2022-08</t>
+        </is>
+      </c>
+      <c r="I60" s="12" t="inlineStr"/>
+      <c r="J60" s="12" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="K60" s="12" t="inlineStr">
+        <is>
+          <t>Cedars-Sinai's story dated 20 December 2024 (date in the page's own data) reports the two nurses had recently returned from the teaching mission at Eka under the 2022 agreement. The three-year term nominally ran to about August 2025 and no renewal was found.</t>
+        </is>
+      </c>
+      <c r="L60" s="14" t="inlineStr">
+        <is>
+          <t>Cedars-Sinai, 2022-08-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C61" s="13" t="inlineStr">
+        <is>
+          <t>Harvard Medical School</t>
+        </is>
+      </c>
+      <c r="D61" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E61" s="12" t="inlineStr">
+        <is>
+          <t>Universitas Harkat Negeri and CISDI (Primary Healthcare Impact Lab)</t>
+        </is>
+      </c>
+      <c r="F61" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G61" s="12" t="inlineStr">
+        <is>
+          <t>Harvard Medical School co-founded the Primary Healthcare Impact Lab with CISDI, Universitas Harkat Negeri and PT Tamaris Hidro, launched in Jakarta on 7 May 2026. The lab works on primary care service delivery, research and leadership education in Kota Tegal, Kabupaten Tegal and Brebes, and Harvard Medical School supports the university's medical curriculum.</t>
+        </is>
+      </c>
+      <c r="H61" s="12" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="I61" s="12" t="inlineStr"/>
+      <c r="J61" s="12" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="K61" s="12" t="inlineStr">
+        <is>
+          <t>Suara.com reports the launch at BRIN in Jakarta on 7 May 2026, and CISDI's own page names Harvard Medical School as a founding partner working in Tegal and Brebes. Neither source names Brigham and Women's Hospital.</t>
+        </is>
+      </c>
+      <c r="L61" s="14" t="inlineStr">
+        <is>
+          <t>Suara.com, 2026-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C62" s="13" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center</t>
+        </is>
+      </c>
+      <c r="D62" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E62" s="12" t="inlineStr">
+        <is>
+          <t>Indonesian Ministry of Health and RS Kanker Dharmais</t>
+        </is>
+      </c>
+      <c r="F62" s="12" t="inlineStr">
+        <is>
+          <t>Government agreement</t>
+        </is>
+      </c>
+      <c r="G62" s="12" t="inlineStr">
+        <is>
+          <t>MD Anderson signed a memorandum of understanding with the Ministry of Health in February 2023 covering service comparison, training, research support and cancer data management, with Dharmais as implementing hospital. It runs Project NOTRE, a breast cancer ECHO telementoring program with Dharmais.</t>
+        </is>
+      </c>
+      <c r="H62" s="12" t="inlineStr">
+        <is>
+          <t>2023-02</t>
+        </is>
+      </c>
+      <c r="I62" s="12" t="inlineStr"/>
+      <c r="J62" s="12" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="K62" s="12" t="inlineStr">
+        <is>
+          <t>MD Anderson's ECHO program listing for Project NOTRE with Dharmais is dated 20 June 2025 for a session on 14 June 2025.</t>
+        </is>
+      </c>
+      <c r="L62" s="14" t="inlineStr">
+        <is>
+          <t>WHO Global Breast Cancer Initiative Community, 2025-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C63" s="13" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center</t>
+        </is>
+      </c>
+      <c r="D63" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E63" s="12" t="inlineStr">
+        <is>
+          <t>MRCCC Siloam Semanggi (Siloam Hospitals)</t>
+        </is>
+      </c>
+      <c r="F63" s="12" t="inlineStr">
+        <is>
+          <t>Advisory and consulting</t>
+        </is>
+      </c>
+      <c r="G63" s="12" t="inlineStr">
+        <is>
+          <t>MD Anderson provides strategic and clinical advisory support to MRCCC Siloam Semanggi from January 2026 to January 2027. It covers multidisciplinary care, patient navigation, quality assurance and breast and lung cancer programs.</t>
+        </is>
+      </c>
+      <c r="H63" s="12" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="I63" s="12" t="inlineStr"/>
+      <c r="J63" s="12" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="K63" s="12" t="inlineStr">
+        <is>
+          <t>Kontan, 31 March 2026, reports the advisory collaboration running January 2026 to January 2027, based on an MRCCC release.</t>
+        </is>
+      </c>
+      <c r="L63" s="14" t="inlineStr">
+        <is>
+          <t>Kontan, 2026-03-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B64" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C64" s="13" t="inlineStr">
+        <is>
+          <t>Mayo Clinic</t>
+        </is>
+      </c>
+      <c r="D64" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E64" s="12" t="inlineStr">
+        <is>
+          <t>IHC Rumah Sakit Pusat Pertamina (RSPP)</t>
+        </is>
+      </c>
+      <c r="F64" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G64" s="12" t="inlineStr">
+        <is>
+          <t>RSPP is the first Indonesian member of the Mayo Clinic Care Network, with access to eConsults, eTumor boards and Mayo health care consulting projects. RSPP physicians also visit Mayo Clinic campuses for knowledge exchange.</t>
+        </is>
+      </c>
+      <c r="H64" s="12" t="inlineStr">
+        <is>
+          <t>2023-01</t>
+        </is>
+      </c>
+      <c r="I64" s="12" t="inlineStr"/>
+      <c r="J64" s="12" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="K64" s="12" t="inlineStr">
+        <is>
+          <t>RSPP's own newsroom on 4 December 2024 describes an RSPP endocrinologist visiting Mayo Clinic Florida through the Care Network membership. Mayo announced the membership on 26 January 2023.</t>
+        </is>
+      </c>
+      <c r="L64" s="14" t="inlineStr">
+        <is>
+          <t>RS Pusat Pertamina, 2024-12-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B65" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C65" s="13" t="inlineStr">
+        <is>
+          <t>St. Jude Children's Research Hospital</t>
+        </is>
+      </c>
+      <c r="D65" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E65" s="12" t="inlineStr">
+        <is>
+          <t>RSUPN Dr. Cipto Mangunkusumo (RSCM) and Indonesian Ministry of Health</t>
+        </is>
+      </c>
+      <c r="F65" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G65" s="12" t="inlineStr">
+        <is>
+          <t>St. Jude Global has worked with Indonesia's pediatric oncology community for over 15 years and supports the Ministry of Health in drafting a national pediatric cancer control plan. Its Asia Pacific team visited RSCM in April 2026 to review services and exchange knowledge.</t>
+        </is>
+      </c>
+      <c r="H65" s="12" t="inlineStr"/>
+      <c r="I65" s="12" t="inlineStr"/>
+      <c r="J65" s="12" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="K65" s="12" t="inlineStr">
+        <is>
+          <t>The Ministry of Health hospital directorate reported on 8 April 2026 a St. Jude Global Asia Pacific visit to RSCM on 7 April 2026 to strengthen childhood cancer collaboration.</t>
+        </is>
+      </c>
+      <c r="L65" s="14" t="inlineStr">
+        <is>
+          <t>Kemenkes, 2026-04-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C66" s="13" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals</t>
+        </is>
+      </c>
+      <c r="D66" s="12" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E66" s="12" t="inlineStr">
+        <is>
+          <t>Mayapada Healthcare Group (Mayapada Hospital)</t>
+        </is>
+      </c>
+      <c r="F66" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G66" s="12" t="inlineStr">
+        <is>
+          <t>Apollo and Mayapada signed an MoU in New Delhi in January 2025 covering medical education, case proctorship, nurse and doctor training in India, and technology for the planned Mayapada Apollo Batam International Hospital. Two further MoUs in January 2026 added AI based preventive health and emergency nursing training.</t>
+        </is>
+      </c>
+      <c r="H66" s="12" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="I66" s="12" t="inlineStr"/>
+      <c r="J66" s="12" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="K66" s="12" t="inlineStr">
+        <is>
+          <t>Detik (20 January 2026) and JawaPos report the Apollo leadership visit to Batam and Jakarta on 7 to 9 January 2026 and two new MoUs signed on 8 January 2026 at Mayapada Hospital Jakarta Selatan.</t>
+        </is>
+      </c>
+      <c r="L66" s="14" t="inlineStr">
+        <is>
+          <t>JawaPos, 2026-01-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B67" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C67" s="13" t="inlineStr">
+        <is>
+          <t>Asia OneHealthcare (A1Health, formerly Columbia Asia Healthcare)</t>
+        </is>
+      </c>
+      <c r="D67" s="12" t="inlineStr">
+        <is>
+          <t>Malaysia</t>
+        </is>
+      </c>
+      <c r="E67" s="12" t="inlineStr">
+        <is>
+          <t>RS Premier Jatinegara, Bintaro and Surabaya and Columbia Asia hospitals</t>
+        </is>
+      </c>
+      <c r="F67" s="12" t="inlineStr">
+        <is>
+          <t>Ownership or management</t>
+        </is>
+      </c>
+      <c r="G67" s="12" t="inlineStr">
+        <is>
+          <t>Malaysia based hospital group A1Health owns and operates nine hospitals in Indonesia, including in Jakarta, Surabaya, Banten, Medan and Semarang. They include the three RS Premier hospitals it gained by buying Ramsay Sime Darby Health Care, which closed in 2024.</t>
+        </is>
+      </c>
+      <c r="H67" s="12" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I67" s="12" t="inlineStr"/>
+      <c r="J67" s="12" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="K67" s="12" t="inlineStr">
+        <is>
+          <t>The Edge Malaysia (2 February 2026) reports A1Health has nine hospitals in Indonesia; The Edge (6 September 2024) reports the rename and the completed acquisition of Ramsay Sime Darby Health Care.</t>
+        </is>
+      </c>
+      <c r="L67" s="14" t="inlineStr">
+        <is>
+          <t>The Edge Malaysia, 2026-02-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C68" s="13" t="inlineStr">
+        <is>
+          <t>Chung Shan Medical University (Taiwan)</t>
+        </is>
+      </c>
+      <c r="D68" s="12" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="E68" s="12" t="inlineStr">
+        <is>
+          <t>Universitas Indonesia</t>
+        </is>
+      </c>
+      <c r="F68" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G68" s="12" t="inlineStr">
+        <is>
+          <t>CSMU and Universitas Indonesia signed an MoU in August 2025 on faculty and student exchange, joint curriculum, research and clinical training, building on dental medicine exchanges with UI's Faculty of Dentistry since 2017.</t>
+        </is>
+      </c>
+      <c r="H68" s="12" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="I68" s="12" t="inlineStr"/>
+      <c r="J68" s="12" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="K68" s="12" t="inlineStr">
+        <is>
+          <t>CSMU's press page dated 8 August 2025 reports the MoU signed by both presidents.</t>
+        </is>
+      </c>
+      <c r="L68" s="14" t="inlineStr">
+        <is>
+          <t>Chung Shan Medical University, 2025-08-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B69" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C69" s="13" t="inlineStr">
+        <is>
+          <t>Hong Kong Asia Medical Group (HKAMG)</t>
+        </is>
+      </c>
+      <c r="D69" s="12" t="inlineStr">
+        <is>
+          <t>Hong Kong, China</t>
+        </is>
+      </c>
+      <c r="E69" s="12" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (PT Pertamedika Bali Hospital, IHC)</t>
+        </is>
+      </c>
+      <c r="F69" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G69" s="12" t="inlineStr">
+        <is>
+          <t>HKAMG, a private cardiovascular hospital group whose flagship is Wuhan Asia Heart Hospital, provides cardiology and clinical expertise to Bali International Hospital. Its specialists took part in the hospital's first TAVI procedures in March 2026, which HKAMG funded.</t>
+        </is>
+      </c>
+      <c r="H69" s="12" t="inlineStr"/>
+      <c r="I69" s="12" t="inlineStr"/>
+      <c r="J69" s="12" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="K69" s="12" t="inlineStr">
+        <is>
+          <t>ANTARA (9 March 2026) reports that the first TAVI procedures at Bali International Hospital on 7 March 2026 were supported by HKAMG, quoting HKAMG's CEO; BIH named HKAMG a partner on 25 April 2025.</t>
+        </is>
+      </c>
+      <c r="L69" s="14" t="inlineStr">
+        <is>
+          <t>ANTARA, 2026-03-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C70" s="13" t="inlineStr">
+        <is>
+          <t>Icon Group (Icon Cancer Centre)</t>
+        </is>
+      </c>
+      <c r="D70" s="12" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="E70" s="12" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (PT Pertamina Bina Medika IHC)</t>
+        </is>
+      </c>
+      <c r="F70" s="12" t="inlineStr">
+        <is>
+          <t>Ownership or management</t>
+        </is>
+      </c>
+      <c r="G70" s="12" t="inlineStr">
+        <is>
+          <t>Icon Cancer Centre operates the radiation oncology and cancer service inside Bali International Hospital in the Sanur special economic zone, with its own international doctors, the first allowed to practice in Indonesia. It treated its first patient on 7 May 2025.</t>
+        </is>
+      </c>
+      <c r="H70" s="12" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="I70" s="12" t="inlineStr"/>
+      <c r="J70" s="12" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="K70" s="12" t="inlineStr">
+        <is>
+          <t>Icon Group's release of 26 March 2026 reports the launch of the first stereotactic radiotherapy service and the first brachytherapy treatment at Icon Cancer Centre, Bali International Hospital.</t>
+        </is>
+      </c>
+      <c r="L70" s="14" t="inlineStr">
+        <is>
+          <t>Icon Group, 2026-03-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C71" s="13" t="inlineStr">
+        <is>
+          <t>International University of Health and Welfare (IUHW)</t>
+        </is>
+      </c>
+      <c r="D71" s="12" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="E71" s="12" t="inlineStr">
+        <is>
+          <t>Ministry of Health (Kemenkes)</t>
+        </is>
+      </c>
+      <c r="F71" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G71" s="12" t="inlineStr">
+        <is>
+          <t>The Ministry of Health and IUHW signed an MoU in April 2026 on postgraduate clinical training and specialist development, academic exchange and technical help from Japanese experts.</t>
+        </is>
+      </c>
+      <c r="H71" s="12" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="I71" s="12" t="inlineStr"/>
+      <c r="J71" s="12" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="K71" s="12" t="inlineStr">
+        <is>
+          <t>The Ministry of Health reports the MoU signed on 13 April 2026 by its Secretary General, Kunta Wibawa Dasa Nugraha, and IUHW President Yasuhiro Suzuki, witnessed by the health minister.</t>
+        </is>
+      </c>
+      <c r="L71" s="14" t="inlineStr">
+        <is>
+          <t>Kementerian Kesehatan RI, 2026-04-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B72" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C72" s="13" t="inlineStr">
+        <is>
+          <t>Monash Health</t>
+        </is>
+      </c>
+      <c r="D72" s="12" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="E72" s="12" t="inlineStr">
+        <is>
+          <t>RS Otak Dr. Drs. M. Hatta Bukittinggi (RSOMH, Ministry of Health brain hospital)</t>
+        </is>
+      </c>
+      <c r="F72" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G72" s="12" t="inlineStr">
+        <is>
+          <t>Monash Health and the national brain hospital in Bukittinggi signed an MoU in November 2024 and hold knowledge sharing sessions and clinical case reviews on multidisciplinary stroke rehabilitation. In September 2026 they discussed a wider joint program.</t>
+        </is>
+      </c>
+      <c r="H72" s="12" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="I72" s="12" t="inlineStr"/>
+      <c r="J72" s="12" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="K72" s="12" t="inlineStr">
+        <is>
+          <t>The Health Ministry's hospital directorate reports a 22 July 2026 stroke rehabilitation session under the November 2024 MoU, and meetings on 24 and 28 September 2026.</t>
+        </is>
+      </c>
+      <c r="L72" s="14" t="inlineStr">
+        <is>
+          <t>Ditjen Kesehatan Lanjutan, Kemenkes, 2026-07-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B73" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C73" s="13" t="inlineStr">
+        <is>
+          <t>National Center for Global Health and Medicine (NCGM) and Kobe University</t>
+        </is>
+      </c>
+      <c r="D73" s="12" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="E73" s="12" t="inlineStr">
+        <is>
+          <t>Universitas Airlangga (Institute of Tropical Disease and RS Universitas Airlangga)</t>
+        </is>
+      </c>
+      <c r="F73" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G73" s="12" t="inlineStr">
+        <is>
+          <t>Japanese institutions work with Universitas Airlangga on infectious disease research through the J-GRID program, running since 2007 and renewed in 2015. A delegation visit to Unair Hospital in February 2025 explored widening it.</t>
+        </is>
+      </c>
+      <c r="H73" s="12" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="I73" s="12" t="inlineStr"/>
+      <c r="J73" s="12" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="K73" s="12" t="inlineStr">
+        <is>
+          <t>Unair News (20 February 2025) reports the 19 February 2025 visit of NCGM and Kobe University staff and the hospital director describing continued J-GRID research collaboration.</t>
+        </is>
+      </c>
+      <c r="L73" s="14" t="inlineStr">
+        <is>
+          <t>Universitas Airlangga, 2025-02-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B74" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C74" s="13" t="inlineStr">
+        <is>
+          <t>Ramathibodi Hospital, Mahidol University</t>
+        </is>
+      </c>
+      <c r="D74" s="12" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="E74" s="12" t="inlineStr">
+        <is>
+          <t>Faculty of Medicine Universitas Indonesia and RSCM</t>
+        </is>
+      </c>
+      <c r="F74" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G74" s="12" t="inlineStr">
+        <is>
+          <t>Ramathibodi and FMUI-RSCM signed an MoU in May 2025 for clinical training and academic cooperation, with an initial focus on urology and endoscopic surgical education.</t>
+        </is>
+      </c>
+      <c r="H74" s="12" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="I74" s="12" t="inlineStr"/>
+      <c r="J74" s="12" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="K74" s="12" t="inlineStr">
+        <is>
+          <t>Ramathibodi's international office reports the MoU signing on 21 May 2025 at the Faculty of Medicine Ramathibodi Hospital.</t>
+        </is>
+      </c>
+      <c r="L74" s="14" t="inlineStr">
+        <is>
+          <t>Ramathibodi Hospital, Mahidol University, 2025-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B75" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C75" s="13" t="inlineStr">
+        <is>
+          <t>Sapporo Cardio Vascular Clinic</t>
+        </is>
+      </c>
+      <c r="D75" s="12" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="E75" s="12" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (PT Pertamedika Bali Hospital, IHC)</t>
+        </is>
+      </c>
+      <c r="F75" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G75" s="12" t="inlineStr">
+        <is>
+          <t>Sapporo Cardio Vascular Clinic provides cardiology expertise to Bali International Hospital and introduced itself in Indonesia with the hospital's first TAVI procedures in March 2026. A Sapporo cardiovascular center also hosts Indonesian cardiologists on Ministry of Health fellowships.</t>
+        </is>
+      </c>
+      <c r="H75" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="I75" s="12" t="inlineStr"/>
+      <c r="J75" s="12" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="K75" s="12" t="inlineStr">
+        <is>
+          <t>Investor Daily (17 March 2026) reports two TAVI procedures on 7 March 2026 at Bali International Hospital, performed by an SCVC interventional cardiologist with HKAMG specialists, introducing SCVC's presence in Indonesia through its collaboration with the hospital. BIH named the clinic a cardiology partner on 25 April 2025.</t>
+        </is>
+      </c>
+      <c r="L75" s="14" t="inlineStr">
+        <is>
+          <t>investor.id, 2026-03-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B76" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C76" s="13" t="inlineStr">
+        <is>
+          <t>Seoul National University Hospital (SNUH)</t>
+        </is>
+      </c>
+      <c r="D76" s="12" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="E76" s="12" t="inlineStr">
+        <is>
+          <t>Faculty of Medicine Universitas Indonesia and RSUPN Dr. Cipto Mangunkusumo (RSCM)</t>
+        </is>
+      </c>
+      <c r="F76" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G76" s="12" t="inlineStr">
+        <is>
+          <t>SNUH, Universitas Indonesia and RSCM signed an MoU in July 2024 covering joint research, academic exchange, online education and staff and student exchange. SNUH's urology department signed a five-year implementation agreement with FMUI and RSCM on 13 January 2025.</t>
+        </is>
+      </c>
+      <c r="H76" s="12" t="inlineStr">
+        <is>
+          <t>2024-07</t>
+        </is>
+      </c>
+      <c r="I76" s="12" t="inlineStr"/>
+      <c r="J76" s="12" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="K76" s="12" t="inlineStr">
+        <is>
+          <t>Medipharm Health (4 February 2025) reports the implementation agreement signed on 13 January 2025 as a follow-up to the July 2024 MoU.</t>
+        </is>
+      </c>
+      <c r="L76" s="14" t="inlineStr">
+        <is>
+          <t>Medipharm Health News, 2025-02-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B77" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C77" s="13" t="inlineStr">
+        <is>
+          <t>Seoul National University Hospital (SNUH)</t>
+        </is>
+      </c>
+      <c r="D77" s="12" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="E77" s="12" t="inlineStr">
+        <is>
+          <t>RSUP Fatmawati (Ministry of Health hospital)</t>
+        </is>
+      </c>
+      <c r="F77" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G77" s="12" t="inlineStr">
+        <is>
+          <t>Fatmawati and SNUH signed an MoU in March 2023, witnessed by the health minister, to build liver, kidney and orthopedic transplant capacity. Fatmawati's living donor liver transplant program is being developed with SNUH to build the skills of its medical staff.</t>
+        </is>
+      </c>
+      <c r="H77" s="12" t="inlineStr">
+        <is>
+          <t>2023-03</t>
+        </is>
+      </c>
+      <c r="I77" s="12" t="inlineStr"/>
+      <c r="J77" s="12" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="K77" s="12" t="inlineStr">
+        <is>
+          <t>The Health Ministry's release of 10 April 2026 on Fatmawati's third liver transplant (9 April 2026) says the program is developed through cooperation with SNUH.</t>
+        </is>
+      </c>
+      <c r="L77" s="14" t="inlineStr">
+        <is>
+          <t>Kementerian Kesehatan RI, 2026-04-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B78" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C78" s="13" t="inlineStr">
+        <is>
+          <t>SingHealth</t>
+        </is>
+      </c>
+      <c r="D78" s="12" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="E78" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia Healthcare Corporation (PT Pertamina Bina Medika) and Bali International Hospital</t>
+        </is>
+      </c>
+      <c r="F78" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G78" s="12" t="inlineStr">
+        <is>
+          <t>SingHealth and IHC signed an MoU in April 2024 on sharing clinical practice, hospital management, staff training and nursing transformation, aimed at supporting Bali International Hospital, where SingHealth is the academic partner for continuing medical education.</t>
+        </is>
+      </c>
+      <c r="H78" s="12" t="inlineStr">
+        <is>
+          <t>2024-04</t>
+        </is>
+      </c>
+      <c r="I78" s="12" t="inlineStr"/>
+      <c r="J78" s="12" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="K78" s="12" t="inlineStr">
+        <is>
+          <t>Bali International Hospital's press release of 25 April 2025 names SingHealth as its academic partner for continuing medical education and clinical advancement.</t>
+        </is>
+      </c>
+      <c r="L78" s="14" t="inlineStr">
+        <is>
+          <t>Bali.com, 2025-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B79" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C79" s="13" t="inlineStr">
+        <is>
+          <t>SingHealth Duke-NUS Global Health Institute (SingHealth and Duke-NUS Medical School)</t>
+        </is>
+      </c>
+      <c r="D79" s="12" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="E79" s="12" t="inlineStr">
+        <is>
+          <t>Universitas Sumatera Utara (Faculty of Medicine)</t>
+        </is>
+      </c>
+      <c r="F79" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G79" s="12" t="inlineStr">
+        <is>
+          <t>SingHealth and the National University of Singapore (Duke-NUS) signed a partnership with USU in July 2023 on global health research, education and capacity building. The institute and USU's medical faculty ran a joint international summer course in July 2025.</t>
+        </is>
+      </c>
+      <c r="H79" s="12" t="inlineStr">
+        <is>
+          <t>2023-07</t>
+        </is>
+      </c>
+      <c r="I79" s="12" t="inlineStr"/>
+      <c r="J79" s="12" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="K79" s="12" t="inlineStr">
+        <is>
+          <t>USU reports the summer course with the SingHealth Duke-NUS Global Health Institute opened on 21 July 2025; USU's 8 August 2023 news item reports the partnership.</t>
+        </is>
+      </c>
+      <c r="L79" s="14" t="inlineStr">
+        <is>
+          <t>Universitas Sumatera Utara, 2025-08-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B80" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C80" s="13" t="inlineStr">
+        <is>
+          <t>Sun Medical Center (Sun Healthcare International)</t>
+        </is>
+      </c>
+      <c r="D80" s="12" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="E80" s="12" t="inlineStr">
+        <is>
+          <t>RSUP Prof. Dr. I.G.N.G. Ngoerah</t>
+        </is>
+      </c>
+      <c r="F80" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G80" s="12" t="inlineStr">
+        <is>
+          <t>Ngoerah hospital and Korea's Sun Medical Hospital signed an MoU in March 2023, witnessed by the health minister, to support health tourism in Bali. The health minister opened the Ngoerah Sun Wellness and Aesthetic Center, run in collaboration with Sun Healthcare International, on 3 October 2024.</t>
+        </is>
+      </c>
+      <c r="H80" s="12" t="inlineStr">
+        <is>
+          <t>2023-03</t>
+        </is>
+      </c>
+      <c r="I80" s="12" t="inlineStr"/>
+      <c r="J80" s="12" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="K80" s="12" t="inlineStr">
+        <is>
+          <t>Liputan6 (5 October 2024) reports the opening of the Ngoerah Sun Wellness and Aesthetic Center on 3 October 2024 in collaboration with Sun Healthcare International of South Korea.</t>
+        </is>
+      </c>
+      <c r="L80" s="14" t="inlineStr">
+        <is>
+          <t>Liputan6, 2024-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B81" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C81" s="13" t="inlineStr">
+        <is>
+          <t>Taipei Veterans General Hospital</t>
+        </is>
+      </c>
+      <c r="D81" s="12" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="E81" s="12" t="inlineStr">
+        <is>
+          <t>DKH Hospitals Group</t>
+        </is>
+      </c>
+      <c r="F81" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G81" s="12" t="inlineStr">
+        <is>
+          <t>TVGH and DKH Hospitals Group signed a two year MoU in May 2025 covering exchange of medical staff, research and clinical trials, telehealth, training and international patient referrals.</t>
+        </is>
+      </c>
+      <c r="H81" s="12" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="I81" s="12" t="inlineStr"/>
+      <c r="J81" s="12" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="K81" s="12" t="inlineStr">
+        <is>
+          <t>Antara, 23 May 2025, reports the MoU signed in Bogor on 23 May 2025, running two years with an option to extend.</t>
+        </is>
+      </c>
+      <c r="L81" s="14" t="inlineStr">
+        <is>
+          <t>Antara, 2025-05-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B82" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C82" s="13" t="inlineStr">
+        <is>
+          <t>Tokushukai Medical Group</t>
+        </is>
+      </c>
+      <c r="D82" s="12" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="E82" s="12" t="inlineStr">
+        <is>
+          <t>RSJPD Harapan Kita (National Heart Center) and Ministry of Health</t>
+        </is>
+      </c>
+      <c r="F82" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G82" s="12" t="inlineStr">
+        <is>
+          <t>Tokushukai has worked with Harapan Kita since 2004, exchanging doctors and knowledge, and signed a December 2023 agreement for a new cardiac building that the Health Ministry describes as a grant of about Rp 1 trillion. The building is planned as a center for cardiovascular education and international collaboration.</t>
+        </is>
+      </c>
+      <c r="H82" s="12" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="I82" s="12" t="inlineStr"/>
+      <c r="J82" s="12" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="K82" s="12" t="inlineStr">
+        <is>
+          <t>The Health Ministry reports the topping off ceremony for the Harapan Kita-Tokushukai Building on 15 April 2026, attended by the health minister, with a Da Vinci surgical robot due in November 2026.</t>
+        </is>
+      </c>
+      <c r="L82" s="14" t="inlineStr">
+        <is>
+          <t>Kementerian Kesehatan RI, 2026-04-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B83" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C83" s="13" t="inlineStr">
+        <is>
+          <t>Wuhan Asia Heart Hospital</t>
+        </is>
+      </c>
+      <c r="D83" s="12" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E83" s="12" t="inlineStr">
+        <is>
+          <t>Ministry of Health (Kemenkes)</t>
+        </is>
+      </c>
+      <c r="F83" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G83" s="12" t="inlineStr">
+        <is>
+          <t>Under a Ministry of Health fellowship program funded by LPDP, Indonesian cardiologists train in cardiac intervention for 12 months at Wuhan Asia Heart Hospital, the flagship of Hong Kong Asia Medical Group.</t>
+        </is>
+      </c>
+      <c r="H83" s="12" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="I83" s="12" t="inlineStr"/>
+      <c r="J83" s="12" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="K83" s="12" t="inlineStr">
+        <is>
+          <t>The Health Ministry's release of 12 November 2024 reports six of 13 cardiology fellows placed at Wuhan Asia Heart Hospital for 12 months.</t>
+        </is>
+      </c>
+      <c r="L83" s="14" t="inlineStr">
+        <is>
+          <t>Kementerian Kesehatan RI, 2024-11-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B84" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C84" s="13" t="inlineStr">
+        <is>
+          <t>Zhongda Hospital (Southeast University)</t>
+        </is>
+      </c>
+      <c r="D84" s="12" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E84" s="12" t="inlineStr">
+        <is>
+          <t>Ministry of Health (Kemenkes)</t>
+        </is>
+      </c>
+      <c r="F84" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G84" s="12" t="inlineStr">
+        <is>
+          <t>Zhongda Hospital is one of the named host hospitals for the Ministry of Health's one-year interventional cardiology and neurology fellowships.</t>
+        </is>
+      </c>
+      <c r="H84" s="12" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="I84" s="12" t="inlineStr"/>
+      <c r="J84" s="12" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="K84" s="12" t="inlineStr">
+        <is>
+          <t>The Health Ministry's release of 6 January 2025 names Zhongda Hospital among the hosts for 27 fellows.</t>
+        </is>
+      </c>
+      <c r="L84" s="14" t="inlineStr">
+        <is>
+          <t>Kementerian Kesehatan RI, 2025-01-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B85" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C85" s="13" t="inlineStr">
+        <is>
+          <t>Zhongshan Hospital (Fudan University)</t>
+        </is>
+      </c>
+      <c r="D85" s="12" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E85" s="12" t="inlineStr">
+        <is>
+          <t>Ministry of Health (Kemenkes)</t>
+        </is>
+      </c>
+      <c r="F85" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G85" s="12" t="inlineStr">
+        <is>
+          <t>Under a Ministry of Health cardiology fellowship program funded by LPDP, Indonesian cardiologists train in cardiac intervention for 12 months at Fudan University Zhongshan Hospital. The ministry signed a cooperation agreement with the hospital in June 2024.</t>
+        </is>
+      </c>
+      <c r="H85" s="12" t="inlineStr">
+        <is>
+          <t>2023-11</t>
+        </is>
+      </c>
+      <c r="I85" s="12" t="inlineStr"/>
+      <c r="J85" s="12" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="K85" s="12" t="inlineStr">
+        <is>
+          <t>The Health Ministry reports seven of 13 cardiology fellows placed at Zhongshan Hospital in November 2024, and names the hospital among hosts for a further 27 fellows sent on 6 January 2025.</t>
+        </is>
+      </c>
+      <c r="L85" s="14" t="inlineStr">
+        <is>
+          <t>Kementerian Kesehatan RI, 2025-01-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B86" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C86" s="13" t="inlineStr">
+        <is>
+          <t>Mayo Clinic</t>
+        </is>
+      </c>
+      <c r="D86" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E86" s="12" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (Indonesia Healthcare Corporation)</t>
+        </is>
+      </c>
+      <c r="F86" s="12" t="inlineStr">
+        <is>
+          <t>Advisory and consulting</t>
+        </is>
+      </c>
+      <c r="G86" s="12" t="inlineStr">
+        <is>
+          <t>Mayo Clinic Global Consulting advised on the planning and design of Bali International Hospital in the Sanur special economic zone. Mayo has said it acts only as a consultant and clinical knowledge partner and does not run the hospital.</t>
+        </is>
+      </c>
+      <c r="H86" s="12" t="inlineStr">
+        <is>
+          <t>2021-12</t>
+        </is>
+      </c>
+      <c r="I86" s="12" t="inlineStr"/>
+      <c r="J86" s="12" t="inlineStr">
+        <is>
+          <t>2023-03</t>
+        </is>
+      </c>
+      <c r="K86" s="12" t="inlineStr">
+        <is>
+          <t>The latest dated source found is the Jakarta Post of 17 March 2023, quoting a Mayo executive that Mayo is only a consultant. Bali International Hospital did not list Mayo among its international partners in its 25 April 2025 partner announcement, and no 2024 to 2026 evidence of continued advisory work was found.</t>
+        </is>
+      </c>
+      <c r="L86" s="14" t="inlineStr">
+        <is>
+          <t>The Jakarta Post, 2023-03-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B87" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C87" s="13" t="inlineStr">
+        <is>
+          <t>UCLA Health</t>
+        </is>
+      </c>
+      <c r="D87" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E87" s="12" t="inlineStr">
+        <is>
+          <t>RS Jantung dan Pembuluh Darah Harapan Kita</t>
+        </is>
+      </c>
+      <c r="F87" s="12" t="inlineStr">
+        <is>
+          <t>Advisory and consulting</t>
+        </is>
+      </c>
+      <c r="G87" s="12" t="inlineStr">
+        <is>
+          <t>UCLA Health worked with Harapan Kita on developing Indonesia's first heart transplant program, as the Ministry of Health reported when the hospital's new building opened in November 2022.</t>
+        </is>
+      </c>
+      <c r="H87" s="12" t="inlineStr"/>
+      <c r="I87" s="12" t="inlineStr"/>
+      <c r="J87" s="12" t="inlineStr">
+        <is>
+          <t>2022-11</t>
+        </is>
+      </c>
+      <c r="K87" s="12" t="inlineStr">
+        <is>
+          <t>The Ministry of Health release of the new Harapan Kita building launch in November 2022 names UCLA Health as a partner for heart transplant services. No newer dated evidence was found.</t>
+        </is>
+      </c>
+      <c r="L87" s="14" t="inlineStr">
+        <is>
+          <t>Kemenkes, 2022-11-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B88" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C88" s="13" t="inlineStr">
+        <is>
+          <t>Asan Medical Center</t>
+        </is>
+      </c>
+      <c r="D88" s="12" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="E88" s="12" t="inlineStr">
+        <is>
+          <t>Siloam Hospitals Group</t>
+        </is>
+      </c>
+      <c r="F88" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G88" s="12" t="inlineStr">
+        <is>
+          <t>Siloam and Asan Medical Center signed an MoU in November 2023 to develop clinical capability, with joint patient care, referrals and exchange of medical staff and researchers.</t>
+        </is>
+      </c>
+      <c r="H88" s="12" t="inlineStr">
+        <is>
+          <t>2023-11</t>
+        </is>
+      </c>
+      <c r="I88" s="12" t="inlineStr"/>
+      <c r="J88" s="12" t="inlineStr">
+        <is>
+          <t>2023-11</t>
+        </is>
+      </c>
+      <c r="K88" s="12" t="inlineStr">
+        <is>
+          <t>Kompas TV reports the MoU press conference held on 2 November 2023, attended by Ministry of Health officials. No newer dated evidence was found.</t>
+        </is>
+      </c>
+      <c r="L88" s="14" t="inlineStr">
+        <is>
+          <t>Kompas TV, 2023-11-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B89" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C89" s="13" t="inlineStr">
+        <is>
+          <t>Icon Group (Icon Cancer Centre, Singapore)</t>
+        </is>
+      </c>
+      <c r="D89" s="12" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="E89" s="12" t="inlineStr">
+        <is>
+          <t>RS Universitas Airlangga (RSUA)</t>
+        </is>
+      </c>
+      <c r="F89" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G89" s="12" t="inlineStr">
+        <is>
+          <t>Airlangga University Hospital and Icon Cancer Centre signed an agreement for medical exchange in cancer service, education and research in April 2023.</t>
+        </is>
+      </c>
+      <c r="H89" s="12" t="inlineStr">
+        <is>
+          <t>2023-04</t>
+        </is>
+      </c>
+      <c r="I89" s="12" t="inlineStr"/>
+      <c r="J89" s="12" t="inlineStr">
+        <is>
+          <t>2023-04</t>
+        </is>
+      </c>
+      <c r="K89" s="12" t="inlineStr">
+        <is>
+          <t>BioSpectrum Asia reports the signing on 10 April 2023; no newer dated activity was found.</t>
+        </is>
+      </c>
+      <c r="L89" s="14" t="inlineStr">
+        <is>
+          <t>BioSpectrum Asia, 2023-04-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B90" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C90" s="13" t="inlineStr">
+        <is>
+          <t>National Center for Global Health and Medicine (NCGM)</t>
+        </is>
+      </c>
+      <c r="D90" s="12" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="E90" s="12" t="inlineStr">
+        <is>
+          <t>Siloam Hospitals Group</t>
+        </is>
+      </c>
+      <c r="F90" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G90" s="12" t="inlineStr">
+        <is>
+          <t>NCGM and Siloam signed an MoU on clinical research cooperation in August 2022 and held a joint seminar to launch Siloam's new Clinical Research Department.</t>
+        </is>
+      </c>
+      <c r="H90" s="12" t="inlineStr">
+        <is>
+          <t>2022-08</t>
+        </is>
+      </c>
+      <c r="I90" s="12" t="inlineStr"/>
+      <c r="J90" s="12" t="inlineStr">
+        <is>
+          <t>2022-10</t>
+        </is>
+      </c>
+      <c r="K90" s="12" t="inlineStr">
+        <is>
+          <t>NCGM's news release of 7 October 2022 reports the MoU concluded on 13 August 2022; nothing newer was found.</t>
+        </is>
+      </c>
+      <c r="L90" s="14" t="inlineStr">
+        <is>
+          <t>NCGM, 2022-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B91" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C91" s="13" t="inlineStr">
+        <is>
+          <t>Peking Union Medical College Hospital</t>
+        </is>
+      </c>
+      <c r="D91" s="12" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E91" s="12" t="inlineStr">
+        <is>
+          <t>Ministry of Health (Kemenkes)</t>
+        </is>
+      </c>
+      <c r="F91" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G91" s="12" t="inlineStr">
+        <is>
+          <t>The Ministry of Health signed a cooperation agreement with PUMCH during its June 2024 China visit, alongside other Chinese hospitals.</t>
+        </is>
+      </c>
+      <c r="H91" s="12" t="inlineStr">
+        <is>
+          <t>2024-06</t>
+        </is>
+      </c>
+      <c r="I91" s="12" t="inlineStr"/>
+      <c r="J91" s="12" t="inlineStr">
+        <is>
+          <t>2024-06</t>
+        </is>
+      </c>
+      <c r="K91" s="12" t="inlineStr">
+        <is>
+          <t>Ministry of Health release dated 11 June 2024 names PUMCH among agreements signed. Content of the agreement is not detailed and nothing newer was found.</t>
+        </is>
+      </c>
+      <c r="L91" s="14" t="inlineStr">
+        <is>
+          <t>Ministry of Health, 2024-06-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B92" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C92" s="13" t="inlineStr">
+        <is>
+          <t>Rizhao Xinyi Hospital (Rizhao Heart Hospital)</t>
+        </is>
+      </c>
+      <c r="D92" s="12" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E92" s="12" t="inlineStr">
+        <is>
+          <t>Ministry of Health (Kemenkes)</t>
+        </is>
+      </c>
+      <c r="F92" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G92" s="12" t="inlineStr">
+        <is>
+          <t>A June 2024 letter of intent provides for sending Indonesian cardiovascular doctors, nurses and technicians to Rizhao for training over five years.</t>
+        </is>
+      </c>
+      <c r="H92" s="12" t="inlineStr">
+        <is>
+          <t>2024-06</t>
+        </is>
+      </c>
+      <c r="I92" s="12" t="inlineStr"/>
+      <c r="J92" s="12" t="inlineStr">
+        <is>
+          <t>2024-06</t>
+        </is>
+      </c>
+      <c r="K92" s="12" t="inlineStr">
+        <is>
+          <t>Ministry of Health release dated 11 June 2024. No newer dated evidence found.</t>
+        </is>
+      </c>
+      <c r="L92" s="14" t="inlineStr">
+        <is>
+          <t>Ministry of Health, 2024-06-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B93" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C93" s="13" t="inlineStr">
+        <is>
+          <t>Royal Brompton and Harefield Hospitals (Guy's and St Thomas' NHS Foundation Trust)</t>
+        </is>
+      </c>
+      <c r="D93" s="12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E93" s="12" t="inlineStr">
+        <is>
+          <t>Mandaya Royal Hospital Puri</t>
+        </is>
+      </c>
+      <c r="F93" s="12" t="inlineStr">
+        <is>
+          <t>Telehealth and second opinion</t>
+        </is>
+      </c>
+      <c r="G93" s="12" t="inlineStr">
+        <is>
+          <t>A November 2020 MoU gave Mandaya patients second opinions and teleconsultations with Royal Brompton clinicians, plus remote training and joint cardiorespiratory service development. A pediatric cardiac centre was launched with the partner in May 2023.</t>
+        </is>
+      </c>
+      <c r="H93" s="12" t="inlineStr">
+        <is>
+          <t>2020-11</t>
+        </is>
+      </c>
+      <c r="I93" s="12" t="inlineStr"/>
+      <c r="J93" s="12" t="inlineStr">
+        <is>
+          <t>2023-05</t>
+        </is>
+      </c>
+      <c r="K93" s="12" t="inlineStr">
+        <is>
+          <t>Mandaya's May 2023 inauguration of a pediatric cardiac centre with Royal Brompton and Harefield is the latest dated evidence found; nothing from October 2024 onward.</t>
+        </is>
+      </c>
+      <c r="L93" s="14" t="inlineStr">
+        <is>
+          <t>Mandaya Hospital Group, 2020-12-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B94" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C94" s="13" t="inlineStr">
+        <is>
+          <t>UMC Utrecht</t>
+        </is>
+      </c>
+      <c r="D94" s="12" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="E94" s="12" t="inlineStr">
+        <is>
+          <t>RS Jantung dan Pembuluh Darah Harapan Kita</t>
+        </is>
+      </c>
+      <c r="F94" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G94" s="12" t="inlineStr">
+        <is>
+          <t>The Health Ministry reported that Harapan Kita works with UMC Utrecht to develop heart failure services, alongside UCLA Health for heart transplantation.</t>
+        </is>
+      </c>
+      <c r="H94" s="12" t="inlineStr">
+        <is>
+          <t>2022-11</t>
+        </is>
+      </c>
+      <c r="I94" s="12" t="inlineStr"/>
+      <c r="J94" s="12" t="inlineStr">
+        <is>
+          <t>2022-11</t>
+        </is>
+      </c>
+      <c r="K94" s="12" t="inlineStr">
+        <is>
+          <t>The Health Ministry's release of 9 November 2022 on the new Harapan Kita building names UMC Utrecht; no newer dated evidence was found.</t>
+        </is>
+      </c>
+      <c r="L94" s="14" t="inlineStr">
+        <is>
+          <t>Kementerian Kesehatan RI, 2022-11-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="16" t="inlineStr">
+        <is>
+          <t>Ended</t>
+        </is>
+      </c>
+      <c r="B95" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C95" s="13" t="inlineStr">
+        <is>
+          <t>KPJ Healthcare</t>
+        </is>
+      </c>
+      <c r="D95" s="12" t="inlineStr">
+        <is>
+          <t>Malaysia</t>
+        </is>
+      </c>
+      <c r="E95" s="12" t="inlineStr">
+        <is>
+          <t>RS Medika BSD</t>
+        </is>
+      </c>
+      <c r="F95" s="12" t="inlineStr">
+        <is>
+          <t>Ownership or management</t>
+        </is>
+      </c>
+      <c r="G95" s="12" t="inlineStr">
+        <is>
+          <t>KPJ Healthcare managed RS Medika BSD until Columbia Asia acquired the hospital in September 2023 and renamed it RS Columbia Asia BSD.</t>
+        </is>
+      </c>
+      <c r="H95" s="12" t="inlineStr"/>
+      <c r="I95" s="12" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="J95" s="12" t="inlineStr">
+        <is>
+          <t>2023-10</t>
+        </is>
+      </c>
+      <c r="K95" s="12" t="inlineStr">
+        <is>
+          <t>Warta Ekonomi (2 October 2023) reports that RS Columbia Asia BSD resulted from the acquisition of RS Medika BSD, previously managed by KPJ Healthcare Group Malaysia; Kontan reports the acquisition on 19 September 2023.</t>
+        </is>
+      </c>
+      <c r="L95" s="14" t="inlineStr">
+        <is>
+          <t>Warta Ekonomi, 2023-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="16" t="inlineStr">
+        <is>
+          <t>Ended</t>
+        </is>
+      </c>
+      <c r="B96" s="12" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C96" s="13" t="inlineStr">
+        <is>
+          <t>Ramsay Health Care</t>
+        </is>
+      </c>
+      <c r="D96" s="12" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="E96" s="12" t="inlineStr">
+        <is>
+          <t>RS Premier Jatinegara, Bintaro and Surabaya</t>
+        </is>
+      </c>
+      <c r="F96" s="12" t="inlineStr">
+        <is>
+          <t>Ownership or management</t>
+        </is>
+      </c>
+      <c r="G96" s="12" t="inlineStr">
+        <is>
+          <t>Ramsay Health Care co-owned the three RS Premier hospitals through Ramsay Sime Darby Health Care, its 50:50 joint venture with Sime Darby, until the venture was sold to Columbia Asia (now A1Health).</t>
+        </is>
+      </c>
+      <c r="H96" s="12" t="inlineStr"/>
+      <c r="I96" s="12" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="J96" s="12" t="inlineStr">
+        <is>
+          <t>2024-09</t>
+        </is>
+      </c>
+      <c r="K96" s="12" t="inlineStr">
+        <is>
+          <t>The Edge (6 September 2024) reports that Columbia Asia had recently completed the purchase of Ramsay Sime Darby Health Care, which operated three hospitals in Indonesia, from Sime Darby and its Australian partner.</t>
+        </is>
+      </c>
+      <c r="L96" s="14" t="inlineStr">
+        <is>
+          <t>The Edge Malaysia, 2024-09-06</t>
         </is>
       </c>
     </row>
@@ -4161,10 +6295,47 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L96" r:id="rId95"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId59"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId96"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4175,7 +6346,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E117"/>
+  <dimension ref="A1:E187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -7337,6 +9508,1888 @@
       <c r="E117" s="5" t="inlineStr">
         <is>
           <t>https://www.mdanderson.org/education-training/outreach-programs/project-echo/programs/palliative-care-africa.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="5" t="inlineStr">
+        <is>
+          <t>Cedars-Sinai</t>
+        </is>
+      </c>
+      <c r="B118" s="5" t="inlineStr">
+        <is>
+          <t>Eka Hospital Group</t>
+        </is>
+      </c>
+      <c r="C118" s="5" t="inlineStr">
+        <is>
+          <t>Cedars-Sinai Cedars-Sinai International Launches Presence in Indonesia</t>
+        </is>
+      </c>
+      <c r="D118" s="5" t="inlineStr">
+        <is>
+          <t>2022-08-24</t>
+        </is>
+      </c>
+      <c r="E118" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cedars-sinai.org/blog/cedars-sinai-launches-collaboration-in-indonesia.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="inlineStr">
+        <is>
+          <t>Cedars-Sinai</t>
+        </is>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>Eka Hospital Group</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>Kompas Eka Hospital Group Jalin Kerja Sama dengan Cedars-Sinai Hospital</t>
+        </is>
+      </c>
+      <c r="D119" s="5" t="inlineStr">
+        <is>
+          <t>2022-08-25</t>
+        </is>
+      </c>
+      <c r="E119" s="5" t="inlineStr">
+        <is>
+          <t>https://biz.kompas.com/read/2022/08/25/121418528/eka-hospital-group-jalin-kerja-sama-dengan-cedars-sinai-hospital</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="5" t="inlineStr">
+        <is>
+          <t>Cedars-Sinai</t>
+        </is>
+      </c>
+      <c r="B120" s="5" t="inlineStr">
+        <is>
+          <t>Eka Hospital Group</t>
+        </is>
+      </c>
+      <c r="C120" s="5" t="inlineStr">
+        <is>
+          <t>Cedars-Sinai Staff Nurses Share Expertise with International EKA Hospital Group</t>
+        </is>
+      </c>
+      <c r="D120" s="5" t="inlineStr">
+        <is>
+          <t>2024-12-20</t>
+        </is>
+      </c>
+      <c r="E120" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cedars-sinai.org/international-stories/nurses-share-expertise-with-international-eka-hospital-group.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="5" t="inlineStr">
+        <is>
+          <t>Harvard Medical School</t>
+        </is>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>Universitas Harkat Negeri and CISDI (Primary Healthcare Impact Lab)</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>Bangun Santoso, Suara.com UHN dan CISDI Gandeng Harvard Medical School, Bangun Pusat Riset Kesehatan Primer di RI</t>
+        </is>
+      </c>
+      <c r="D121" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="E121" s="5" t="inlineStr">
+        <is>
+          <t>https://www.suara.com/news/2026/05/07/202619/uhn-dan-cisdi-gandeng-harvard-medical-school-bangun-pusat-riset-kesehatan-primer-di-ri</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="5" t="inlineStr">
+        <is>
+          <t>Harvard Medical School</t>
+        </is>
+      </c>
+      <c r="B122" s="5" t="inlineStr">
+        <is>
+          <t>Universitas Harkat Negeri and CISDI (Primary Healthcare Impact Lab)</t>
+        </is>
+      </c>
+      <c r="C122" s="5" t="inlineStr">
+        <is>
+          <t>CISDI Primary Healthcare IMPACT Lab</t>
+        </is>
+      </c>
+      <c r="D122" s="5" t="inlineStr"/>
+      <c r="E122" s="5" t="inlineStr">
+        <is>
+          <t>https://cisdi.org/en/our-works/phcimpactlab</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="5" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>Indonesian Ministry of Health and RS Kanker Dharmais</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center Project NOTRE (Indonesia Breast Cancer ECHO)</t>
+        </is>
+      </c>
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>2025-06-20</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="inlineStr">
+        <is>
+          <t>https://knowledge-action-portal.com/en/content/project-notre-indonesia-breast-cancer-echo-jun-14-2025-0300-pm-eest</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="5" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center</t>
+        </is>
+      </c>
+      <c r="B124" s="5" t="inlineStr">
+        <is>
+          <t>Indonesian Ministry of Health and RS Kanker Dharmais</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center MD Anderson announces new collaboration in Indonesia to reduce global cancer burden</t>
+        </is>
+      </c>
+      <c r="D124" s="5" t="inlineStr">
+        <is>
+          <t>2023-02-03</t>
+        </is>
+      </c>
+      <c r="E124" s="5" t="inlineStr">
+        <is>
+          <t>https://www.mdanderson.org/newsroom/md-anderson-announces-new-collaboration-in-indonesia.h00-159616278.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>Indonesian Ministry of Health and RS Kanker Dharmais</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>Kementerian Kesehatan RI Kemenkes dan MD Anderson Cancer Center Jalin Kerja Sama Atasi Kanker</t>
+        </is>
+      </c>
+      <c r="D125" s="5" t="inlineStr">
+        <is>
+          <t>2023-02-03</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="inlineStr">
+        <is>
+          <t>https://www.kemkes.go.id/eng/kemenkes-dan-md-anderson-cancer-center-jalin-kerja-sama-atasi-kanker</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="5" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center</t>
+        </is>
+      </c>
+      <c r="B126" s="5" t="inlineStr">
+        <is>
+          <t>MRCCC Siloam Semanggi (Siloam Hospitals)</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="inlineStr">
+        <is>
+          <t>Kontan Kesenjangan Layanan Kanker di Indonesia, MRCCC Siloam Menggandeng MD Anderson</t>
+        </is>
+      </c>
+      <c r="D126" s="5" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="E126" s="5" t="inlineStr">
+        <is>
+          <t>https://industri.kontan.co.id/news/kesenjangan-layanan-kanker-di-indonesia-mrccc-siloam-menggandeng-md-anderson</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="5" t="inlineStr">
+        <is>
+          <t>Mayo Clinic</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>IHC Rumah Sakit Pusat Pertamina (RSPP)</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>RS Pusat Pertamina Learning from the Best: IHC RSPP Endocrinologist Gains Insights into Innovative Medical Practices firsthand at Mayo Clinic's campus in Jacksonville, Florida</t>
+        </is>
+      </c>
+      <c r="D127" s="5" t="inlineStr">
+        <is>
+          <t>2024-12-04</t>
+        </is>
+      </c>
+      <c r="E127" s="5" t="inlineStr">
+        <is>
+          <t>https://rspp.co.id/artikel-detail-597-Learning-from-the-Best-IHC-RSPP-Endocrinologist-Gains-Insights-into-Innovative-Medical-Practices-firsthand-at-Mayo-Clinic’s-campus-in-Jacksonville,-Florida-.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="5" t="inlineStr">
+        <is>
+          <t>Mayo Clinic</t>
+        </is>
+      </c>
+      <c r="B128" s="5" t="inlineStr">
+        <is>
+          <t>IHC Rumah Sakit Pusat Pertamina (RSPP)</t>
+        </is>
+      </c>
+      <c r="C128" s="5" t="inlineStr">
+        <is>
+          <t>Mayo Clinic News Network IHC Rumah Sakit Pusat Pertamina in Indonesia joins Mayo Clinic Care Network</t>
+        </is>
+      </c>
+      <c r="D128" s="5" t="inlineStr">
+        <is>
+          <t>2023-01-26</t>
+        </is>
+      </c>
+      <c r="E128" s="5" t="inlineStr">
+        <is>
+          <t>https://newsnetwork.mayoclinic.org/discussion/ihc-rumah-sakit-pusat-pertamina-in-indonesia-joins-mayo-clinic-care-network</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="inlineStr">
+        <is>
+          <t>Mayo Clinic</t>
+        </is>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
+        <is>
+          <t>IHC Rumah Sakit Pusat Pertamina (RSPP)</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>RS Pusat Pertamina RSPP Gains Insight from Mayo Clinic for Outpatient Chemotherapy Unit</t>
+        </is>
+      </c>
+      <c r="D129" s="5" t="inlineStr">
+        <is>
+          <t>2023-08-14</t>
+        </is>
+      </c>
+      <c r="E129" s="5" t="inlineStr">
+        <is>
+          <t>https://rspp.co.id/artikel-detail-210-Rumah-Sakit-Pusat-Pertamina-(RSPP)-Gains-Insight-from-Mayo-Clinic-for-Outpatient-Chemotherapy-Unit-.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="5" t="inlineStr">
+        <is>
+          <t>St. Jude Children's Research Hospital</t>
+        </is>
+      </c>
+      <c r="B130" s="5" t="inlineStr">
+        <is>
+          <t>RSUPN Dr. Cipto Mangunkusumo (RSCM) and Indonesian Ministry of Health</t>
+        </is>
+      </c>
+      <c r="C130" s="5" t="inlineStr">
+        <is>
+          <t>Kementerian Kesehatan RI (Ditjen Kesehatan Lanjutan) RSUPN Dr Cipto Mangunkusumo Mendapat Kunjungan dari St Jude Global Asia Pacific Regional Untuk Perkuat Kolaborasi Kanker Anak</t>
+        </is>
+      </c>
+      <c r="D130" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="E130" s="5" t="inlineStr">
+        <is>
+          <t>https://keslan.kemkes.go.id/view_foto/554</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="inlineStr">
+        <is>
+          <t>St. Jude Children's Research Hospital</t>
+        </is>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>RSUPN Dr. Cipto Mangunkusumo (RSCM) and Indonesian Ministry of Health</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>St. Jude Children's Research Hospital St. Jude Global and Indonesian stakeholders unite for first-ever national childhood cancer policy planning</t>
+        </is>
+      </c>
+      <c r="D131" s="5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E131" s="5" t="inlineStr">
+        <is>
+          <t>https://stjude.org/research/progress/2024/st-jude-global-and-indonesian-stakeholders-unite-for-first-ever-national-childhood-cancer-policy-planning.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="5" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals</t>
+        </is>
+      </c>
+      <c r="B132" s="5" t="inlineStr">
+        <is>
+          <t>Mayapada Healthcare Group (Mayapada Hospital)</t>
+        </is>
+      </c>
+      <c r="C132" s="5" t="inlineStr">
+        <is>
+          <t>JawaPos Perkuat kolaborasi lintas negara, Mayapada Healthcare yakin bisa kurangi orang berobat ke luar negeri</t>
+        </is>
+      </c>
+      <c r="D132" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="E132" s="5" t="inlineStr">
+        <is>
+          <t>https://www.jawapos.com/kesehatan/2601230030/perkuat-kolaborasi-lintas-negara-mayapada-healthcare-yakin-bisa-kurangi-orang-berobat-ke-luar-negeri</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="5" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>Mayapada Healthcare Group (Mayapada Hospital)</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t>Detik Health Kolaborasi Klinis Mayapada Healthcare &amp; Apollo Hospitals India Kian Matang</t>
+        </is>
+      </c>
+      <c r="D133" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="E133" s="5" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/berita-detikhealth/d-8316666/kolaborasi-klinis-mayapada-healthcare-apollo-hospitals-india-kian-matang</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="5" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals</t>
+        </is>
+      </c>
+      <c r="B134" s="5" t="inlineStr">
+        <is>
+          <t>Mayapada Healthcare Group (Mayapada Hospital)</t>
+        </is>
+      </c>
+      <c r="C134" s="5" t="inlineStr">
+        <is>
+          <t>Investortrust Mayapada Healthcare Partners with India's Apollo Hospitals to Curb Medical Tourism</t>
+        </is>
+      </c>
+      <c r="D134" s="5" t="inlineStr">
+        <is>
+          <t>2025-01-29</t>
+        </is>
+      </c>
+      <c r="E134" s="5" t="inlineStr">
+        <is>
+          <t>https://investortrust.id/business/54719/mayapada-healthcare-partners-with-indias-apollo-hospitals-to-curb-medical-tourism</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>Asia OneHealthcare (A1Health, formerly Columbia Asia Healthcare)</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>RS Premier Jatinegara, Bintaro and Surabaya and Columbia Asia hospitals</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>The Edge Malaysia Weekly Bankers court A1Health for possible IPO</t>
+        </is>
+      </c>
+      <c r="D135" s="5" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="E135" s="5" t="inlineStr">
+        <is>
+          <t>https://theedgemalaysia.com/node/791491</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="5" t="inlineStr">
+        <is>
+          <t>Asia OneHealthcare (A1Health, formerly Columbia Asia Healthcare)</t>
+        </is>
+      </c>
+      <c r="B136" s="5" t="inlineStr">
+        <is>
+          <t>RS Premier Jatinegara, Bintaro and Surabaya and Columbia Asia hospitals</t>
+        </is>
+      </c>
+      <c r="C136" s="5" t="inlineStr">
+        <is>
+          <t>The Edge Malaysia Columbia Asia Healthcare renamed Asia OneHealthcare (A1Health) after consolidating assets in Malaysia, Indonesia and Vietnam</t>
+        </is>
+      </c>
+      <c r="D136" s="5" t="inlineStr">
+        <is>
+          <t>2024-09-06</t>
+        </is>
+      </c>
+      <c r="E136" s="5" t="inlineStr">
+        <is>
+          <t>https://theedgemalaysia.com/node/725855</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>Asia OneHealthcare (A1Health, formerly Columbia Asia Healthcare)</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>RS Premier Jatinegara, Bintaro and Surabaya and Columbia Asia hospitals</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>Vina Elvira, Kontan Rumah Sakit Internasional Columbia Asia Resmi Akuisisi RS Medika BSD</t>
+        </is>
+      </c>
+      <c r="D137" s="5" t="inlineStr">
+        <is>
+          <t>2023-09-19</t>
+        </is>
+      </c>
+      <c r="E137" s="5" t="inlineStr">
+        <is>
+          <t>https://industri.kontan.co.id/news/rumah-sakit-internasional-columbia-asia-resmi-akuisisi-rs-medika-bsd</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="5" t="inlineStr">
+        <is>
+          <t>Chung Shan Medical University (Taiwan)</t>
+        </is>
+      </c>
+      <c r="B138" s="5" t="inlineStr">
+        <is>
+          <t>Universitas Indonesia</t>
+        </is>
+      </c>
+      <c r="C138" s="5" t="inlineStr">
+        <is>
+          <t>CSMU Chung Shan Medical University Signs MOU with Universitas Indonesia to Advance Comprehensive Collaboration</t>
+        </is>
+      </c>
+      <c r="D138" s="5" t="inlineStr">
+        <is>
+          <t>2025-08-08</t>
+        </is>
+      </c>
+      <c r="E138" s="5" t="inlineStr">
+        <is>
+          <t>https://pr.csmu.edu.tw/p/16-1024-71677.php?Lang=zh-tw</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="5" t="inlineStr">
+        <is>
+          <t>Hong Kong Asia Medical Group (HKAMG)</t>
+        </is>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (PT Pertamedika Bali Hospital, IHC)</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>Ni Putu Putri Muliantari, ANTARA Akhirnya ada prosedur TAVI di KEK Sanur untuk tangani kasus jantung</t>
+        </is>
+      </c>
+      <c r="D139" s="5" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="E139" s="5" t="inlineStr">
+        <is>
+          <t>https://bali.antaranews.com/berita/400683/akhirnya-ada-prosedur-tavi-di-kek-sanur-untuk-tangani-kasus-jantung</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="5" t="inlineStr">
+        <is>
+          <t>Hong Kong Asia Medical Group (HKAMG)</t>
+        </is>
+      </c>
+      <c r="B140" s="5" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (PT Pertamedika Bali Hospital, IHC)</t>
+        </is>
+      </c>
+      <c r="C140" s="5" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (press release) Bali International Hospital Hosts Meet &amp; Greet with Global Medical Partners</t>
+        </is>
+      </c>
+      <c r="D140" s="5" t="inlineStr">
+        <is>
+          <t>2025-04-25</t>
+        </is>
+      </c>
+      <c r="E140" s="5" t="inlineStr">
+        <is>
+          <t>https://bali.com/news/press-releases/bali-international-hospital-hosts-meet-greet-with-global-medical-partners</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="5" t="inlineStr">
+        <is>
+          <t>Hong Kong Asia Medical Group (HKAMG)</t>
+        </is>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (PT Pertamedika Bali Hospital, IHC)</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>International Finance Corporation Asia Heart project (Hong Kong Asia Medical Holding and Wuhan Asia Heart Hospital)</t>
+        </is>
+      </c>
+      <c r="D141" s="5" t="inlineStr"/>
+      <c r="E141" s="5" t="inlineStr">
+        <is>
+          <t>https://disclosures.ifc.org/project-detail/SII/33623/asia-heart-project</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="5" t="inlineStr">
+        <is>
+          <t>Icon Group (Icon Cancer Centre)</t>
+        </is>
+      </c>
+      <c r="B142" s="5" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (PT Pertamina Bina Medika IHC)</t>
+        </is>
+      </c>
+      <c r="C142" s="5" t="inlineStr">
+        <is>
+          <t>Icon Writers Icon Cancer Centre at Bali International Hospital marks regional first with advanced radiotherapy cancer treatments</t>
+        </is>
+      </c>
+      <c r="D142" s="5" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="E142" s="5" t="inlineStr">
+        <is>
+          <t>https://icongroup.global/?p=18098</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="inlineStr">
+        <is>
+          <t>Icon Group (Icon Cancer Centre)</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (PT Pertamina Bina Medika IHC)</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>Icon Writers Icon Cancer Centre Bali treats first patient</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="inlineStr">
+        <is>
+          <t>2025-05-07</t>
+        </is>
+      </c>
+      <c r="E143" s="5" t="inlineStr">
+        <is>
+          <t>https://icongroup.global/en/news/2025-05-07/icon-cancer-centre-bali-treats-first-patient/</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="5" t="inlineStr">
+        <is>
+          <t>Icon Group (Icon Cancer Centre)</t>
+        </is>
+      </c>
+      <c r="B144" s="5" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (PT Pertamina Bina Medika IHC)</t>
+        </is>
+      </c>
+      <c r="C144" s="5" t="inlineStr">
+        <is>
+          <t>Icon Group Icon Group, Bali International Hospital partnership to deliver exceptional cancer care</t>
+        </is>
+      </c>
+      <c r="D144" s="5" t="inlineStr">
+        <is>
+          <t>2025-03-04</t>
+        </is>
+      </c>
+      <c r="E144" s="5" t="inlineStr">
+        <is>
+          <t>https://icongroup.global/en/news/2025-03-04/icon-group-and-bali-international-hospital/</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="5" t="inlineStr">
+        <is>
+          <t>International University of Health and Welfare (IUHW)</t>
+        </is>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health (Kemenkes)</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health of Indonesia Kemenkes dan IUHW Jepang Kerja Sama Perkuat Pendidikan Dokter Spesialis</t>
+        </is>
+      </c>
+      <c r="D145" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="E145" s="5" t="inlineStr">
+        <is>
+          <t>https://kemkes.go.id/id/kemenkes-dan-iuhw-jepang-kerja-sama-perkuat-pendidikan-dokter-spesialis</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="5" t="inlineStr">
+        <is>
+          <t>International University of Health and Welfare (IUHW)</t>
+        </is>
+      </c>
+      <c r="B146" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health (Kemenkes)</t>
+        </is>
+      </c>
+      <c r="C146" s="5" t="inlineStr">
+        <is>
+          <t>RRI Indonesia and Japan Expand Cooperation in Specialist Medical Education</t>
+        </is>
+      </c>
+      <c r="D146" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="E146" s="5" t="inlineStr">
+        <is>
+          <t>https://rri.co.id/en/education/2332993/indonesia-and-japan-expand-cooperation-in-specialist-medical-education</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="5" t="inlineStr">
+        <is>
+          <t>Monash Health</t>
+        </is>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>RS Otak Dr. Drs. M. Hatta Bukittinggi (RSOMH, Ministry of Health brain hospital)</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>Humas RSOMH Bukittinggi RSOMH Bukittinggi dan Monash Health Perkuat Kolaborasi Pengembangan Rehabilitasi Stroke</t>
+        </is>
+      </c>
+      <c r="D147" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="E147" s="5" t="inlineStr">
+        <is>
+          <t>https://keslan.kemkes.go.id/read/4058/rsomh-bukittinggi-dan-monash-health-perkuat-kolaborasi-pengembangan-rehabilitasi-stroke</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="5" t="inlineStr">
+        <is>
+          <t>Monash Health</t>
+        </is>
+      </c>
+      <c r="B148" s="5" t="inlineStr">
+        <is>
+          <t>RS Otak Dr. Drs. M. Hatta Bukittinggi (RSOMH, Ministry of Health brain hospital)</t>
+        </is>
+      </c>
+      <c r="C148" s="5" t="inlineStr">
+        <is>
+          <t>Humas RSOMH Bukittinggi RSOMH Bukittinggi Dukung Rencana Program Kerja Sama Bersama Monash Health</t>
+        </is>
+      </c>
+      <c r="D148" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="E148" s="5" t="inlineStr">
+        <is>
+          <t>https://keslan.kemkes.go.id/read/4358/rsomh-bukittinggi-dukung-rencana-program-kerja-sama-bersama-monash-health</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="5" t="inlineStr">
+        <is>
+          <t>National Center for Global Health and Medicine (NCGM) and Kobe University</t>
+        </is>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>Universitas Airlangga (Institute of Tropical Disease and RS Universitas Airlangga)</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>UNAIR News Japanese delegation visits UNAIR Hospital to strengthen research and innovation collaboration</t>
+        </is>
+      </c>
+      <c r="D149" s="5" t="inlineStr">
+        <is>
+          <t>2025-02-20</t>
+        </is>
+      </c>
+      <c r="E149" s="5" t="inlineStr">
+        <is>
+          <t>https://unair.ac.id/en/japanese-delegation-visits-unair-hospital-to-strengthen-research-and-innovation-collaboration/</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="5" t="inlineStr">
+        <is>
+          <t>Ramathibodi Hospital, Mahidol University</t>
+        </is>
+      </c>
+      <c r="B150" s="5" t="inlineStr">
+        <is>
+          <t>Faculty of Medicine Universitas Indonesia and RSCM</t>
+        </is>
+      </c>
+      <c r="C150" s="5" t="inlineStr">
+        <is>
+          <t>Ramathibodi International Office Ramathibodi Hospital and Universitas Indonesia Strengthen Medical Ties with MOU Signing</t>
+        </is>
+      </c>
+      <c r="D150" s="5" t="inlineStr">
+        <is>
+          <t>2025-05-21</t>
+        </is>
+      </c>
+      <c r="E150" s="5" t="inlineStr">
+        <is>
+          <t>https://www.rama.mahidol.ac.th/international/news/event/22052025-1111</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="5" t="inlineStr">
+        <is>
+          <t>Sapporo Cardio Vascular Clinic</t>
+        </is>
+      </c>
+      <c r="B151" s="5" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (PT Pertamedika Bali Hospital, IHC)</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>Mardiana Makmun, Investor Daily Teknologi TAVI Tangani Penyakit Katup Jantung</t>
+        </is>
+      </c>
+      <c r="D151" s="5" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="E151" s="5" t="inlineStr">
+        <is>
+          <t>https://investor.id/lifestyle/432385/teknologi-tavi-tangani-penyakit-katup-jantung</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="5" t="inlineStr">
+        <is>
+          <t>Sapporo Cardio Vascular Clinic</t>
+        </is>
+      </c>
+      <c r="B152" s="5" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (PT Pertamedika Bali Hospital, IHC)</t>
+        </is>
+      </c>
+      <c r="C152" s="5" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (press release) Bali International Hospital Hosts Meet &amp; Greet with Global Medical Partners</t>
+        </is>
+      </c>
+      <c r="D152" s="5" t="inlineStr">
+        <is>
+          <t>2025-04-25</t>
+        </is>
+      </c>
+      <c r="E152" s="5" t="inlineStr">
+        <is>
+          <t>https://bali.com/news/press-releases/bali-international-hospital-hosts-meet-greet-with-global-medical-partners</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="5" t="inlineStr">
+        <is>
+          <t>Sapporo Cardio Vascular Clinic</t>
+        </is>
+      </c>
+      <c r="B153" s="5" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (PT Pertamedika Bali Hospital, IHC)</t>
+        </is>
+      </c>
+      <c r="C153" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health of Indonesia Atasi Kekurangan Dokter Spesialis, Kemenkes Berangkatkan 27 Dokter Belajar ke RRT dan Jepang</t>
+        </is>
+      </c>
+      <c r="D153" s="5" t="inlineStr">
+        <is>
+          <t>2025-01-06</t>
+        </is>
+      </c>
+      <c r="E153" s="5" t="inlineStr">
+        <is>
+          <t>https://kemkes.go.id/eng/atasi-kekurangan-dokter-spesialis-kemenkes-berangkatkan-27-dokter-belajar-ke-rrt-dan-jepang</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="5" t="inlineStr">
+        <is>
+          <t>Seoul National University Hospital (SNUH)</t>
+        </is>
+      </c>
+      <c r="B154" s="5" t="inlineStr">
+        <is>
+          <t>Faculty of Medicine Universitas Indonesia and RSUPN Dr. Cipto Mangunkusumo (RSCM)</t>
+        </is>
+      </c>
+      <c r="C154" s="5" t="inlineStr">
+        <is>
+          <t>Noh Jae-young, Medipharm Health 서울대병원-인도네시아 의대-RSCM 병원 간 AOI 체결</t>
+        </is>
+      </c>
+      <c r="D154" s="5" t="inlineStr">
+        <is>
+          <t>2025-02-04</t>
+        </is>
+      </c>
+      <c r="E154" s="5" t="inlineStr">
+        <is>
+          <t>https://medipharmhealth.co.kr/news/article.html?no=105006</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="5" t="inlineStr">
+        <is>
+          <t>Seoul National University Hospital (SNUH)</t>
+        </is>
+      </c>
+      <c r="B155" s="5" t="inlineStr">
+        <is>
+          <t>RSUP Fatmawati (Ministry of Health hospital)</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health of Indonesia Lakukan Transplantasi Hati Ketiga RSUP Fatmawati Perkuat Kemandirian Layanan Dalam Negeri</t>
+        </is>
+      </c>
+      <c r="D155" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="E155" s="5" t="inlineStr">
+        <is>
+          <t>https://www.kemkes.go.id/eng/lakukan-transplantasi-hati-ketiga-rsup-fatmawati-perkuat-kemandirian-layanan-dalam-negeri</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="5" t="inlineStr">
+        <is>
+          <t>Seoul National University Hospital (SNUH)</t>
+        </is>
+      </c>
+      <c r="B156" s="5" t="inlineStr">
+        <is>
+          <t>RSUP Fatmawati (Ministry of Health hospital)</t>
+        </is>
+      </c>
+      <c r="C156" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health of Indonesia Kerja Sama Indonesia-Korea Dukung Implementasi Transformasi Kesehatan</t>
+        </is>
+      </c>
+      <c r="D156" s="5" t="inlineStr">
+        <is>
+          <t>2023-03-27</t>
+        </is>
+      </c>
+      <c r="E156" s="5" t="inlineStr">
+        <is>
+          <t>https://www.kemkes.go.id/eng/kerja-sama-indonesia-korea-dukung-implementasi-transformasi-kesehatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="5" t="inlineStr">
+        <is>
+          <t>SingHealth</t>
+        </is>
+      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>Indonesia Healthcare Corporation (PT Pertamina Bina Medika) and Bali International Hospital</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (press release) Bali International Hospital Hosts Meet &amp; Greet with Global Medical Partners</t>
+        </is>
+      </c>
+      <c r="D157" s="5" t="inlineStr">
+        <is>
+          <t>2025-04-25</t>
+        </is>
+      </c>
+      <c r="E157" s="5" t="inlineStr">
+        <is>
+          <t>https://bali.com/news/press-releases/bali-international-hospital-hosts-meet-greet-with-global-medical-partners</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="5" t="inlineStr">
+        <is>
+          <t>SingHealth</t>
+        </is>
+      </c>
+      <c r="B158" s="5" t="inlineStr">
+        <is>
+          <t>Indonesia Healthcare Corporation (PT Pertamina Bina Medika) and Bali International Hospital</t>
+        </is>
+      </c>
+      <c r="C158" s="5" t="inlineStr">
+        <is>
+          <t>Indonesia Business Post IHC, Singhealth seals deal collaboration to improve patient care</t>
+        </is>
+      </c>
+      <c r="D158" s="5" t="inlineStr">
+        <is>
+          <t>2024-05-02</t>
+        </is>
+      </c>
+      <c r="E158" s="5" t="inlineStr">
+        <is>
+          <t>https://indonesiabusinesspost.com/1823/Politics/ihc-singhealth-seals-deal-collaboration-to-improve-patient-care</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="5" t="inlineStr">
+        <is>
+          <t>SingHealth</t>
+        </is>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>Indonesia Healthcare Corporation (PT Pertamina Bina Medika) and Bali International Hospital</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>Pertamina Pertamina Bina Medika IHC and SingHealth collaborate to enhance healthcare services</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="inlineStr">
+        <is>
+          <t>2024-05-02</t>
+        </is>
+      </c>
+      <c r="E159" s="5" t="inlineStr">
+        <is>
+          <t>https://pertamina.com/en/news-room/news-release/pertamina-bina-medika-ihc-and-singhealth-collaborate-to-enhance-healthcare-services</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="5" t="inlineStr">
+        <is>
+          <t>SingHealth Duke-NUS Global Health Institute (SingHealth and Duke-NUS Medical School)</t>
+        </is>
+      </c>
+      <c r="B160" s="5" t="inlineStr">
+        <is>
+          <t>Universitas Sumatera Utara (Faculty of Medicine)</t>
+        </is>
+      </c>
+      <c r="C160" s="5" t="inlineStr">
+        <is>
+          <t>Universitas Sumatera Utara Collaboration between the Faculty of Medicine, Universitas Sumatera Utara (USU) and SingHealth Duke-NUS Global Health Institute on the 2025 Summer Course</t>
+        </is>
+      </c>
+      <c r="D160" s="5" t="inlineStr">
+        <is>
+          <t>2025-08-01</t>
+        </is>
+      </c>
+      <c r="E160" s="5" t="inlineStr">
+        <is>
+          <t>https://www.usu.ac.id/en/news/collaboration-between-the-faculty-of-medicine-universitas-sumatera-utara-usu-and-singhealth-duke-nus-global-health-institute-on-the-2025-summer-course</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="inlineStr">
+        <is>
+          <t>SingHealth Duke-NUS Global Health Institute (SingHealth and Duke-NUS Medical School)</t>
+        </is>
+      </c>
+      <c r="B161" s="5" t="inlineStr">
+        <is>
+          <t>Universitas Sumatera Utara (Faculty of Medicine)</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>Universitas Sumatera Utara USU-Duke NUS Global Health Strengthen Partnerships</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="inlineStr">
+        <is>
+          <t>2023-08-08</t>
+        </is>
+      </c>
+      <c r="E161" s="5" t="inlineStr">
+        <is>
+          <t>https://www.usu.ac.id/en/news/usu-duke-nus-global-health-strengthen-partnerships</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="5" t="inlineStr">
+        <is>
+          <t>Sun Medical Center (Sun Healthcare International)</t>
+        </is>
+      </c>
+      <c r="B162" s="5" t="inlineStr">
+        <is>
+          <t>RSUP Prof. Dr. I.G.N.G. Ngoerah</t>
+        </is>
+      </c>
+      <c r="C162" s="5" t="inlineStr">
+        <is>
+          <t>Benedikta Desideria, Liputan6 Dorong Wisata Medis Bali, Menkes Budi: Jangan Pilih yang Kuratif tapi Wellness</t>
+        </is>
+      </c>
+      <c r="D162" s="5" t="inlineStr">
+        <is>
+          <t>2024-10-05</t>
+        </is>
+      </c>
+      <c r="E162" s="5" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/health/read/5731675/dorong-wisata-medis-bali-menkes-budi-jangan-pilih-yang-kuratif-tapi-wellness</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="inlineStr">
+        <is>
+          <t>Sun Medical Center (Sun Healthcare International)</t>
+        </is>
+      </c>
+      <c r="B163" s="5" t="inlineStr">
+        <is>
+          <t>RSUP Prof. Dr. I.G.N.G. Ngoerah</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health of Indonesia Kerja Sama Indonesia-Korea Dukung Implementasi Transformasi Kesehatan</t>
+        </is>
+      </c>
+      <c r="D163" s="5" t="inlineStr">
+        <is>
+          <t>2023-03-27</t>
+        </is>
+      </c>
+      <c r="E163" s="5" t="inlineStr">
+        <is>
+          <t>https://www.kemkes.go.id/eng/kerja-sama-indonesia-korea-dukung-implementasi-transformasi-kesehatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="5" t="inlineStr">
+        <is>
+          <t>Taipei Veterans General Hospital</t>
+        </is>
+      </c>
+      <c r="B164" s="5" t="inlineStr">
+        <is>
+          <t>DKH Hospitals Group</t>
+        </is>
+      </c>
+      <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>Antara DKH Hospitals dan TVGH teken MoU tingkatkan layanan kesehatan di RI</t>
+        </is>
+      </c>
+      <c r="D164" s="5" t="inlineStr">
+        <is>
+          <t>2025-05-23</t>
+        </is>
+      </c>
+      <c r="E164" s="5" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/4853713/dkh-hospitals-dan-tvgh-teken-mou-tingkatkan-layanan-kesehatan-di-ri</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="5" t="inlineStr">
+        <is>
+          <t>Tokushukai Medical Group</t>
+        </is>
+      </c>
+      <c r="B165" s="5" t="inlineStr">
+        <is>
+          <t>RSJPD Harapan Kita (National Heart Center) and Ministry of Health</t>
+        </is>
+      </c>
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health of Indonesia Perkuat Layanan Jantung Berkelas Dunia di Indonesia, Gedung Baru RS Harkit Resmi Topping Off</t>
+        </is>
+      </c>
+      <c r="D165" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="E165" s="5" t="inlineStr">
+        <is>
+          <t>https://www.kemkes.go.id/eng/perkuat-layanan-jantung-berkelas-dunia-di-indonesia-gedung-baru-rs-harkit-resmi-topping-off</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="5" t="inlineStr">
+        <is>
+          <t>Tokushukai Medical Group</t>
+        </is>
+      </c>
+      <c r="B166" s="5" t="inlineStr">
+        <is>
+          <t>RSJPD Harapan Kita (National Heart Center) and Ministry of Health</t>
+        </is>
+      </c>
+      <c r="C166" s="5" t="inlineStr">
+        <is>
+          <t>Antara Indonesia, Japan back Harapan Kita as Asia's biggest cardiac hub</t>
+        </is>
+      </c>
+      <c r="D166" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="E166" s="5" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412388/indonesia-japan-back-harapan-kita-as-asias-biggest-cardiac-hub</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="5" t="inlineStr">
+        <is>
+          <t>Tokushukai Medical Group</t>
+        </is>
+      </c>
+      <c r="B167" s="5" t="inlineStr">
+        <is>
+          <t>RSJPD Harapan Kita (National Heart Center) and Ministry of Health</t>
+        </is>
+      </c>
+      <c r="C167" s="5" t="inlineStr">
+        <is>
+          <t>SSEK SSEK Acts for Tokushukai Medical Corporation Group in Major Cooperation Project in Indonesian Health Sector</t>
+        </is>
+      </c>
+      <c r="D167" s="5" t="inlineStr">
+        <is>
+          <t>2023-12-11</t>
+        </is>
+      </c>
+      <c r="E167" s="5" t="inlineStr">
+        <is>
+          <t>https://ssek.com/blog/ssek-acts-for-tokushukai-medical-corporation-group-in-major-cooperation-project-in-indonesian-health-sector/?lang=id</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="5" t="inlineStr">
+        <is>
+          <t>Wuhan Asia Heart Hospital</t>
+        </is>
+      </c>
+      <c r="B168" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health (Kemenkes)</t>
+        </is>
+      </c>
+      <c r="C168" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health of Indonesia Perkuat Layanan Jantung Nasional: 13 Dokter Spesialis Jantung Indonesia Berguru ke Tiongkok</t>
+        </is>
+      </c>
+      <c r="D168" s="5" t="inlineStr">
+        <is>
+          <t>2024-11-12</t>
+        </is>
+      </c>
+      <c r="E168" s="5" t="inlineStr">
+        <is>
+          <t>https://kemkes.go.id/id/perkuat-layanan-jantung-nasional-13-dokter-spesialis-jantung-indonesia-berguru-ke-tiongkok</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="5" t="inlineStr">
+        <is>
+          <t>Zhongda Hospital (Southeast University)</t>
+        </is>
+      </c>
+      <c r="B169" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health (Kemenkes)</t>
+        </is>
+      </c>
+      <c r="C169" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health of Indonesia Atasi Kekurangan Dokter Spesialis, Kemenkes Berangkatkan 27 Dokter Belajar ke RRT dan Jepang</t>
+        </is>
+      </c>
+      <c r="D169" s="5" t="inlineStr">
+        <is>
+          <t>2025-01-06</t>
+        </is>
+      </c>
+      <c r="E169" s="5" t="inlineStr">
+        <is>
+          <t>https://kemkes.go.id/eng/atasi-kekurangan-dokter-spesialis-kemenkes-berangkatkan-27-dokter-belajar-ke-rrt-dan-jepang</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="5" t="inlineStr">
+        <is>
+          <t>Zhongshan Hospital (Fudan University)</t>
+        </is>
+      </c>
+      <c r="B170" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health (Kemenkes)</t>
+        </is>
+      </c>
+      <c r="C170" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health of Indonesia Atasi Kekurangan Dokter Spesialis, Kemenkes Berangkatkan 27 Dokter Belajar ke RRT dan Jepang</t>
+        </is>
+      </c>
+      <c r="D170" s="5" t="inlineStr">
+        <is>
+          <t>2025-01-06</t>
+        </is>
+      </c>
+      <c r="E170" s="5" t="inlineStr">
+        <is>
+          <t>https://kemkes.go.id/eng/atasi-kekurangan-dokter-spesialis-kemenkes-berangkatkan-27-dokter-belajar-ke-rrt-dan-jepang</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="5" t="inlineStr">
+        <is>
+          <t>Zhongshan Hospital (Fudan University)</t>
+        </is>
+      </c>
+      <c r="B171" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health (Kemenkes)</t>
+        </is>
+      </c>
+      <c r="C171" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health of Indonesia Perkuat Layanan Jantung Nasional: 13 Dokter Spesialis Jantung Indonesia Berguru ke Tiongkok</t>
+        </is>
+      </c>
+      <c r="D171" s="5" t="inlineStr">
+        <is>
+          <t>2024-11-12</t>
+        </is>
+      </c>
+      <c r="E171" s="5" t="inlineStr">
+        <is>
+          <t>https://kemkes.go.id/id/perkuat-layanan-jantung-nasional-13-dokter-spesialis-jantung-indonesia-berguru-ke-tiongkok</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="5" t="inlineStr">
+        <is>
+          <t>Zhongshan Hospital (Fudan University)</t>
+        </is>
+      </c>
+      <c r="B172" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health (Kemenkes)</t>
+        </is>
+      </c>
+      <c r="C172" s="5" t="inlineStr">
+        <is>
+          <t>Kemenkes Kemenkes RI dan RS Rizhao Xinyi Kerja Sama Pelatihan Dokter Kardiovaskular</t>
+        </is>
+      </c>
+      <c r="D172" s="5" t="inlineStr">
+        <is>
+          <t>2024-06-11</t>
+        </is>
+      </c>
+      <c r="E172" s="5" t="inlineStr">
+        <is>
+          <t>https://www.kemkes.go.id/eng/kemenkes-ri-dan-rs-rizhao-xinyi-kerja-sama-pelatihan-dokter-kardiovaskular</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="5" t="inlineStr">
+        <is>
+          <t>Mayo Clinic</t>
+        </is>
+      </c>
+      <c r="B173" s="5" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (Indonesia Healthcare Corporation)</t>
+        </is>
+      </c>
+      <c r="C173" s="5" t="inlineStr">
+        <is>
+          <t>The Jakarta Post Mayo Clinic only acting as consultant for Bali International Hospital, executive says</t>
+        </is>
+      </c>
+      <c r="D173" s="5" t="inlineStr">
+        <is>
+          <t>2023-03-17</t>
+        </is>
+      </c>
+      <c r="E173" s="5" t="inlineStr">
+        <is>
+          <t>https://www.thejakartapost.com/business/2023/03/17/mayo-clinic-only-acting-as-consultant-for-bali-international-hospital-executive-says</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="5" t="inlineStr">
+        <is>
+          <t>Mayo Clinic</t>
+        </is>
+      </c>
+      <c r="B174" s="5" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (Indonesia Healthcare Corporation)</t>
+        </is>
+      </c>
+      <c r="C174" s="5" t="inlineStr">
+        <is>
+          <t>Becker's Hospital Review Mayo Clinic to advise on building, operating hospital in Indonesia</t>
+        </is>
+      </c>
+      <c r="D174" s="5" t="inlineStr">
+        <is>
+          <t>2021-12</t>
+        </is>
+      </c>
+      <c r="E174" s="5" t="inlineStr">
+        <is>
+          <t>https://www.beckershospitalreview.com/capital/mayo-clinic-to-help-build-operate-hospital-in-indonesia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="5" t="inlineStr">
+        <is>
+          <t>Mayo Clinic</t>
+        </is>
+      </c>
+      <c r="B175" s="5" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (Indonesia Healthcare Corporation)</t>
+        </is>
+      </c>
+      <c r="C175" s="5" t="inlineStr">
+        <is>
+          <t>Bali International Hospital (press release) Bali International Hospital Hosts Meet &amp; Greet with Global Medical Partners</t>
+        </is>
+      </c>
+      <c r="D175" s="5" t="inlineStr">
+        <is>
+          <t>2025-04-25</t>
+        </is>
+      </c>
+      <c r="E175" s="5" t="inlineStr">
+        <is>
+          <t>https://bali.com/news/press-releases/bali-international-hospital-hosts-meet-greet-with-global-medical-partners</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="5" t="inlineStr">
+        <is>
+          <t>UCLA Health</t>
+        </is>
+      </c>
+      <c r="B176" s="5" t="inlineStr">
+        <is>
+          <t>RS Jantung dan Pembuluh Darah Harapan Kita</t>
+        </is>
+      </c>
+      <c r="C176" s="5" t="inlineStr">
+        <is>
+          <t>Kementerian Kesehatan RI Wujudkan Transformasi Layanan Rujukan, RS Jantung Harapan Kita jadi RS Pertama Transplantasi Jantung di Indonesia</t>
+        </is>
+      </c>
+      <c r="D176" s="5" t="inlineStr">
+        <is>
+          <t>2022-11-09</t>
+        </is>
+      </c>
+      <c r="E176" s="5" t="inlineStr">
+        <is>
+          <t>https://kemkes.go.id/eng/wujudkan-transformasi-layanan-rujukan-rs-jantung-harapan-kita-jadi-rs-pertama-transplantasi-jantung-di-indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="5" t="inlineStr">
+        <is>
+          <t>Asan Medical Center</t>
+        </is>
+      </c>
+      <c r="B177" s="5" t="inlineStr">
+        <is>
+          <t>Siloam Hospitals Group</t>
+        </is>
+      </c>
+      <c r="C177" s="5" t="inlineStr">
+        <is>
+          <t>Adv Team Grup RS Siloam Jalin Kerja Sama dengan Asan Medical Center Korea Selatan</t>
+        </is>
+      </c>
+      <c r="D177" s="5" t="inlineStr">
+        <is>
+          <t>2023-11-03</t>
+        </is>
+      </c>
+      <c r="E177" s="5" t="inlineStr">
+        <is>
+          <t>https://www.kompas.tv/advertorial/457691/grup-rs-siloam-jalin-kerja-sama-dengan-asan-medical-center-korea-selatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="5" t="inlineStr">
+        <is>
+          <t>Icon Group (Icon Cancer Centre, Singapore)</t>
+        </is>
+      </c>
+      <c r="B178" s="5" t="inlineStr">
+        <is>
+          <t>RS Universitas Airlangga (RSUA)</t>
+        </is>
+      </c>
+      <c r="C178" s="5" t="inlineStr">
+        <is>
+          <t>BioSpectrum Asia Airlangga University Hospital signs MoU with Singapore's Icon Cancer Center</t>
+        </is>
+      </c>
+      <c r="D178" s="5" t="inlineStr">
+        <is>
+          <t>2023-04-10</t>
+        </is>
+      </c>
+      <c r="E178" s="5" t="inlineStr">
+        <is>
+          <t>https://www.biospectrumasia.com/news/54/22260/airlangga-university-hospital-signs-mou-with-singapores-icon-cancer-center.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="5" t="inlineStr">
+        <is>
+          <t>National Center for Global Health and Medicine (NCGM)</t>
+        </is>
+      </c>
+      <c r="B179" s="5" t="inlineStr">
+        <is>
+          <t>Siloam Hospitals Group</t>
+        </is>
+      </c>
+      <c r="C179" s="5" t="inlineStr">
+        <is>
+          <t>National Center for Global Health and Medicine The National Center for Global Health and Medicine and the Siloam Hospitals Group have signed a Memorandum of Understanding (MoU) for clinical research cooperation</t>
+        </is>
+      </c>
+      <c r="D179" s="5" t="inlineStr">
+        <is>
+          <t>2022-10-07</t>
+        </is>
+      </c>
+      <c r="E179" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ncgm.go.jp/en/news/FY2022/20221007.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="5" t="inlineStr">
+        <is>
+          <t>Peking Union Medical College Hospital</t>
+        </is>
+      </c>
+      <c r="B180" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health (Kemenkes)</t>
+        </is>
+      </c>
+      <c r="C180" s="5" t="inlineStr">
+        <is>
+          <t>Kemenkes Kemenkes RI dan RS Rizhao Xinyi Kerja Sama Pelatihan Dokter Kardiovaskular</t>
+        </is>
+      </c>
+      <c r="D180" s="5" t="inlineStr">
+        <is>
+          <t>2024-06-11</t>
+        </is>
+      </c>
+      <c r="E180" s="5" t="inlineStr">
+        <is>
+          <t>https://www.kemkes.go.id/eng/kemenkes-ri-dan-rs-rizhao-xinyi-kerja-sama-pelatihan-dokter-kardiovaskular</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="5" t="inlineStr">
+        <is>
+          <t>Rizhao Xinyi Hospital (Rizhao Heart Hospital)</t>
+        </is>
+      </c>
+      <c r="B181" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health (Kemenkes)</t>
+        </is>
+      </c>
+      <c r="C181" s="5" t="inlineStr">
+        <is>
+          <t>Kemenkes Kemenkes RI dan RS Rizhao Xinyi Kerja Sama Pelatihan Dokter Kardiovaskular</t>
+        </is>
+      </c>
+      <c r="D181" s="5" t="inlineStr">
+        <is>
+          <t>2024-06-11</t>
+        </is>
+      </c>
+      <c r="E181" s="5" t="inlineStr">
+        <is>
+          <t>https://www.kemkes.go.id/eng/kemenkes-ri-dan-rs-rizhao-xinyi-kerja-sama-pelatihan-dokter-kardiovaskular</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="5" t="inlineStr">
+        <is>
+          <t>Royal Brompton and Harefield Hospitals (Guy's and St Thomas' NHS Foundation Trust)</t>
+        </is>
+      </c>
+      <c r="B182" s="5" t="inlineStr">
+        <is>
+          <t>Mandaya Royal Hospital Puri</t>
+        </is>
+      </c>
+      <c r="C182" s="5" t="inlineStr">
+        <is>
+          <t>Mandaya Hospital Group Mandaya Royal Hospital Puri and London's Royal Brompton &amp; Harefield Hospitals Announce Strategic Partnership</t>
+        </is>
+      </c>
+      <c r="D182" s="5" t="inlineStr">
+        <is>
+          <t>2020-12-19</t>
+        </is>
+      </c>
+      <c r="E182" s="5" t="inlineStr">
+        <is>
+          <t>https://mandayahospitalgroup.com/?p=11304</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="5" t="inlineStr">
+        <is>
+          <t>Royal Brompton and Harefield Hospitals (Guy's and St Thomas' NHS Foundation Trust)</t>
+        </is>
+      </c>
+      <c r="B183" s="5" t="inlineStr">
+        <is>
+          <t>Mandaya Royal Hospital Puri</t>
+        </is>
+      </c>
+      <c r="C183" s="5" t="inlineStr">
+        <is>
+          <t>RM.id Gandeng Royal Brompton, Mandaya Hospital resmikan pusat jantung anak</t>
+        </is>
+      </c>
+      <c r="D183" s="5" t="inlineStr">
+        <is>
+          <t>2023-05-22</t>
+        </is>
+      </c>
+      <c r="E183" s="5" t="inlineStr">
+        <is>
+          <t>https://rm.id/baca-berita/life-style/172779/gandeng-royal-brompton-mandaya-hospital-resmikan-pusat-jantung-anak</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="5" t="inlineStr">
+        <is>
+          <t>UMC Utrecht</t>
+        </is>
+      </c>
+      <c r="B184" s="5" t="inlineStr">
+        <is>
+          <t>RS Jantung dan Pembuluh Darah Harapan Kita</t>
+        </is>
+      </c>
+      <c r="C184" s="5" t="inlineStr">
+        <is>
+          <t>Ministry of Health of Indonesia Wujudkan Transformasi Layanan Rujukan, RS Jantung Harapan Kita jadi RS Pertama Transplantasi Jantung di Indonesia</t>
+        </is>
+      </c>
+      <c r="D184" s="5" t="inlineStr">
+        <is>
+          <t>2022-11-09</t>
+        </is>
+      </c>
+      <c r="E184" s="5" t="inlineStr">
+        <is>
+          <t>https://kemkes.go.id/eng/wujudkan-transformasi-layanan-rujukan-rs-jantung-harapan-kita-jadi-rs-pertama-transplantasi-jantung-di-indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="5" t="inlineStr">
+        <is>
+          <t>KPJ Healthcare</t>
+        </is>
+      </c>
+      <c r="B185" s="5" t="inlineStr">
+        <is>
+          <t>RS Medika BSD</t>
+        </is>
+      </c>
+      <c r="C185" s="5" t="inlineStr">
+        <is>
+          <t>Warta Ekonomi Ekspansi Besar-besaran, RS Columbia Asia Buka Dua Rumah Sakit dalam Seminggu</t>
+        </is>
+      </c>
+      <c r="D185" s="5" t="inlineStr">
+        <is>
+          <t>2023-10-02</t>
+        </is>
+      </c>
+      <c r="E185" s="5" t="inlineStr">
+        <is>
+          <t>https://wartaekonomi.co.id/read515939/ekspansi-besar-besaran-rs-columbia-asia-buka-dua-rumah-sakit-dalam-seminggu</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="5" t="inlineStr">
+        <is>
+          <t>KPJ Healthcare</t>
+        </is>
+      </c>
+      <c r="B186" s="5" t="inlineStr">
+        <is>
+          <t>RS Medika BSD</t>
+        </is>
+      </c>
+      <c r="C186" s="5" t="inlineStr">
+        <is>
+          <t>Vina Elvira, Kontan Rumah Sakit Internasional Columbia Asia Resmi Akuisisi RS Medika BSD</t>
+        </is>
+      </c>
+      <c r="D186" s="5" t="inlineStr">
+        <is>
+          <t>2023-09-19</t>
+        </is>
+      </c>
+      <c r="E186" s="5" t="inlineStr">
+        <is>
+          <t>https://industri.kontan.co.id/news/rumah-sakit-internasional-columbia-asia-resmi-akuisisi-rs-medika-bsd</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="5" t="inlineStr">
+        <is>
+          <t>Ramsay Health Care</t>
+        </is>
+      </c>
+      <c r="B187" s="5" t="inlineStr">
+        <is>
+          <t>RS Premier Jatinegara, Bintaro and Surabaya</t>
+        </is>
+      </c>
+      <c r="C187" s="5" t="inlineStr">
+        <is>
+          <t>The Edge Malaysia Columbia Asia Healthcare renamed Asia OneHealthcare (A1Health) after consolidating assets in Malaysia, Indonesia and Vietnam</t>
+        </is>
+      </c>
+      <c r="D187" s="5" t="inlineStr">
+        <is>
+          <t>2024-09-06</t>
+        </is>
+      </c>
+      <c r="E187" s="5" t="inlineStr">
+        <is>
+          <t>https://theedgemalaysia.com/node/725855</t>
         </is>
       </c>
     </row>
@@ -7458,6 +11511,76 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E115" r:id="rId114"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E116" r:id="rId115"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E134" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E135" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E136" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E137" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E149" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E150" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E151" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E152" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E153" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E154" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E155" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E156" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E157" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E158" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E159" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E160" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E161" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E162" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E163" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E164" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E165" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E166" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E167" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E168" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E169" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E170" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E171" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E172" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E173" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E174" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E175" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E176" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E177" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E178" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E179" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E180" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E181" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E182" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E183" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E184" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E185" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E186" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E187" r:id="rId186"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nigeria: verified profile, 28 tracker records and partnership map
Three independent verifiers; single-verifier flags re-checked in resolution.
Adds the 20 October 2026 Ebola case and newer CBN, NBS and NHIA figures.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ChEN58PbdXFZmwUoBZYBRb
</commit_message>
<xml_diff>
--- a/output/Partnerships_Tracker.xlsx
+++ b/output/Partnerships_Tracker.xlsx
@@ -231,8 +231,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tracker" displayName="Tracker" ref="A1:L122" headerRowCount="1">
-  <autoFilter ref="A1:L122"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tracker" displayName="Tracker" ref="A1:L150" headerRowCount="1">
+  <autoFilter ref="A1:L150"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Status"/>
     <tableColumn id="2" name="Country"/>
@@ -558,7 +558,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Scope: partnerships that are active, or ended or last active within the past five years. Last checked 2026-10-20.</t>
+          <t>Scope: partnerships that are active, or ended or last active within the past five years. Last checked 2026-10-21.</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Tracker!$A$2:$A$122,A5)</f>
+        <f>COUNTIF(Tracker!$A$2:$A$150,A5)</f>
         <v/>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF(Tracker!$A$2:$A$122,A6)</f>
+        <f>COUNTIF(Tracker!$A$2:$A$150,A6)</f>
         <v/>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Tracker!$A$2:$A$122,A7)</f>
+        <f>COUNTIF(Tracker!$A$2:$A$150,A7)</f>
         <v/>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -670,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L122"/>
+  <dimension ref="A1:L150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7732,6 +7732,1622 @@
       <c r="L122" s="14" t="inlineStr">
         <is>
           <t>The Edge Malaysia, 2024-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B123" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C123" s="13" t="inlineStr">
+        <is>
+          <t>Johns Hopkins University (Johns Hopkins Hospital)</t>
+        </is>
+      </c>
+      <c r="D123" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E123" s="12" t="inlineStr">
+        <is>
+          <t>Afe Babalola University (ABUAD)</t>
+        </is>
+      </c>
+      <c r="F123" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G123" s="12" t="inlineStr">
+        <is>
+          <t>Tripartite agreement with the Little by Little Foundation letting high performing ABUAD medical students do part of their fifth year clinical electives at Johns Hopkins Hospital.</t>
+        </is>
+      </c>
+      <c r="H123" s="12" t="inlineStr">
+        <is>
+          <t>2023-01</t>
+        </is>
+      </c>
+      <c r="I123" s="12" t="inlineStr"/>
+      <c r="J123" s="12" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="K123" s="12" t="inlineStr">
+        <is>
+          <t>ABUAD notice dated 17 January 2023 reports the signing on 10 January 2023. No later evidence of placements found in 2024 to 2026 searches. ABUAD's 5 February 2025 release on its seventh induction ceremony describes the six-week Johns Hopkins Hospital electives as ongoing.</t>
+        </is>
+      </c>
+      <c r="L123" s="14" t="inlineStr">
+        <is>
+          <t>Afe Babalola University, 2023-01-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B124" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C124" s="13" t="inlineStr">
+        <is>
+          <t>Mayo Clinic (Mayo Clinic Global Consulting)</t>
+        </is>
+      </c>
+      <c r="D124" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E124" s="12" t="inlineStr">
+        <is>
+          <t>Iwosan Investments Limited (Iwosan Lagoon Hospitals and Lagos Medipark Hospital)</t>
+        </is>
+      </c>
+      <c r="F124" s="12" t="inlineStr">
+        <is>
+          <t>Advisory and consulting</t>
+        </is>
+      </c>
+      <c r="G124" s="12" t="inlineStr">
+        <is>
+          <t>Iwosan Investments, owner of the Iwosan Lagoon Hospitals group, engaged Mayo Clinic Global Consulting for strategic advice on organisation and clinical practice. The work starts with Iwosan Lagoon Hospitals and the planned Lagos Medipark Hospital.</t>
+        </is>
+      </c>
+      <c r="H124" s="12" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="I124" s="12" t="inlineStr"/>
+      <c r="J124" s="12" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="K124" s="12" t="inlineStr">
+        <is>
+          <t>Iwosan's announcement was syndicated on 17 April 2025 (The Sun) and carried by BusinessDay and BrandIconImage. No page on Mayo's own newsroom was found, so confirmation rests on the Nigerian company's release. No end date or contract term is stated.</t>
+        </is>
+      </c>
+      <c r="L124" s="14" t="inlineStr">
+        <is>
+          <t>The Sun Nigeria, 2025-04-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B125" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C125" s="13" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center</t>
+        </is>
+      </c>
+      <c r="D125" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E125" s="12" t="inlineStr">
+        <is>
+          <t>Lagos University Teaching Hospital (LUTH) and College of Medicine, University of Lagos</t>
+        </is>
+      </c>
+      <c r="F125" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G125" s="12" t="inlineStr">
+        <is>
+          <t>LUTH and the University of Lagos College of Medicine serve as research and training hubs of the MSK founded ARGO consortium. They take part in joint cancer studies, including a colorectal cancer immunotherapy trial.</t>
+        </is>
+      </c>
+      <c r="H125" s="12" t="inlineStr"/>
+      <c r="I125" s="12" t="inlineStr"/>
+      <c r="J125" s="12" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="K125" s="12" t="inlineStr">
+        <is>
+          <t>MSK's 2025 GCRT Update names OAUTHC and the College of Medicine, University of Lagos/LUTH as ARGO's research and training hubs. MSK's press page describes the colorectal immunotherapy trial with OAUTHC, LUTH and Medserve. Start year not stated on a dated page.</t>
+        </is>
+      </c>
+      <c r="L125" s="14" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B126" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C126" s="13" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center</t>
+        </is>
+      </c>
+      <c r="D126" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E126" s="12" t="inlineStr">
+        <is>
+          <t>Obafemi Awolowo University Teaching Hospitals Complex (OAUTHC)</t>
+        </is>
+      </c>
+      <c r="F126" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G126" s="12" t="inlineStr">
+        <is>
+          <t>MSK's Global Cancer Research and Training program partners with OAUTHC, home of the African Research Group for Oncology (ARGO), an NCI recognised consortium founded in 2013. The work covers cancer research, trials and training for Nigerian clinicians.</t>
+        </is>
+      </c>
+      <c r="H126" s="12" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+      <c r="I126" s="12" t="inlineStr"/>
+      <c r="J126" s="12" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="K126" s="12" t="inlineStr">
+        <is>
+          <t>MSK's 2025 GCRT Update reports the annual ARGO symposium held at Ile-Ife in September 2025 and a colorectal immunotherapy trial run with OAUTHC. MSK's program page dates the partnership to the 2009 training of OAUTHC surgeon Isaac Alatise; start year is that visit, ARGO itself dates to 2013.</t>
+        </is>
+      </c>
+      <c r="L126" s="14" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B127" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C127" s="13" t="inlineStr">
+        <is>
+          <t>St. Jude Children's Research Hospital</t>
+        </is>
+      </c>
+      <c r="D127" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E127" s="12" t="inlineStr">
+        <is>
+          <t>Abubakar Tafawa Balewa University Teaching Hospital (ATBUTH)</t>
+        </is>
+      </c>
+      <c r="F127" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G127" s="12" t="inlineStr">
+        <is>
+          <t>ATBUTH signed a Medical Institution Membership Agreement and joined the St. Jude Global Alliance, a care and training network for childhood cancer. Membership gives access to mentorship, shared treatment protocols and training.</t>
+        </is>
+      </c>
+      <c r="H127" s="12" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="I127" s="12" t="inlineStr"/>
+      <c r="J127" s="12" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="K127" s="12" t="inlineStr">
+        <is>
+          <t>Leadership newspaper published the hospital's statement on 26 October 2025 (signing described as the day before). Not confirmed on St. Jude's own site.</t>
+        </is>
+      </c>
+      <c r="L127" s="14" t="inlineStr">
+        <is>
+          <t>Leadership Newspapers, 2025-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B128" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C128" s="13" t="inlineStr">
+        <is>
+          <t>St. Jude Children's Research Hospital</t>
+        </is>
+      </c>
+      <c r="D128" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E128" s="12" t="inlineStr">
+        <is>
+          <t>The Dorcas Cancer Foundation (TDCF)</t>
+        </is>
+      </c>
+      <c r="F128" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G128" s="12" t="inlineStr">
+        <is>
+          <t>TDCF joined the St. Jude Global Alliance as the first Nigerian non profit member, to improve paediatric cancer outcomes in Nigeria and sub Saharan Africa. TDCF runs a paediatric radiation oncology training course.</t>
+        </is>
+      </c>
+      <c r="H128" s="12" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="I128" s="12" t="inlineStr"/>
+      <c r="J128" s="12" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="K128" s="12" t="inlineStr">
+        <is>
+          <t>ThisDay and BusinessDay reported the admission on 17 December 2024. The Nigerian party is a non profit, not a hospital, and the tie is an alliance membership; flag for the verifier. Not confirmed on St. Jude's site. Caveat: the Nigerian party is a cancer foundation working with pediatric oncology units, not a hospital.</t>
+        </is>
+      </c>
+      <c r="L128" s="14" t="inlineStr">
+        <is>
+          <t>ThisDay, 2024-12-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B129" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C129" s="13" t="inlineStr">
+        <is>
+          <t>University of Illinois Chicago (UIC School of Public Health)</t>
+        </is>
+      </c>
+      <c r="D129" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E129" s="12" t="inlineStr">
+        <is>
+          <t>Lagos State University (LASU)</t>
+        </is>
+      </c>
+      <c r="F129" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G129" s="12" t="inlineStr">
+        <is>
+          <t>Framework agreement signed 28 July 2026 for academic collaboration, joint research and student and faculty exchange, focused on urban health, emergency preparedness and AI-enabled public health tools.</t>
+        </is>
+      </c>
+      <c r="H129" s="12" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="I129" s="12" t="inlineStr"/>
+      <c r="J129" s="12" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="K129" s="12" t="inlineStr">
+        <is>
+          <t>UIC School of Public Health news, 4 August 2026, reports the memorandum signed on 28 July 2026 in Chicago by LASU's Vice Chancellor and UIC representatives. A university to university agreement with no hospital named.</t>
+        </is>
+      </c>
+      <c r="L129" s="14" t="inlineStr">
+        <is>
+          <t>UIC School of Public Health, 2026-08-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B130" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C130" s="13" t="inlineStr">
+        <is>
+          <t>University of Maryland School of Medicine (Institute of Human Virology)</t>
+        </is>
+      </c>
+      <c r="D130" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E130" s="12" t="inlineStr">
+        <is>
+          <t>Institute of Human Virology Nigeria (IHVN)</t>
+        </is>
+      </c>
+      <c r="F130" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G130" s="12" t="inlineStr">
+        <is>
+          <t>IHVN is the Nigerian affiliate of the Maryland Institute of Human Virology, delivering HIV, TB and cancer care, training and research. It opened a multi campus site in Abuja in 2023.</t>
+        </is>
+      </c>
+      <c r="H130" s="12" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="I130" s="12" t="inlineStr"/>
+      <c r="J130" s="12" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="K130" s="12" t="inlineStr">
+        <is>
+          <t>University of Maryland news from June 2023 reports the Abuja campus launch with UMB leadership present. No dated evidence from October 2024 onward found. IHVN is an NGO affiliate, not a hospital; flag for the verifier. NIH RePORTER shows Fogarty training grant D43TW012280 awarded to IHVN for FY2026 (budget start 1 February 2026), co-led with the UMSOM Institute of Human Virology. Caveat: IHVN is the Institute's Nigerian NGO affiliate, not a hospital.</t>
+        </is>
+      </c>
+      <c r="L130" s="14" t="inlineStr">
+        <is>
+          <t>University of Maryland School of Medicine, 2023-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B131" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C131" s="13" t="inlineStr">
+        <is>
+          <t>University of Miami (Sylvester Comprehensive Cancer Center)</t>
+        </is>
+      </c>
+      <c r="D131" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E131" s="12" t="inlineStr">
+        <is>
+          <t>Ahmadu Bello University Teaching Hospital (ABUTH)</t>
+        </is>
+      </c>
+      <c r="F131" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G131" s="12" t="inlineStr">
+        <is>
+          <t>ABUTH is a recruiting site in a University of Miami led trial of niraparib maintenance therapy for ovarian cancer in women of African ancestry. The tie began with a Miami delegation visit to ABUTH in 2023.</t>
+        </is>
+      </c>
+      <c r="H131" s="12" t="inlineStr">
+        <is>
+          <t>2023-08</t>
+        </is>
+      </c>
+      <c r="I131" s="12" t="inlineStr"/>
+      <c r="J131" s="12" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="K131" s="12" t="inlineStr">
+        <is>
+          <t>ClinicalTrials.gov NCT06412120 lists ABUTH Zaria as recruiting, study start 28 July 2026, record updated 5 August 2026, Miami investigators Schlumbrecht and George. ABUTH's August 2023 news item reports the planning visit (page not retrievable; seen in search results only).</t>
+        </is>
+      </c>
+      <c r="L131" s="14" t="inlineStr">
+        <is>
+          <t>US National Library of Medicine, 2026-08-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B132" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C132" s="13" t="inlineStr">
+        <is>
+          <t>University of Virginia Health System</t>
+        </is>
+      </c>
+      <c r="D132" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E132" s="12" t="inlineStr">
+        <is>
+          <t>Federal Medical Centre Umuahia</t>
+        </is>
+      </c>
+      <c r="F132" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G132" s="12" t="inlineStr">
+        <is>
+          <t>UVA nephrology supports the kidney transplant programme at FMC Umuahia through mentorship, coordinator training and joint research under the ISN and TTS Sister Transplant Centers Program. The pair reached Level B in 2026.</t>
+        </is>
+      </c>
+      <c r="H132" s="12" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I132" s="12" t="inlineStr"/>
+      <c r="J132" s="12" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="K132" s="12" t="inlineStr">
+        <is>
+          <t>UVA Medicine in Motion news, 13 May 2026, reports the move from Level C to Level B, shorter post transplant stays (14 to 8 days), four trained coordinators and eight joint publications in the first two years, which puts the start near 2024.</t>
+        </is>
+      </c>
+      <c r="L132" s="14" t="inlineStr">
+        <is>
+          <t>UVA Medicine in Motion, 2026-05-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B133" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C133" s="13" t="inlineStr">
+        <is>
+          <t>Vanderbilt University Medical Center (Vanderbilt Institute for Global Health)</t>
+        </is>
+      </c>
+      <c r="D133" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E133" s="12" t="inlineStr">
+        <is>
+          <t>Aminu Kano Teaching Hospital and Bayero University Kano</t>
+        </is>
+      </c>
+      <c r="F133" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G133" s="12" t="inlineStr">
+        <is>
+          <t>Long running research and training partnership, now in its second Fogarty funded phase (V-BRCH 2), building Nigerian capacity for clinical research on HIV and related chronic diseases. Related programmes cover child neurology and research administration.</t>
+        </is>
+      </c>
+      <c r="H133" s="12" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="I133" s="12" t="inlineStr"/>
+      <c r="J133" s="12" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="K133" s="12" t="inlineStr">
+        <is>
+          <t>Fogarty grant D43TW011544 lists Aminu Kano Teaching Hospital as principal institution with award years 2020 to 2029, and Vanderbilt's V-BRCH page describes V-BRCH 2 as a continuation. Both pages are undated, so last evidence reflects page content as read on 16 October 2026; flag for the verifier. Start year is the 2020 award; the AKTH tie is older. Fogarty grant D43TW011544 was renewed in 2025 with Aminu Kano Teaching Hospital as grantee; the FY2026 award notice is dated 18 December 2025 (NIH RePORTER).</t>
+        </is>
+      </c>
+      <c r="L133" s="14" t="inlineStr">
+        <is>
+          <t>US National Institutes of Health</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B134" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C134" s="13" t="inlineStr">
+        <is>
+          <t>Virginia Commonwealth University (VCU Massey Comprehensive Cancer Center)</t>
+        </is>
+      </c>
+      <c r="D134" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E134" s="12" t="inlineStr">
+        <is>
+          <t>National Hospital Abuja</t>
+        </is>
+      </c>
+      <c r="F134" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G134" s="12" t="inlineStr">
+        <is>
+          <t>Two year memorandum of understanding between the National Hospital and VCU Massey Comprehensive Cancer Center to build cancer research capacity. Focus areas are clinical trials, training of new scientists and moving research into patient care.</t>
+        </is>
+      </c>
+      <c r="H134" s="12" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="I134" s="12" t="inlineStr"/>
+      <c r="J134" s="12" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="K134" s="12" t="inlineStr">
+        <is>
+          <t>News Agency of Nigeria and Nairametrics reported the signing on 1 July 2025 by Prof Muhammad Mahmud and Dr Robert Winn, saying it was signed on a Tuesday (24 June or 1 July 2025). Term is two years, so it runs to mid 2027.</t>
+        </is>
+      </c>
+      <c r="L134" s="14" t="inlineStr">
+        <is>
+          <t>Nairametrics, 2025-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B135" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C135" s="13" t="inlineStr">
+        <is>
+          <t>Evercare Group (owned at its 2021 launch by the TPG-managed Evercare Health Fund)</t>
+        </is>
+      </c>
+      <c r="D135" s="12" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="E135" s="12" t="inlineStr">
+        <is>
+          <t>Evercare Hospital Lekki</t>
+        </is>
+      </c>
+      <c r="F135" s="12" t="inlineStr">
+        <is>
+          <t>Ownership or management</t>
+        </is>
+      </c>
+      <c r="G135" s="12" t="inlineStr">
+        <is>
+          <t>Evercare Group owns and operates Evercare Hospital Lekki, a 165-bed tertiary hospital in Lagos that opened in February 2021, as part of its network of hospitals in Africa and South Asia.</t>
+        </is>
+      </c>
+      <c r="H135" s="12" t="inlineStr">
+        <is>
+          <t>2021-03</t>
+        </is>
+      </c>
+      <c r="I135" s="12" t="inlineStr"/>
+      <c r="J135" s="12" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="K135" s="12" t="inlineStr">
+        <is>
+          <t>ThisDay, 10 October 2024, describes Evercare Hospital Lekki as part of the Evercare Group, which operates in Kenya and Pakistan as well as Nigeria, announcing new cochlear implant surgery. TPG's release and a 2021 report document the group's ownership and the February 2021 opening. A 2026 LinkedIn post suggests continued operation but was not verified. Ownership is as of the 2021 launch; no later ownership confirmation was found.</t>
+        </is>
+      </c>
+      <c r="L135" s="14" t="inlineStr">
+        <is>
+          <t>ThisDay, 2024-10-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B136" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C136" s="13" t="inlineStr">
+        <is>
+          <t>King's College Hospital NHS Foundation Trust</t>
+        </is>
+      </c>
+      <c r="D136" s="12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E136" s="12" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="F136" s="12" t="inlineStr">
+        <is>
+          <t>Advisory and consulting</t>
+        </is>
+      </c>
+      <c r="G136" s="12" t="inlineStr">
+        <is>
+          <t>King's is the appointed Clinical Partner of the AMCE, supporting clinical protocols, governance, service set-up, recruitment and training for the 170-bed specialist hospital in Abuja. Clinical services were commissioned in June 2025.</t>
+        </is>
+      </c>
+      <c r="H136" s="12" t="inlineStr">
+        <is>
+          <t>2021-06</t>
+        </is>
+      </c>
+      <c r="I136" s="12" t="inlineStr"/>
+      <c r="J136" s="12" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="K136" s="12" t="inlineStr">
+        <is>
+          <t>Afreximbank announced on 3 June 2021 that it had signed an agreement appointing King's College Hospital as Clinical Partner. Nairametrics reports the AMCE was commissioned on 5 June 2025 with Vice President Shettima praising the AMCE and King's partnership. Brand Spur (19 September 2026) describes the centre as developed with King's College Hospital and now commissioned.</t>
+        </is>
+      </c>
+      <c r="L136" s="14" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (amce.net), 2021-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B137" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C137" s="13" t="inlineStr">
+        <is>
+          <t>King's College London</t>
+        </is>
+      </c>
+      <c r="D137" s="12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E137" s="12" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="F137" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G137" s="12" t="inlineStr">
+        <is>
+          <t>King's College London and Afreximbank agreed to plan a medical and nursing school at the AMCE in Abuja, drawing on King's healthcare education expertise. A further terms of agreement was signed in June 2025.</t>
+        </is>
+      </c>
+      <c r="H137" s="12" t="inlineStr">
+        <is>
+          <t>2023-11</t>
+        </is>
+      </c>
+      <c r="I137" s="12" t="inlineStr"/>
+      <c r="J137" s="12" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="K137" s="12" t="inlineStr">
+        <is>
+          <t>King's news release of 28 November 2023 reports the memorandum of agreement signed on 24 November 2023 for a scoping study of the school. Nairametrics reports a terms of agreement between Afreximbank and King's College London on the school was signed at the AMCE commissioning on 5 June 2025.</t>
+        </is>
+      </c>
+      <c r="L137" s="14" t="inlineStr">
+        <is>
+          <t>King's College London, 2023-11-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B138" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C138" s="13" t="inlineStr">
+        <is>
+          <t>Liverpool School of Tropical Medicine</t>
+        </is>
+      </c>
+      <c r="D138" s="12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E138" s="12" t="inlineStr">
+        <is>
+          <t>National Postgraduate Medical College of Nigeria (with Wellbeing Foundation Africa)</t>
+        </is>
+      </c>
+      <c r="F138" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G138" s="12" t="inlineStr">
+        <is>
+          <t>LSTM leads Advanced Obstetrics and Surgical Skills training for obstetrics and gynaecology examiners and residents of the National Postgraduate Medical College, with centres of excellence in Lagos and Abuja and later sites in Port Harcourt and Gombe. It is funded by the UK Global Health Workforce Programme.</t>
+        </is>
+      </c>
+      <c r="H138" s="12" t="inlineStr">
+        <is>
+          <t>2024-02</t>
+        </is>
+      </c>
+      <c r="I138" s="12" t="inlineStr"/>
+      <c r="J138" s="12" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="K138" s="12" t="inlineStr">
+        <is>
+          <t>LSTM reports the course began on 6 May 2024 at the college's centre of excellence at LUTH. The Wellbeing Foundation Africa reported on 12 February 2025 that 225 doctors had been trained, and on 22 May 2025 that training had expanded to the University of Port Harcourt Teaching Hospital. LSTM's May 2024 release names the site as 'Lagos State University Teaching Hospital (LUTH)', which is ambiguous; WBFA reported 225 examiners and 120 residents trained by May 2025.</t>
+        </is>
+      </c>
+      <c r="L138" s="14" t="inlineStr">
+        <is>
+          <t>Liverpool School of Tropical Medicine, 2024-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B139" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C139" s="13" t="inlineStr">
+        <is>
+          <t>Manipal Hospitals</t>
+        </is>
+      </c>
+      <c r="D139" s="12" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E139" s="12" t="inlineStr">
+        <is>
+          <t>Afe Babalola University Multi-System Hospital</t>
+        </is>
+      </c>
+      <c r="F139" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G139" s="12" t="inlineStr">
+        <is>
+          <t>Afe Babalola University Multi-System Hospital and Manipal Hospitals signed an MoU to expand capacity, deepen specialist training, improve clinical exchange and support advanced surgical care.</t>
+        </is>
+      </c>
+      <c r="H139" s="12" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="I139" s="12" t="inlineStr"/>
+      <c r="J139" s="12" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="K139" s="12" t="inlineStr">
+        <is>
+          <t>News Agency of Nigeria, 26 June 2026, reports the MoU announced at a press briefing by the hospital's chief medical director, with Dr Rajit Sood speaking for Manipal and the university's Vice-Chancellor present.</t>
+        </is>
+      </c>
+      <c r="L139" s="14" t="inlineStr">
+        <is>
+          <t>News Agency of Nigeria, 2026-06-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B140" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C140" s="13" t="inlineStr">
+        <is>
+          <t>The Christie NHS Foundation Trust</t>
+        </is>
+      </c>
+      <c r="D140" s="12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E140" s="12" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="F140" s="12" t="inlineStr">
+        <is>
+          <t>Advisory and consulting</t>
+        </is>
+      </c>
+      <c r="G140" s="12" t="inlineStr">
+        <is>
+          <t>The Christie, through Christie International, is the oncology partner to King's College Hospital in advising the AMCE, supporting oncology staff recruitment, education and quality assurance. It continues to support the oncology service after opening.</t>
+        </is>
+      </c>
+      <c r="H140" s="12" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="I140" s="12" t="inlineStr"/>
+      <c r="J140" s="12" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="K140" s="12" t="inlineStr">
+        <is>
+          <t>The Christie's news story of 25 October 2024 reports an AMCE delegation visit to Manchester and says its advice, which began in 2021, would continue into operations. The Christie's project page, as indexed in search, states that clinical services were commissioned on 5 June 2025 with Christie International's head attending.</t>
+        </is>
+      </c>
+      <c r="L140" s="14" t="inlineStr">
+        <is>
+          <t>The Christie NHS Foundation Trust, 2024-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B141" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C141" s="13" t="inlineStr">
+        <is>
+          <t>The Royal Marsden NHS Foundation Trust</t>
+        </is>
+      </c>
+      <c r="D141" s="12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E141" s="12" t="inlineStr">
+        <is>
+          <t>Marcelle Ruth Cancer Centre &amp; Specialist Hospital</t>
+        </is>
+      </c>
+      <c r="F141" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G141" s="12" t="inlineStr">
+        <is>
+          <t>The two cancer centres signed a strategic partnership covering clinical expertise, research, professional development and training, aimed at keeping cancer care in Nigeria and West Africa.</t>
+        </is>
+      </c>
+      <c r="H141" s="12" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="I141" s="12" t="inlineStr"/>
+      <c r="J141" s="12" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="K141" s="12" t="inlineStr">
+        <is>
+          <t>BusinessDay reported on 24 September 2026 that Marcelle Ruth had entered a strategic partnership with The Royal Marsden. Search results also show the agreement described as an MoU on a Royal Marsden Private Care LinkedIn post; no Royal Marsden press release was found.</t>
+        </is>
+      </c>
+      <c r="L141" s="14" t="inlineStr">
+        <is>
+          <t>BusinessDay, 2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B142" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C142" s="13" t="inlineStr">
+        <is>
+          <t>University of Birmingham</t>
+        </is>
+      </c>
+      <c r="D142" s="12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E142" s="12" t="inlineStr">
+        <is>
+          <t>University of Lagos (with Lagos University Teaching Hospital)</t>
+        </is>
+      </c>
+      <c r="F142" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G142" s="12" t="inlineStr">
+        <is>
+          <t>The University of Lagos and the University of Birmingham signed a memorandum on transnational education covering student and staff exchange and curriculum development. It builds on more than a decade of global surgery collaboration that introduced a master's programme in surgery at LUTH.</t>
+        </is>
+      </c>
+      <c r="H142" s="12" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="I142" s="12" t="inlineStr"/>
+      <c r="J142" s="12" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="K142" s="12" t="inlineStr">
+        <is>
+          <t>Vanguard, 29 January 2026, reports the MoU signed at UNILAG's Senate Chamber, witnessed by the Minister of Education; UNILAG's Vice Chancellor cites the Birmingham global surgery work and the LUTH master's in surgery. Birmingham described the MoU as a statement of intent. Not yet confirmed on Birmingham's newsroom.</t>
+        </is>
+      </c>
+      <c r="L142" s="14" t="inlineStr">
+        <is>
+          <t>Vanguard, 29 January 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B143" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C143" s="13" t="inlineStr">
+        <is>
+          <t>University of Glasgow</t>
+        </is>
+      </c>
+      <c r="D143" s="12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E143" s="12" t="inlineStr">
+        <is>
+          <t>Ahmadu Bello University</t>
+        </is>
+      </c>
+      <c r="F143" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G143" s="12" t="inlineStr">
+        <is>
+          <t>A university-level MoU provides a framework for joint research programmes, postgraduate co-supervision and academic exchange on global health challenges, coordinated by the School of Infection and Immunity. A university-wide MoU; no teaching-hospital or clinical component is named.</t>
+        </is>
+      </c>
+      <c r="H143" s="12" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="I143" s="12" t="inlineStr"/>
+      <c r="J143" s="12" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="K143" s="12" t="inlineStr">
+        <is>
+          <t>The University of Glasgow news item of 12 May 2026 reports the MoU signed during a visit on 28 and 29 April 2026, following an exploratory visit in December 2025. The MoU is university-wide and not limited to the teaching hospital.</t>
+        </is>
+      </c>
+      <c r="L143" s="14" t="inlineStr">
+        <is>
+          <t>University of Glasgow, 2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B144" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C144" s="13" t="inlineStr">
+        <is>
+          <t>University of Maryland School of Medicine</t>
+        </is>
+      </c>
+      <c r="D144" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E144" s="12" t="inlineStr">
+        <is>
+          <t>Lagos University Teaching Hospital (LUTH)</t>
+        </is>
+      </c>
+      <c r="F144" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G144" s="12" t="inlineStr">
+        <is>
+          <t>The University of Maryland School of Medicine and LUTH announced a chronic disease collaboration in August 2024, initially for four to five years with a stated ten-year ambition.</t>
+        </is>
+      </c>
+      <c r="H144" s="12" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="I144" s="12" t="inlineStr"/>
+      <c r="J144" s="12" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="K144" s="12" t="inlineStr">
+        <is>
+          <t>Nairametrics (19 August 2024) and LUTH report a partnership planned over ten years, following a visit by Dean Mark Gladwin. No signed text or later 2024 to 2026 update found, so it falls just before the Active cutoff.</t>
+        </is>
+      </c>
+      <c r="L144" s="14" t="inlineStr">
+        <is>
+          <t>Lagos University Teaching Hospital, 2024-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B145" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C145" s="13" t="inlineStr">
+        <is>
+          <t>University of Virginia Health System</t>
+        </is>
+      </c>
+      <c r="D145" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E145" s="12" t="inlineStr">
+        <is>
+          <t>Federal Medical Centre Owo</t>
+        </is>
+      </c>
+      <c r="F145" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G145" s="12" t="inlineStr">
+        <is>
+          <t>UVA's nephrology division built a partnership with FMC Owo covering research and career development programmes, with the International Society of Nephrology, and donated textbooks.</t>
+        </is>
+      </c>
+      <c r="H145" s="12" t="inlineStr"/>
+      <c r="I145" s="12" t="inlineStr"/>
+      <c r="J145" s="12" t="inlineStr">
+        <is>
+          <t>2023-01</t>
+        </is>
+      </c>
+      <c r="K145" s="12" t="inlineStr">
+        <is>
+          <t>UVA news item describes a textbook donation on 6 January 2023. No later dated evidence found, and the work may now sit inside the FMC Umuahia programme.</t>
+        </is>
+      </c>
+      <c r="L145" s="14" t="inlineStr">
+        <is>
+          <t>UVA Medicine in Motion, 2023-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B146" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C146" s="13" t="inlineStr">
+        <is>
+          <t>Yale School of Medicine (Department of Psychiatry)</t>
+        </is>
+      </c>
+      <c r="D146" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E146" s="12" t="inlineStr">
+        <is>
+          <t>Imo State University Teaching Hospital</t>
+        </is>
+      </c>
+      <c r="F146" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G146" s="12" t="inlineStr">
+        <is>
+          <t>Yale's HAPPINESS Project, run with the Imo State teaching hospital, trains primary care workers to treat mental, neurological and substance use disorders, with telemedicine specialist support. It has begun integrating mental health into HIV clinics.</t>
+        </is>
+      </c>
+      <c r="H146" s="12" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="I146" s="12" t="inlineStr"/>
+      <c r="J146" s="12" t="inlineStr">
+        <is>
+          <t>2023-09</t>
+        </is>
+      </c>
+      <c r="K146" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria Health Watch, 6 September 2023, reports over 100 workers trained; Yale's programme page is undated. No dated evidence from October 2024 onward found. The teaching hospital is in Orlu, Imo State.</t>
+        </is>
+      </c>
+      <c r="L146" s="14" t="inlineStr">
+        <is>
+          <t>Nigeria Health Watch, 2023-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B147" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C147" s="13" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals</t>
+        </is>
+      </c>
+      <c r="D147" s="12" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E147" s="12" t="inlineStr">
+        <is>
+          <t>Duchess International Hospital (Reddington Hospital Group)</t>
+        </is>
+      </c>
+      <c r="F147" s="12" t="inlineStr">
+        <is>
+          <t>Ownership or management</t>
+        </is>
+      </c>
+      <c r="G147" s="12" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals supports the operation and management of the 100-bed Duchess International Hospital in Ikeja, Lagos, to strengthen efficiency and clinical quality. The arrangement was announced when the hospital launched in October 2021.</t>
+        </is>
+      </c>
+      <c r="H147" s="12" t="inlineStr">
+        <is>
+          <t>2021-10</t>
+        </is>
+      </c>
+      <c r="I147" s="12" t="inlineStr"/>
+      <c r="J147" s="12" t="inlineStr">
+        <is>
+          <t>2021-11</t>
+        </is>
+      </c>
+      <c r="K147" s="12" t="inlineStr">
+        <is>
+          <t>ThisDay (11 November 2021) and New Telegraph report that operation and management of the Duchess are supported by Apollo Hospitals, India. No dated confirmation from October 2024 onward was found; the hospital's 2024 and 2025 award releases do not mention Apollo.</t>
+        </is>
+      </c>
+      <c r="L147" s="14" t="inlineStr">
+        <is>
+          <t>ThisDay, 11 November 2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B148" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C148" s="13" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals</t>
+        </is>
+      </c>
+      <c r="D148" s="12" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E148" s="12" t="inlineStr">
+        <is>
+          <t>State House Clinic</t>
+        </is>
+      </c>
+      <c r="F148" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G148" s="12" t="inlineStr">
+        <is>
+          <t>Apollo doctors visit the State House Clinic to give free consultations and lectures, and clinic staff have been sent to Apollo in India for up to six weeks of training at no charge.</t>
+        </is>
+      </c>
+      <c r="H148" s="12" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="I148" s="12" t="inlineStr"/>
+      <c r="J148" s="12" t="inlineStr">
+        <is>
+          <t>2022-07</t>
+        </is>
+      </c>
+      <c r="K148" s="12" t="inlineStr">
+        <is>
+          <t>Blueprint, 29 July 2022, quotes the clinic's medical director describing a collaboration of almost six to seven years and a visiting Apollo team in Abuja. Start year is approximate, back-calculated from that quote. No later dated activity was found; a March 2024 ThisDay report records only Apollo's stated intent to partner with Nigerian hospitals.</t>
+        </is>
+      </c>
+      <c r="L148" s="14" t="inlineStr">
+        <is>
+          <t>Blueprint, 2022-07-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B149" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C149" s="13" t="inlineStr">
+        <is>
+          <t>Memorial Hospitals Group</t>
+        </is>
+      </c>
+      <c r="D149" s="12" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="E149" s="12" t="inlineStr">
+        <is>
+          <t>Kasi Healthcare</t>
+        </is>
+      </c>
+      <c r="F149" s="12" t="inlineStr">
+        <is>
+          <t>Telehealth and second opinion</t>
+        </is>
+      </c>
+      <c r="G149" s="12" t="inlineStr">
+        <is>
+          <t>Memorial specialists provide second opinions and specialist screenings, with monthly visiting specialists and training courses for Nigerian providers at Kasi's Lagos airport clinic, linked to referral of patients to Turkey. Close to a patient-referral arrangement.</t>
+        </is>
+      </c>
+      <c r="H149" s="12" t="inlineStr">
+        <is>
+          <t>2024-09</t>
+        </is>
+      </c>
+      <c r="I149" s="12" t="inlineStr"/>
+      <c r="J149" s="12" t="inlineStr">
+        <is>
+          <t>2024-09</t>
+        </is>
+      </c>
+      <c r="K149" s="12" t="inlineStr">
+        <is>
+          <t>BusinessDay, 27 September 2024, reports the partnership announced with Memorial's country executive. No later dated activity was found.</t>
+        </is>
+      </c>
+      <c r="L149" s="14" t="inlineStr">
+        <is>
+          <t>BusinessDay, 2024-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B150" s="12" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="C150" s="13" t="inlineStr">
+        <is>
+          <t>Peking University People's Hospital (named variously in press as People's University Hospital, Beijing)</t>
+        </is>
+      </c>
+      <c r="D150" s="12" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E150" s="12" t="inlineStr">
+        <is>
+          <t>University of Abuja Teaching Hospital</t>
+        </is>
+      </c>
+      <c r="F150" s="12" t="inlineStr">
+        <is>
+          <t>Government agreement</t>
+        </is>
+      </c>
+      <c r="G150" s="12" t="inlineStr">
+        <is>
+          <t>A China-Nigeria government letter of intent names these two hospitals as the pioneer project for hospital cooperation under the 2021 FOCAC health programmes, covering knowledge sharing and research.</t>
+        </is>
+      </c>
+      <c r="H150" s="12" t="inlineStr">
+        <is>
+          <t>2022-08</t>
+        </is>
+      </c>
+      <c r="I150" s="12" t="inlineStr"/>
+      <c r="J150" s="12" t="inlineStr">
+        <is>
+          <t>2022-08</t>
+        </is>
+      </c>
+      <c r="K150" s="12" t="inlineStr">
+        <is>
+          <t>Within Nigeria and the University of Abuja Teaching Hospital website report the letter of intent signed in Abuja by the Chinese Ambassador and Nigeria's Health Minister in August 2022. No follow-up activity was found. The Chinese hospital's name varies between sources and is inferred.</t>
+        </is>
+      </c>
+      <c r="L150" s="14" t="inlineStr">
+        <is>
+          <t>Within Nigeria, 2022-08-20</t>
         </is>
       </c>
     </row>
@@ -7858,10 +9474,38 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L120" r:id="rId119"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L121" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L134" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L135" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L136" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L137" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L149" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L150" r:id="rId149"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId122"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId150"/>
   </tableParts>
 </worksheet>
 </file>
@@ -7872,7 +9516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E244"/>
+  <dimension ref="A1:E297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -14455,6 +16099,1417 @@
       <c r="E244" s="5" t="inlineStr">
         <is>
           <t>https://theedgemalaysia.com/node/725855</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="5" t="inlineStr">
+        <is>
+          <t>Johns Hopkins University (Johns Hopkins Hospital)</t>
+        </is>
+      </c>
+      <c r="B245" s="5" t="inlineStr">
+        <is>
+          <t>Afe Babalola University (ABUAD)</t>
+        </is>
+      </c>
+      <c r="C245" s="5" t="inlineStr">
+        <is>
+          <t>Afe Babalola University ABUAD Tripartite agreement with John Hopkins University USA and Little by Little Foundation</t>
+        </is>
+      </c>
+      <c r="D245" s="5" t="inlineStr">
+        <is>
+          <t>2023-01-17</t>
+        </is>
+      </c>
+      <c r="E245" s="5" t="inlineStr">
+        <is>
+          <t>https://www.abuad.edu.ng/abuad-tripartite-agreement-with-john-hopkins-university-usa-and-little-by-little-foundation/</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="5" t="inlineStr">
+        <is>
+          <t>Johns Hopkins University (Johns Hopkins Hospital)</t>
+        </is>
+      </c>
+      <c r="B246" s="5" t="inlineStr">
+        <is>
+          <t>Afe Babalola University (ABUAD)</t>
+        </is>
+      </c>
+      <c r="C246" s="5" t="inlineStr">
+        <is>
+          <t>ThisDay ABUAD, John Hopkins Partner to Boost Medical Training</t>
+        </is>
+      </c>
+      <c r="D246" s="5" t="inlineStr">
+        <is>
+          <t>2023-01-18</t>
+        </is>
+      </c>
+      <c r="E246" s="5" t="inlineStr">
+        <is>
+          <t>https://www.thisdaylive.com/2023/01/18/abuad-john-hopkins-partner-to-boost-medical-training/</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="5" t="inlineStr">
+        <is>
+          <t>Johns Hopkins University (Johns Hopkins Hospital)</t>
+        </is>
+      </c>
+      <c r="B247" s="5" t="inlineStr">
+        <is>
+          <t>Afe Babalola University (ABUAD)</t>
+        </is>
+      </c>
+      <c r="C247" s="5" t="inlineStr">
+        <is>
+          <t>Afe Babalola University ABUAD Holds Seventh Induction Ceremony for Fresh Doctors</t>
+        </is>
+      </c>
+      <c r="D247" s="5" t="inlineStr">
+        <is>
+          <t>5 February 2025</t>
+        </is>
+      </c>
+      <c r="E247" s="5" t="inlineStr">
+        <is>
+          <t>https://vc.abuad.edu.ng/abuad-holds-seventh-induction-ceremony-for-fresh-doctors/</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="5" t="inlineStr">
+        <is>
+          <t>Mayo Clinic (Mayo Clinic Global Consulting)</t>
+        </is>
+      </c>
+      <c r="B248" s="5" t="inlineStr">
+        <is>
+          <t>Iwosan Investments Limited (Iwosan Lagoon Hospitals and Lagos Medipark Hospital)</t>
+        </is>
+      </c>
+      <c r="C248" s="5" t="inlineStr">
+        <is>
+          <t>The Sun Iwosan engages Mayo Clinic to advance high-quality patient-centered healthcare</t>
+        </is>
+      </c>
+      <c r="D248" s="5" t="inlineStr">
+        <is>
+          <t>2025-04-17</t>
+        </is>
+      </c>
+      <c r="E248" s="5" t="inlineStr">
+        <is>
+          <t>https://thesun.ng/iwosan-engages-mayo-clinic-to-advance-high-quality-patient-centered-healthcare/</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="5" t="inlineStr">
+        <is>
+          <t>Mayo Clinic (Mayo Clinic Global Consulting)</t>
+        </is>
+      </c>
+      <c r="B249" s="5" t="inlineStr">
+        <is>
+          <t>Iwosan Investments Limited (Iwosan Lagoon Hospitals and Lagos Medipark Hospital)</t>
+        </is>
+      </c>
+      <c r="C249" s="5" t="inlineStr">
+        <is>
+          <t>BrandIconImage Iwosan Investments Limited Engages Mayo Clinic Global Consulting to Advance High-Quality Patient-Centered Healthcare in Nigeria</t>
+        </is>
+      </c>
+      <c r="D249" s="5" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="E249" s="5" t="inlineStr">
+        <is>
+          <t>https://www.brandiconimage.com/2025/04/iwosan-investments-limited-engages-mayo.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="5" t="inlineStr">
+        <is>
+          <t>Mayo Clinic (Mayo Clinic Global Consulting)</t>
+        </is>
+      </c>
+      <c r="B250" s="5" t="inlineStr">
+        <is>
+          <t>Iwosan Investments Limited (Iwosan Lagoon Hospitals and Lagos Medipark Hospital)</t>
+        </is>
+      </c>
+      <c r="C250" s="5" t="inlineStr">
+        <is>
+          <t>BusinessDay Iwosan engages Mayo Clinic to advance high quality patient centered healthcare in Nigeria</t>
+        </is>
+      </c>
+      <c r="D250" s="5" t="inlineStr">
+        <is>
+          <t>8 April 2025</t>
+        </is>
+      </c>
+      <c r="E250" s="5" t="inlineStr">
+        <is>
+          <t>https://businessday.ng/health/article/iwosan-engages-mayo-clinic-to-advance-high-quality-patient-centered-healthcare-in-nigeria/</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="5" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center</t>
+        </is>
+      </c>
+      <c r="B251" s="5" t="inlineStr">
+        <is>
+          <t>Lagos University Teaching Hospital (LUTH) and College of Medicine, University of Lagos</t>
+        </is>
+      </c>
+      <c r="C251" s="5" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center Global Cancer Research and Training Program 2025 Update</t>
+        </is>
+      </c>
+      <c r="D251" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E251" s="5" t="inlineStr">
+        <is>
+          <t>https://www.mskcc.org/sites/default/files/node/118066/documents/gcrt_report_2026_6_01-29-98-44.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="5" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center</t>
+        </is>
+      </c>
+      <c r="B252" s="5" t="inlineStr">
+        <is>
+          <t>Obafemi Awolowo University Teaching Hospitals Complex (OAUTHC)</t>
+        </is>
+      </c>
+      <c r="C252" s="5" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center Global Cancer Research and Training Program 2025 Update</t>
+        </is>
+      </c>
+      <c r="D252" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E252" s="5" t="inlineStr">
+        <is>
+          <t>https://www.mskcc.org/sites/default/files/node/118066/documents/gcrt_report_2026_6_01-29-98-44.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="5" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center</t>
+        </is>
+      </c>
+      <c r="B253" s="5" t="inlineStr">
+        <is>
+          <t>Obafemi Awolowo University Teaching Hospitals Complex (OAUTHC)</t>
+        </is>
+      </c>
+      <c r="C253" s="5" t="inlineStr">
+        <is>
+          <t>Memorial Sloan Kettering Cancer Center MSK's Global Cancer Research and Training (GCRT) Program</t>
+        </is>
+      </c>
+      <c r="D253" s="5" t="inlineStr"/>
+      <c r="E253" s="5" t="inlineStr">
+        <is>
+          <t>https://www.mskcc.org/hcp-education-training/international/global-cancer-disparities-initiatives</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="5" t="inlineStr">
+        <is>
+          <t>St. Jude Children's Research Hospital</t>
+        </is>
+      </c>
+      <c r="B254" s="5" t="inlineStr">
+        <is>
+          <t>Abubakar Tafawa Balewa University Teaching Hospital (ATBUTH)</t>
+        </is>
+      </c>
+      <c r="C254" s="5" t="inlineStr">
+        <is>
+          <t>Leadership Bauchi Teaching Hospital Seeks Alliance To Strengthen Cancer Care</t>
+        </is>
+      </c>
+      <c r="D254" s="5" t="inlineStr">
+        <is>
+          <t>2025-10-26</t>
+        </is>
+      </c>
+      <c r="E254" s="5" t="inlineStr">
+        <is>
+          <t>https://leadership.ng/bauchi-teaching-hospital-seeks-alliance-to-strengthen-cancer-care/</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="5" t="inlineStr">
+        <is>
+          <t>St. Jude Children's Research Hospital</t>
+        </is>
+      </c>
+      <c r="B255" s="5" t="inlineStr">
+        <is>
+          <t>The Dorcas Cancer Foundation (TDCF)</t>
+        </is>
+      </c>
+      <c r="C255" s="5" t="inlineStr">
+        <is>
+          <t>Sunday Ehigiator TDCF, St. Jude Global Alliance, Partner on Improving Pediatric Cancer Outcomes in Nigeria, Others</t>
+        </is>
+      </c>
+      <c r="D255" s="5" t="inlineStr">
+        <is>
+          <t>2024-12-17</t>
+        </is>
+      </c>
+      <c r="E255" s="5" t="inlineStr">
+        <is>
+          <t>https://www.thisdaylive.com/2024/12/17/tdcf-st-jude-global-alliance-partner-on-improving-pediatric-cancer-outcomes-in-nigeria-others/</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="5" t="inlineStr">
+        <is>
+          <t>St. Jude Children's Research Hospital</t>
+        </is>
+      </c>
+      <c r="B256" s="5" t="inlineStr">
+        <is>
+          <t>The Dorcas Cancer Foundation (TDCF)</t>
+        </is>
+      </c>
+      <c r="C256" s="5" t="inlineStr">
+        <is>
+          <t>BusinessDay TDCF admitted into St Jude Global Alliance to improve pediatric cancer outcomes in Nigeria</t>
+        </is>
+      </c>
+      <c r="D256" s="5" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="E256" s="5" t="inlineStr">
+        <is>
+          <t>https://businessday.ng/life/article/tdcf-admitted-into-st-jude-global-alliance-to-improve-pediatric-cancer-outcomes-in-nigeria/</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="5" t="inlineStr">
+        <is>
+          <t>University of Illinois Chicago (UIC School of Public Health)</t>
+        </is>
+      </c>
+      <c r="B257" s="5" t="inlineStr">
+        <is>
+          <t>Lagos State University (LASU)</t>
+        </is>
+      </c>
+      <c r="C257" s="5" t="inlineStr">
+        <is>
+          <t>UIC School of Public Health UIC and Lagos State University Sign Memorandum of Agreement</t>
+        </is>
+      </c>
+      <c r="D257" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="E257" s="5" t="inlineStr">
+        <is>
+          <t>https://publichealth.uic.edu/news-stories/uic-and-lagos-state-university-sign-memorandum-of-agreement/</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="5" t="inlineStr">
+        <is>
+          <t>University of Maryland School of Medicine (Institute of Human Virology)</t>
+        </is>
+      </c>
+      <c r="B258" s="5" t="inlineStr">
+        <is>
+          <t>Institute of Human Virology Nigeria (IHVN)</t>
+        </is>
+      </c>
+      <c r="C258" s="5" t="inlineStr">
+        <is>
+          <t>University of Maryland School of Medicine University of Maryland Baltimore leadership helps IHV Nigeria launch campus in Abuja</t>
+        </is>
+      </c>
+      <c r="D258" s="5" t="inlineStr">
+        <is>
+          <t>2023-06</t>
+        </is>
+      </c>
+      <c r="E258" s="5" t="inlineStr">
+        <is>
+          <t>https://ihv.umaryland.edu/news/2023/university-of-maryland-baltimore-leadership-helps-ihv-nigeria-launch-state-of-the-art-campus-in-public-healthcare-treatment-training-and-research-in-nigeria.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="5" t="inlineStr">
+        <is>
+          <t>University of Maryland School of Medicine (Institute of Human Virology)</t>
+        </is>
+      </c>
+      <c r="B259" s="5" t="inlineStr">
+        <is>
+          <t>Institute of Human Virology Nigeria (IHVN)</t>
+        </is>
+      </c>
+      <c r="C259" s="5" t="inlineStr">
+        <is>
+          <t>US National Institutes of Health RePORTER: 5D43TW012280-05, Expanding the pool of Independent Investigators in Implementation Science (Institute of Human Virology Nigeria)</t>
+        </is>
+      </c>
+      <c r="D259" s="5" t="inlineStr">
+        <is>
+          <t>FY2026 (budget start 1 February 2026)</t>
+        </is>
+      </c>
+      <c r="E259" s="5" t="inlineStr">
+        <is>
+          <t>https://reporter.nih.gov/project-details/11251575</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="5" t="inlineStr">
+        <is>
+          <t>University of Miami (Sylvester Comprehensive Cancer Center)</t>
+        </is>
+      </c>
+      <c r="B260" s="5" t="inlineStr">
+        <is>
+          <t>Ahmadu Bello University Teaching Hospital (ABUTH)</t>
+        </is>
+      </c>
+      <c r="C260" s="5" t="inlineStr">
+        <is>
+          <t>ClinicalTrials.gov Study Evaluating Safety, Tolerability, and Metabolism of Niraparib (NCT06412120)</t>
+        </is>
+      </c>
+      <c r="D260" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="E260" s="5" t="inlineStr">
+        <is>
+          <t>https://clinicaltrials.gov/study/NCT06412120</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="5" t="inlineStr">
+        <is>
+          <t>University of Miami (Sylvester Comprehensive Cancer Center)</t>
+        </is>
+      </c>
+      <c r="B261" s="5" t="inlineStr">
+        <is>
+          <t>Ahmadu Bello University Teaching Hospital (ABUTH)</t>
+        </is>
+      </c>
+      <c r="C261" s="5" t="inlineStr">
+        <is>
+          <t>Ahmadu Bello University ABUTH to begin clinical trials on ovarian cancer next year</t>
+        </is>
+      </c>
+      <c r="D261" s="5" t="inlineStr">
+        <is>
+          <t>2023-08</t>
+        </is>
+      </c>
+      <c r="E261" s="5" t="inlineStr">
+        <is>
+          <t>https://abu.edu.ng/abuth-to-begin-clinical-trials-on-ovarian-cancer-next-year/</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="5" t="inlineStr">
+        <is>
+          <t>University of Miami (Sylvester Comprehensive Cancer Center)</t>
+        </is>
+      </c>
+      <c r="B262" s="5" t="inlineStr">
+        <is>
+          <t>Ahmadu Bello University Teaching Hospital (ABUTH)</t>
+        </is>
+      </c>
+      <c r="C262" s="5" t="inlineStr">
+        <is>
+          <t>US National Library of Medicine NCT06412120: Niraparib as Maintenance Following Front-Line Treatment for Ovarian Cancer in Women of African Ancestry</t>
+        </is>
+      </c>
+      <c r="D262" s="5" t="inlineStr">
+        <is>
+          <t>5 August 2026</t>
+        </is>
+      </c>
+      <c r="E262" s="5" t="inlineStr">
+        <is>
+          <t>https://clinicaltrials.gov/study/NCT06412120</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="5" t="inlineStr">
+        <is>
+          <t>University of Virginia Health System</t>
+        </is>
+      </c>
+      <c r="B263" s="5" t="inlineStr">
+        <is>
+          <t>Federal Medical Centre Umuahia</t>
+        </is>
+      </c>
+      <c r="C263" s="5" t="inlineStr">
+        <is>
+          <t>UVA School of Medicine UVA Partners With Federal Medical Center in Nigeria to Elevate Global Kidney Care</t>
+        </is>
+      </c>
+      <c r="D263" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="E263" s="5" t="inlineStr">
+        <is>
+          <t>https://news.med.virginia.edu/community/uva-nigeria-elevating-global-kidney-care/</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="5" t="inlineStr">
+        <is>
+          <t>Vanderbilt University Medical Center (Vanderbilt Institute for Global Health)</t>
+        </is>
+      </c>
+      <c r="B264" s="5" t="inlineStr">
+        <is>
+          <t>Aminu Kano Teaching Hospital and Bayero University Kano</t>
+        </is>
+      </c>
+      <c r="C264" s="5" t="inlineStr">
+        <is>
+          <t>Fogarty International Center Vanderbilt-Nigeria Building Research Capacity in HIV and NCDs (V-BRCH)</t>
+        </is>
+      </c>
+      <c r="D264" s="5" t="inlineStr"/>
+      <c r="E264" s="5" t="inlineStr">
+        <is>
+          <t>https://fic.nih.gov/Grants/Search/Pages/hiv-research-training-d43tw011544.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="5" t="inlineStr">
+        <is>
+          <t>Vanderbilt University Medical Center (Vanderbilt Institute for Global Health)</t>
+        </is>
+      </c>
+      <c r="B265" s="5" t="inlineStr">
+        <is>
+          <t>Aminu Kano Teaching Hospital and Bayero University Kano</t>
+        </is>
+      </c>
+      <c r="C265" s="5" t="inlineStr">
+        <is>
+          <t>Vanderbilt Institute for Global Health V-BRCH</t>
+        </is>
+      </c>
+      <c r="D265" s="5" t="inlineStr"/>
+      <c r="E265" s="5" t="inlineStr">
+        <is>
+          <t>https://www.vumc.org/global-health/v-brch</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="5" t="inlineStr">
+        <is>
+          <t>Vanderbilt University Medical Center (Vanderbilt Institute for Global Health)</t>
+        </is>
+      </c>
+      <c r="B266" s="5" t="inlineStr">
+        <is>
+          <t>Aminu Kano Teaching Hospital and Bayero University Kano</t>
+        </is>
+      </c>
+      <c r="C266" s="5" t="inlineStr">
+        <is>
+          <t>US National Institutes of Health RePORTER: 5D43TW011544-07, Vanderbilt-Nigeria Building Research Capacity in HIV and Non-communicable Diseases (V-BRCH)</t>
+        </is>
+      </c>
+      <c r="D266" s="5" t="inlineStr">
+        <is>
+          <t>FY2026 (budget start 1 January 2026)</t>
+        </is>
+      </c>
+      <c r="E266" s="5" t="inlineStr">
+        <is>
+          <t>https://reporter.nih.gov/project-details/11378551</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="5" t="inlineStr">
+        <is>
+          <t>Virginia Commonwealth University (VCU Massey Comprehensive Cancer Center)</t>
+        </is>
+      </c>
+      <c r="B267" s="5" t="inlineStr">
+        <is>
+          <t>National Hospital Abuja</t>
+        </is>
+      </c>
+      <c r="C267" s="5" t="inlineStr">
+        <is>
+          <t>Anthonia Obokoh National Hospital signs MoU with U.S. cancer center to boost research, clinical trials in Nigeria</t>
+        </is>
+      </c>
+      <c r="D267" s="5" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="E267" s="5" t="inlineStr">
+        <is>
+          <t>https://nairametrics.com/2025/07/01/national-hospital-signs-mou-with-u-s-cancer-center-to-boost-research-clinical-trials-in-nigeria/</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="5" t="inlineStr">
+        <is>
+          <t>Evercare Group (owned at its 2021 launch by the TPG-managed Evercare Health Fund)</t>
+        </is>
+      </c>
+      <c r="B268" s="5" t="inlineStr">
+        <is>
+          <t>Evercare Hospital Lekki</t>
+        </is>
+      </c>
+      <c r="C268" s="5" t="inlineStr">
+        <is>
+          <t>Esther Oluku Evercare, MedEI, Commence Advanced Cochlear Implant Surgery in Nigeria</t>
+        </is>
+      </c>
+      <c r="D268" s="5" t="inlineStr">
+        <is>
+          <t>2024-10-10</t>
+        </is>
+      </c>
+      <c r="E268" s="5" t="inlineStr">
+        <is>
+          <t>https://www.thisdaylive.com/2024/10/10/evercare-medei-commence-advanced-cochlear-implant-surgery-in-nigeria/</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="5" t="inlineStr">
+        <is>
+          <t>Evercare Group (owned at its 2021 launch by the TPG-managed Evercare Health Fund)</t>
+        </is>
+      </c>
+      <c r="B269" s="5" t="inlineStr">
+        <is>
+          <t>Evercare Hospital Lekki</t>
+        </is>
+      </c>
+      <c r="C269" s="5" t="inlineStr">
+        <is>
+          <t>TPG Evercare Group set to deliver accessible, quality healthcare in Nigeria</t>
+        </is>
+      </c>
+      <c r="D269" s="5" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="E269" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tpg.com/news-and-insights/evercare-group-set-deliver-accessible-quality-healthcare-nigeria</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="5" t="inlineStr">
+        <is>
+          <t>Evercare Group (owned at its 2021 launch by the TPG-managed Evercare Health Fund)</t>
+        </is>
+      </c>
+      <c r="B270" s="5" t="inlineStr">
+        <is>
+          <t>Evercare Hospital Lekki</t>
+        </is>
+      </c>
+      <c r="C270" s="5" t="inlineStr">
+        <is>
+          <t>TPG Evercare Group set to deliver accessible, quality healthcare in Nigeria through a new world-class multispecialty hospital</t>
+        </is>
+      </c>
+      <c r="D270" s="5" t="inlineStr">
+        <is>
+          <t>26 February 2021</t>
+        </is>
+      </c>
+      <c r="E270" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tpg.com/news-and-insights/evercare-group-set-deliver-accessible-quality-healthcare-nigeria</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="5" t="inlineStr">
+        <is>
+          <t>King's College Hospital NHS Foundation Trust</t>
+        </is>
+      </c>
+      <c r="B271" s="5" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="C271" s="5" t="inlineStr">
+        <is>
+          <t>Afreximbank King's College Hospital, London (KCH) affirmed as Clinical Partner</t>
+        </is>
+      </c>
+      <c r="D271" s="5" t="inlineStr">
+        <is>
+          <t>2021-06-03</t>
+        </is>
+      </c>
+      <c r="E271" s="5" t="inlineStr">
+        <is>
+          <t>https://www.amce.net/?p=10738</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="5" t="inlineStr">
+        <is>
+          <t>King's College Hospital NHS Foundation Trust</t>
+        </is>
+      </c>
+      <c r="B272" s="5" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="C272" s="5" t="inlineStr">
+        <is>
+          <t>Nnaemeka Onyekachi Afreximbank, BOI sign $75 million financing support for local manufacturers in Nigerian healthcare sector (reports AMCE commissioning)</t>
+        </is>
+      </c>
+      <c r="D272" s="5" t="inlineStr">
+        <is>
+          <t>2025-06-05</t>
+        </is>
+      </c>
+      <c r="E272" s="5" t="inlineStr">
+        <is>
+          <t>https://nairametrics.com/2025/06/05/afreximbank-boi-sign-75-million-financing-support-for-local-manufacturers-in-nigerian-healthcare-sector/</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="5" t="inlineStr">
+        <is>
+          <t>King's College Hospital NHS Foundation Trust</t>
+        </is>
+      </c>
+      <c r="B273" s="5" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="C273" s="5" t="inlineStr">
+        <is>
+          <t>Brand Spur African Medical Centre Of Excellence Opens In Abuja As Nigeria Targets $2.2bn Health Sector Overhaul</t>
+        </is>
+      </c>
+      <c r="D273" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="E273" s="5" t="inlineStr">
+        <is>
+          <t>https://brandspurng.com/2026/09/19/african-medical-centre-of-excellence-opens-in-abuja-as-nigeria-targets-2-2bn-health-sector-overhaul/</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="5" t="inlineStr">
+        <is>
+          <t>King's College London</t>
+        </is>
+      </c>
+      <c r="B274" s="5" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="C274" s="5" t="inlineStr">
+        <is>
+          <t>King's College London New partnership to deliver medical excellence in Nigeria</t>
+        </is>
+      </c>
+      <c r="D274" s="5" t="inlineStr">
+        <is>
+          <t>2023-11-28</t>
+        </is>
+      </c>
+      <c r="E274" s="5" t="inlineStr">
+        <is>
+          <t>https://www.kcl.ac.uk/news/new-partnership-to-deliver-medical-excellence-in-nigeria</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="5" t="inlineStr">
+        <is>
+          <t>King's College London</t>
+        </is>
+      </c>
+      <c r="B275" s="5" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="C275" s="5" t="inlineStr">
+        <is>
+          <t>Nnaemeka Onyekachi Afreximbank, BOI sign $75 million financing support for local manufacturers in Nigerian healthcare sector (reports KCL terms of agreement)</t>
+        </is>
+      </c>
+      <c r="D275" s="5" t="inlineStr">
+        <is>
+          <t>2025-06-05</t>
+        </is>
+      </c>
+      <c r="E275" s="5" t="inlineStr">
+        <is>
+          <t>https://nairametrics.com/2025/06/05/afreximbank-boi-sign-75-million-financing-support-for-local-manufacturers-in-nigerian-healthcare-sector/</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="5" t="inlineStr">
+        <is>
+          <t>Liverpool School of Tropical Medicine</t>
+        </is>
+      </c>
+      <c r="B276" s="5" t="inlineStr">
+        <is>
+          <t>National Postgraduate Medical College of Nigeria (with Wellbeing Foundation Africa)</t>
+        </is>
+      </c>
+      <c r="C276" s="5" t="inlineStr">
+        <is>
+          <t>Liverpool School of Tropical Medicine LSTM and Wellbeing Foundation Africa launch Advanced Training for Resident Doctors in Nigeria</t>
+        </is>
+      </c>
+      <c r="D276" s="5" t="inlineStr">
+        <is>
+          <t>2024-05</t>
+        </is>
+      </c>
+      <c r="E276" s="5" t="inlineStr">
+        <is>
+          <t>https://lstmed.ac.uk/news/liverpool-school-of-tropical-medicine-and-wellbeing-foundation-africa-launch-advanced-training-for-resident-doctors-in-nigeria/</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="5" t="inlineStr">
+        <is>
+          <t>Liverpool School of Tropical Medicine</t>
+        </is>
+      </c>
+      <c r="B277" s="5" t="inlineStr">
+        <is>
+          <t>National Postgraduate Medical College of Nigeria (with Wellbeing Foundation Africa)</t>
+        </is>
+      </c>
+      <c r="C277" s="5" t="inlineStr">
+        <is>
+          <t>Wellbeing Foundation Africa AOSS Training Expands to Port Harcourt and Gombe</t>
+        </is>
+      </c>
+      <c r="D277" s="5" t="inlineStr">
+        <is>
+          <t>2025-05-22</t>
+        </is>
+      </c>
+      <c r="E277" s="5" t="inlineStr">
+        <is>
+          <t>https://wbfafrica.org/aoss-training-expands-to-port-harcourt-and-gombe-ghwp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="5" t="inlineStr">
+        <is>
+          <t>Liverpool School of Tropical Medicine</t>
+        </is>
+      </c>
+      <c r="B278" s="5" t="inlineStr">
+        <is>
+          <t>National Postgraduate Medical College of Nigeria (with Wellbeing Foundation Africa)</t>
+        </is>
+      </c>
+      <c r="C278" s="5" t="inlineStr">
+        <is>
+          <t>Wellbeing Foundation Africa Liverpool School of Tropical Medicine, Wellbeing Foundation Africa, and Global Health Workforce Partnership</t>
+        </is>
+      </c>
+      <c r="D278" s="5" t="inlineStr">
+        <is>
+          <t>2025-02-12</t>
+        </is>
+      </c>
+      <c r="E278" s="5" t="inlineStr">
+        <is>
+          <t>https://wbfafrica.org/liverpool-school-of-tropical-medicine-wellbeing-foundation-africa-and-global-health-workforce-partnership/</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="5" t="inlineStr">
+        <is>
+          <t>Manipal Hospitals</t>
+        </is>
+      </c>
+      <c r="B279" s="5" t="inlineStr">
+        <is>
+          <t>Afe Babalola University Multi-System Hospital</t>
+        </is>
+      </c>
+      <c r="C279" s="5" t="inlineStr">
+        <is>
+          <t>Folasade Akpan ABUAD multi-system hospital records 50 successful kidney transplants</t>
+        </is>
+      </c>
+      <c r="D279" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="E279" s="5" t="inlineStr">
+        <is>
+          <t>https://nannews.ng/abuad-multi-system-hospital-records-50-successful-kidney-transplants/</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="5" t="inlineStr">
+        <is>
+          <t>The Christie NHS Foundation Trust</t>
+        </is>
+      </c>
+      <c r="B280" s="5" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="C280" s="5" t="inlineStr">
+        <is>
+          <t>The Christie NHS Foundation Trust The Christie International hosts African Medical Centre of Excellence visit</t>
+        </is>
+      </c>
+      <c r="D280" s="5" t="inlineStr">
+        <is>
+          <t>2024-10-25</t>
+        </is>
+      </c>
+      <c r="E280" s="5" t="inlineStr">
+        <is>
+          <t>https://christie.nhs.uk/about-us/news-at-the-christie/latest-news-stories/the-christie-international-hosts-african-medical-centre-of-excellence-visit</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="5" t="inlineStr">
+        <is>
+          <t>The Christie NHS Foundation Trust</t>
+        </is>
+      </c>
+      <c r="B281" s="5" t="inlineStr">
+        <is>
+          <t>African Medical Centre of Excellence (AMCE), developed by Afreximbank</t>
+        </is>
+      </c>
+      <c r="C281" s="5" t="inlineStr">
+        <is>
+          <t>The Christie NHS Foundation Trust The Christie supporting a new African Medical Centre of Excellence project</t>
+        </is>
+      </c>
+      <c r="D281" s="5" t="inlineStr"/>
+      <c r="E281" s="5" t="inlineStr">
+        <is>
+          <t>https://christie.nhs.uk/about-us/about-the-christie/the-christie-international/partnerships-experience/the-christie-supporting-a-new-african-medical-centre-of-excellence-project</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="5" t="inlineStr">
+        <is>
+          <t>The Royal Marsden NHS Foundation Trust</t>
+        </is>
+      </c>
+      <c r="B282" s="5" t="inlineStr">
+        <is>
+          <t>Marcelle Ruth Cancer Centre &amp; Specialist Hospital</t>
+        </is>
+      </c>
+      <c r="C282" s="5" t="inlineStr">
+        <is>
+          <t>BusinessDay Marcelle Ruth Cancer Centre partners UK's Royal Marsden to improve healthcare delivery in West Africa</t>
+        </is>
+      </c>
+      <c r="D282" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E282" s="5" t="inlineStr">
+        <is>
+          <t>https://businessday.ng/news/article/marcelle-ruth-cancer-centre-royal-marsden-partner-to-elevate-west-africas-oncology-care/</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="5" t="inlineStr">
+        <is>
+          <t>University of Birmingham</t>
+        </is>
+      </c>
+      <c r="B283" s="5" t="inlineStr">
+        <is>
+          <t>University of Lagos (with Lagos University Teaching Hospital)</t>
+        </is>
+      </c>
+      <c r="C283" s="5" t="inlineStr">
+        <is>
+          <t>Adesina Wahab UNILAG, University of Birmingham sign MoU on Transnational Education Engagement</t>
+        </is>
+      </c>
+      <c r="D283" s="5" t="inlineStr">
+        <is>
+          <t>29 January 2026</t>
+        </is>
+      </c>
+      <c r="E283" s="5" t="inlineStr">
+        <is>
+          <t>https://www.vanguardngr.com/2026/01/unilag-university-of-birmingham-sign-mou-on-transnational-education-engagement/</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="5" t="inlineStr">
+        <is>
+          <t>University of Glasgow</t>
+        </is>
+      </c>
+      <c r="B284" s="5" t="inlineStr">
+        <is>
+          <t>Ahmadu Bello University</t>
+        </is>
+      </c>
+      <c r="C284" s="5" t="inlineStr">
+        <is>
+          <t>University of Glasgow School of Infection &amp; Immunity's Professor Harry de-Koning helps facilitate UofG-ABU MoU</t>
+        </is>
+      </c>
+      <c r="D284" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="E284" s="5" t="inlineStr">
+        <is>
+          <t>https://www.gla.ac.uk/schools/infectionimmunity/newsevents/headline_1265451_en.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="5" t="inlineStr">
+        <is>
+          <t>University of Maryland School of Medicine</t>
+        </is>
+      </c>
+      <c r="B285" s="5" t="inlineStr">
+        <is>
+          <t>Lagos University Teaching Hospital (LUTH)</t>
+        </is>
+      </c>
+      <c r="C285" s="5" t="inlineStr">
+        <is>
+          <t>Lagos University Teaching Hospital Maryland LUTH</t>
+        </is>
+      </c>
+      <c r="D285" s="5" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="E285" s="5" t="inlineStr">
+        <is>
+          <t>https://luth.gov.ng/news/maryland-luth</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="5" t="inlineStr">
+        <is>
+          <t>University of Maryland School of Medicine</t>
+        </is>
+      </c>
+      <c r="B286" s="5" t="inlineStr">
+        <is>
+          <t>Lagos University Teaching Hospital (LUTH)</t>
+        </is>
+      </c>
+      <c r="C286" s="5" t="inlineStr">
+        <is>
+          <t>Lagos University Teaching Hospital University of Maryland School of Medicine Collaborates with Lagos University Teaching Hospital on Non-Communicable Diseases</t>
+        </is>
+      </c>
+      <c r="D286" s="5" t="inlineStr">
+        <is>
+          <t>August 2024</t>
+        </is>
+      </c>
+      <c r="E286" s="5" t="inlineStr">
+        <is>
+          <t>https://luth.gov.ng/news/maryland-luth</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="5" t="inlineStr">
+        <is>
+          <t>University of Maryland School of Medicine</t>
+        </is>
+      </c>
+      <c r="B287" s="5" t="inlineStr">
+        <is>
+          <t>Lagos University Teaching Hospital (LUTH)</t>
+        </is>
+      </c>
+      <c r="C287" s="5" t="inlineStr">
+        <is>
+          <t>IHV Nigeria University of Maryland Dean of Medicine Visits LUTH</t>
+        </is>
+      </c>
+      <c r="D287" s="5" t="inlineStr">
+        <is>
+          <t>August 2024</t>
+        </is>
+      </c>
+      <c r="E287" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ihvnigeria.org/university-of-maryland-dean-of-medicine-visits-luth/</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="5" t="inlineStr">
+        <is>
+          <t>University of Virginia Health System</t>
+        </is>
+      </c>
+      <c r="B288" s="5" t="inlineStr">
+        <is>
+          <t>Federal Medical Centre Owo</t>
+        </is>
+      </c>
+      <c r="C288" s="5" t="inlineStr">
+        <is>
+          <t>UVA School of Medicine UVA Department of Nephrology Partners With Nigerian Federal Medical Center</t>
+        </is>
+      </c>
+      <c r="D288" s="5" t="inlineStr">
+        <is>
+          <t>2023-01</t>
+        </is>
+      </c>
+      <c r="E288" s="5" t="inlineStr">
+        <is>
+          <t>https://news.med.virginia.edu/community/uva-department-of-nephrology-partners-with-nigerian-federal-medical-center/</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="5" t="inlineStr">
+        <is>
+          <t>Yale School of Medicine (Department of Psychiatry)</t>
+        </is>
+      </c>
+      <c r="B289" s="5" t="inlineStr">
+        <is>
+          <t>Imo State University Teaching Hospital</t>
+        </is>
+      </c>
+      <c r="C289" s="5" t="inlineStr">
+        <is>
+          <t>Nigeria Health Watch Making Happiness Local: How a Project is Improving Access to Mental Healthcare in Imo State</t>
+        </is>
+      </c>
+      <c r="D289" s="5" t="inlineStr">
+        <is>
+          <t>2023-09-06</t>
+        </is>
+      </c>
+      <c r="E289" s="5" t="inlineStr">
+        <is>
+          <t>https://nigeriahealthwatch.com/articles/torchlight/making-happiness-local-how-a-project-is-improving-access-to-mental-healthcare-in-imo-state/</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="5" t="inlineStr">
+        <is>
+          <t>Yale School of Medicine (Department of Psychiatry)</t>
+        </is>
+      </c>
+      <c r="B290" s="5" t="inlineStr">
+        <is>
+          <t>Imo State University Teaching Hospital</t>
+        </is>
+      </c>
+      <c r="C290" s="5" t="inlineStr">
+        <is>
+          <t>Yale School of Medicine The HAPPINESS Project</t>
+        </is>
+      </c>
+      <c r="D290" s="5" t="inlineStr"/>
+      <c r="E290" s="5" t="inlineStr">
+        <is>
+          <t>https://medicine.yale.edu/psychiatry/education/programs-and-initiatives/happiness</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="5" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals</t>
+        </is>
+      </c>
+      <c r="B291" s="5" t="inlineStr">
+        <is>
+          <t>Duchess International Hospital (Reddington Hospital Group)</t>
+        </is>
+      </c>
+      <c r="C291" s="5" t="inlineStr">
+        <is>
+          <t>ThisDay Duchess International Hospital Has Put Lagos on World Healthcare Map, Says US Consul General</t>
+        </is>
+      </c>
+      <c r="D291" s="5" t="inlineStr">
+        <is>
+          <t>11 November 2021</t>
+        </is>
+      </c>
+      <c r="E291" s="5" t="inlineStr">
+        <is>
+          <t>https://www.thisdaylive.com/index.php/2021/11/11/duchess-international-hospital-has-put-lagos-on-world-healthcare-map-says-us-consul-general/</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="5" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals</t>
+        </is>
+      </c>
+      <c r="B292" s="5" t="inlineStr">
+        <is>
+          <t>Duchess International Hospital (Reddington Hospital Group)</t>
+        </is>
+      </c>
+      <c r="C292" s="5" t="inlineStr">
+        <is>
+          <t>Appolonia Adeyemi Duchess International Hospital debuts in Lagos, builds capacity</t>
+        </is>
+      </c>
+      <c r="D292" s="5" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="E292" s="5" t="inlineStr">
+        <is>
+          <t>https://newtelegraphng.com/?p=192437</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="5" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals</t>
+        </is>
+      </c>
+      <c r="B293" s="5" t="inlineStr">
+        <is>
+          <t>State House Clinic</t>
+        </is>
+      </c>
+      <c r="C293" s="5" t="inlineStr">
+        <is>
+          <t>Blueprint State House Clinic, Indian hospital collaborate to assist heart, kidney, cancer patients</t>
+        </is>
+      </c>
+      <c r="D293" s="5" t="inlineStr">
+        <is>
+          <t>2022-07-29</t>
+        </is>
+      </c>
+      <c r="E293" s="5" t="inlineStr">
+        <is>
+          <t>https://blueprint.ng/state-house-clinic-indian-hospital-collaborate-to-assist-heart-kidney-cancer-patients/</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="5" t="inlineStr">
+        <is>
+          <t>Apollo Hospitals</t>
+        </is>
+      </c>
+      <c r="B294" s="5" t="inlineStr">
+        <is>
+          <t>State House Clinic</t>
+        </is>
+      </c>
+      <c r="C294" s="5" t="inlineStr">
+        <is>
+          <t>ThisDay Medical Tourism: Indian Hospital to Train Nigerian Doctors on Cancer Treatment</t>
+        </is>
+      </c>
+      <c r="D294" s="5" t="inlineStr">
+        <is>
+          <t>2024-03-05</t>
+        </is>
+      </c>
+      <c r="E294" s="5" t="inlineStr">
+        <is>
+          <t>https://www.thisdaylive.com/2024/03/05/medical-tourism-indian-hospital-to-train-nigerian-doctors-on-cancer-treatment/</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="5" t="inlineStr">
+        <is>
+          <t>Memorial Hospitals Group</t>
+        </is>
+      </c>
+      <c r="B295" s="5" t="inlineStr">
+        <is>
+          <t>Kasi Healthcare</t>
+        </is>
+      </c>
+      <c r="C295" s="5" t="inlineStr">
+        <is>
+          <t>Temitayo Ayetoto-Oladehinde Nigeria partners Turkey to tap $8.5trn healthcare market</t>
+        </is>
+      </c>
+      <c r="D295" s="5" t="inlineStr">
+        <is>
+          <t>2024-09-27</t>
+        </is>
+      </c>
+      <c r="E295" s="5" t="inlineStr">
+        <is>
+          <t>https://businessday.ng/news/article/nigeria-partners-turkey-to-tap-8-5trn-healthcare-market/</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="5" t="inlineStr">
+        <is>
+          <t>Peking University People's Hospital (named variously in press as People's University Hospital, Beijing)</t>
+        </is>
+      </c>
+      <c r="B296" s="5" t="inlineStr">
+        <is>
+          <t>University of Abuja Teaching Hospital</t>
+        </is>
+      </c>
+      <c r="C296" s="5" t="inlineStr">
+        <is>
+          <t>Within Nigeria Nigeria signs letter of intent with China to improve health sector</t>
+        </is>
+      </c>
+      <c r="D296" s="5" t="inlineStr">
+        <is>
+          <t>2022-08-20</t>
+        </is>
+      </c>
+      <c r="E296" s="5" t="inlineStr">
+        <is>
+          <t>https://www.withinnigeria.com/broadnews/2022/08/20/nigeria-signs-letter-of-intent-with-china-to-improve-health-sector/</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="5" t="inlineStr">
+        <is>
+          <t>Peking University People's Hospital (named variously in press as People's University Hospital, Beijing)</t>
+        </is>
+      </c>
+      <c r="B297" s="5" t="inlineStr">
+        <is>
+          <t>University of Abuja Teaching Hospital</t>
+        </is>
+      </c>
+      <c r="C297" s="5" t="inlineStr">
+        <is>
+          <t>University of Abuja Teaching Hospital Nigeria, China signs letter of intent to improve health sector</t>
+        </is>
+      </c>
+      <c r="D297" s="5" t="inlineStr">
+        <is>
+          <t>2022-08</t>
+        </is>
+      </c>
+      <c r="E297" s="5" t="inlineStr">
+        <is>
+          <t>https://uathospital.ng/nigeria-china-signs-letter-of-intent-to-improve-health-sector/</t>
         </is>
       </c>
     </row>
@@ -14703,6 +17758,59 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E242" r:id="rId241"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E243" r:id="rId242"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E244" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E245" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E246" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E247" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E248" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E249" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E250" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E251" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E252" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E253" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E254" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E255" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E256" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E257" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E258" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E259" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E260" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E261" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E262" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E263" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E264" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E265" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E266" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E267" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E268" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E269" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E270" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E271" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E272" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E273" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E274" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E275" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E276" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E277" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E278" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E279" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E280" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E281" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E282" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E283" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E284" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E285" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E286" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E287" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E288" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E289" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E290" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E291" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E292" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E293" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E294" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E295" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E296" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E297" r:id="rId296"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Spain: verified profile research, partnerships tracker and map
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ChEN58PbdXFZmwUoBZYBRb
</commit_message>
<xml_diff>
--- a/output/Partnerships_Tracker.xlsx
+++ b/output/Partnerships_Tracker.xlsx
@@ -231,8 +231,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tracker" displayName="Tracker" ref="A1:L165" headerRowCount="1">
-  <autoFilter ref="A1:L165"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tracker" displayName="Tracker" ref="A1:L188" headerRowCount="1">
+  <autoFilter ref="A1:L188"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Status"/>
     <tableColumn id="2" name="Country"/>
@@ -558,7 +558,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Scope: partnerships that are active, or ended or last active within the past five years. Last checked 2026-10-21.</t>
+          <t>Scope: partnerships that are active, or ended or last active within the past five years. Last checked 2026-10-30.</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Tracker!$A$2:$A$165,A5)</f>
+        <f>COUNTIF(Tracker!$A$2:$A$188,A5)</f>
         <v/>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF(Tracker!$A$2:$A$165,A6)</f>
+        <f>COUNTIF(Tracker!$A$2:$A$188,A6)</f>
         <v/>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Tracker!$A$2:$A$165,A7)</f>
+        <f>COUNTIF(Tracker!$A$2:$A$188,A7)</f>
         <v/>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -670,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L165"/>
+  <dimension ref="A1:L188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10222,6 +10222,1336 @@
       <c r="L165" s="14" t="inlineStr">
         <is>
           <t>Within Nigeria, 2022-08-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B166" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C166" s="13" t="inlineStr">
+        <is>
+          <t>Cleveland Clinic</t>
+        </is>
+      </c>
+      <c r="D166" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E166" s="12" t="inlineStr">
+        <is>
+          <t>Vall d'Hebron University Hospital (Advanced Clinical Simulation Centre)</t>
+        </is>
+      </c>
+      <c r="F166" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G166" s="12" t="inlineStr">
+        <is>
+          <t>Vall d'Hebron and Cleveland Clinic signed an agreement in February 2025 for educator development and courses in clinical simulation, shared resources and joint research on health education. The collaboration was renewed in 2025 and Vall d'Hebron instructors teach Cleveland Clinic's SEVA ventilation course.</t>
+        </is>
+      </c>
+      <c r="H166" s="12" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="I166" s="12" t="inlineStr"/>
+      <c r="J166" s="12" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="K166" s="12" t="inlineStr">
+        <is>
+          <t>Vall d'Hebron news item dated 07/02/2025 announces the agreement; Vall d'Hebron's 2025 report says the Advanced Clinical Simulation Centre signed 20 agreements in 2025, including the renewal of its collaboration with Cleveland Clinic.</t>
+        </is>
+      </c>
+      <c r="L166" s="14" t="inlineStr">
+        <is>
+          <t>Vall d'Hebron, 2025-02-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B167" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C167" s="13" t="inlineStr">
+        <is>
+          <t>George Washington University (School of Medicine and Health Sciences)</t>
+        </is>
+      </c>
+      <c r="D167" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E167" s="12" t="inlineStr">
+        <is>
+          <t>Universidad Autonoma de Madrid (Faculty of Medicine)</t>
+        </is>
+      </c>
+      <c r="F167" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G167" s="12" t="inlineStr">
+        <is>
+          <t>George Washington University's medical school and the Universidad Autonoma de Madrid run a reciprocal clinical rotation program under a framework agreement. Each year the Madrid faculty funds three of its students to spend a month on clinical rotations at George Washington.</t>
+        </is>
+      </c>
+      <c r="H167" s="12" t="inlineStr">
+        <is>
+          <t>2018-06</t>
+        </is>
+      </c>
+      <c r="I167" s="12" t="inlineStr"/>
+      <c r="J167" s="12" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="K167" s="12" t="inlineStr">
+        <is>
+          <t>UAM's Faculty of Medicine published its 2026-2027 call for three grants for one month clinical rotations at George Washington University in July or August 2027. Applications ran from 13 to 18 October 2026 and the provisional admitted list is out. The specific agreement for the International Clinical Rotation Program between GW's SMHS and UAM was approved by UAM's governing council on 15 June 2018.</t>
+        </is>
+      </c>
+      <c r="L167" s="14" t="inlineStr">
+        <is>
+          <t>Universidad Autonoma de Madrid, 2026-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B168" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C168" s="13" t="inlineStr">
+        <is>
+          <t>Harvard Medical School (Harvard University)</t>
+        </is>
+      </c>
+      <c r="D168" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E168" s="12" t="inlineStr">
+        <is>
+          <t>Universidad Complutense de Madrid (Faculty of Medicine; Hospital Clinico San Carlos, Hospital 12 de Octubre, Hospital Gregorio Maranon)</t>
+        </is>
+      </c>
+      <c r="F168" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G168" s="12" t="inlineStr">
+        <is>
+          <t>Under the long standing agreement between Complutense University and Harvard, Harvard medical students take clinical electives at Complutense's teaching hospitals in Madrid. Complutense fifth year medical students spend a month in the Harvard Medical School Exchange Clerkship Program on scholarships from the Fundacion Fernandez-Cruz.</t>
+        </is>
+      </c>
+      <c r="H168" s="12" t="inlineStr">
+        <is>
+          <t>1991</t>
+        </is>
+      </c>
+      <c r="I168" s="12" t="inlineStr"/>
+      <c r="J168" s="12" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="K168" s="12" t="inlineStr">
+        <is>
+          <t>Complutense's Faculty of Medicine posted an elective description for the 2025-26 HMS to Complutense clinical rotation, created 28 October 2025, covering Hospital Clinico San Carlos, Hospital 12 de Octubre and Gregorio Maranon. Complutense reported on 30 January 2020 that seven medical students would spend a month at Harvard Medical School under this agreement, which is nearly three decades old (so dating from about 1991; the start year is approximate). The Real Colegio Complutense at Harvard has been affiliated with Harvard since 1990. The 2022-23 scholarship call offered 7 to 9 places in the HMS Exchange Clerkship Program.</t>
+        </is>
+      </c>
+      <c r="L168" s="14" t="inlineStr">
+        <is>
+          <t>Universidad Complutense de Madrid, 2025-10-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B169" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C169" s="13" t="inlineStr">
+        <is>
+          <t>Johns Hopkins University (Bloomberg School of Public Health)</t>
+        </is>
+      </c>
+      <c r="D169" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E169" s="12" t="inlineStr">
+        <is>
+          <t>Universitat Pompeu Fabra (JHU-UPF Public Policy Center), with the Agencia de Salut Publica de Barcelona</t>
+        </is>
+      </c>
+      <c r="F169" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G169" s="12" t="inlineStr">
+        <is>
+          <t>Johns Hopkins and Universitat Pompeu Fabra have run a joint public policy centre in Barcelona since 2013, with a health and well-being research line. With the Barcelona Public Health Agency they have also run, since 2004, the yearly Hopkins Fall Institute in Health Policy and Management, which Bloomberg School faculty teach.</t>
+        </is>
+      </c>
+      <c r="H169" s="12" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="I169" s="12" t="inlineStr"/>
+      <c r="J169" s="12" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="K169" s="12" t="inlineStr">
+        <is>
+          <t>UPF's repository holds the JHU-UPF Public Policy Center Annual Report 2024 to 2025, deposited in November 2025, which lists health and well-being among five research areas and mentions joint programs including the Fall Institute in Health Policy and Management. The Fall Institute began in 2004 (its 20th edition was in 2023), sponsored by the Barcelona Public Health Agency and the Bloomberg School in collaboration with UPF. A Bloomberg School page lists the November 2025 edition at UPF Barcelona School of Management. The Bloomberg School and UPF pages could not be fetched (HTTP 403), so the details come from search snippets.</t>
+        </is>
+      </c>
+      <c r="L169" s="14" t="inlineStr">
+        <is>
+          <t>Universitat Pompeu Fabra repository, 2025-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B170" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C170" s="13" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center</t>
+        </is>
+      </c>
+      <c r="D170" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E170" s="12" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center Madrid (operated by Grupo Hospiten)</t>
+        </is>
+      </c>
+      <c r="F170" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G170" s="12" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center Madrid opened in 2000 as the first international affiliate of MD Anderson in Houston and still carries its name. Grupo Hospiten owns and runs the hospital, and Hospiten says Houston's protocols and standards are applied to care in Madrid.</t>
+        </is>
+      </c>
+      <c r="H170" s="12" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="I170" s="12" t="inlineStr"/>
+      <c r="J170" s="12" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="K170" s="12" t="inlineStr">
+        <is>
+          <t>A Hospiten page of 18 September 2026 on the Newsweek and Statista ranking says MD Anderson Cancer Center Madrid has the backing of MD Anderson Cancer Center in Houston and is its only affiliate outside the United States. Forbes Spain ranked it among the three best oncology hospitals in Spain in December 2025. Hospiten's release of 10 January 2013 reported buying a further 39.98 percent of the shares; Hospiten later reported holding 99.97 percent, with MD Anderson Houston keeping 0.03 percent. In an MD Anderson oral history, former president John Mendelsohn describes MD Anderson Espana in Madrid as one of the sister institutions he created. Madrid does not appear on recent MD Anderson Sister Institution Network lists, so the tie is a branded affiliation, not a GAP sister institution.</t>
+        </is>
+      </c>
+      <c r="L170" s="14" t="inlineStr">
+        <is>
+          <t>Hospiten, 2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B171" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C171" s="13" t="inlineStr">
+        <is>
+          <t>Mount Sinai Health System (Icahn School of Medicine, Mount Sinai Fuster Heart Hospital)</t>
+        </is>
+      </c>
+      <c r="D171" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E171" s="12" t="inlineStr">
+        <is>
+          <t>Centro Nacional de Investigaciones Cardiovasculares Carlos III (CNIC)</t>
+        </is>
+      </c>
+      <c r="F171" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G171" s="12" t="inlineStr">
+        <is>
+          <t>Mount Sinai and Spain's national cardiovascular research centre CNIC have a long running research partnership with researcher exchanges, shared cardiac imaging work and jointly led clinical trials. Valentín Fuster is general director of CNIC and president of Mount Sinai Fuster Heart Hospital.</t>
+        </is>
+      </c>
+      <c r="H171" s="12" t="inlineStr"/>
+      <c r="I171" s="12" t="inlineStr"/>
+      <c r="J171" s="12" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="K171" s="12" t="inlineStr">
+        <is>
+          <t>A Mount Sinai release of 30 August 2025 presents the REBOOT trial and quotes Fuster that it joins earlier landmark trials led by CNIC and Mount Sinai, SECURE and DapaTAVI. A Mount Sinai release of 30 September 2024 reports BioImage results from the Mount Sinai and CNIC collaboration. A 2015 CNIC article describes the partnership program set up when Fuster took charge of CNIC while leading Mount Sinai's heart institute, starting with shared MRI imaging. No signing date for the original agreement was found.</t>
+        </is>
+      </c>
+      <c r="L171" s="14" t="inlineStr">
+        <is>
+          <t>EurekAlert, 2025-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B172" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C172" s="13" t="inlineStr">
+        <is>
+          <t>Penn State College of Medicine and Penn State Health (Beat Childhood Cancer Research Consortium)</t>
+        </is>
+      </c>
+      <c r="D172" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E172" s="12" t="inlineStr">
+        <is>
+          <t>Hospital Sant Joan de Déu Barcelona (Pediatric Cancer Center Barcelona)</t>
+        </is>
+      </c>
+      <c r="F172" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G172" s="12" t="inlineStr">
+        <is>
+          <t>SJD's Pediatric Cancer Center Barcelona joined the Beat Childhood Cancer Research Consortium, headquartered at Penn State College of Medicine, in November 2025, the first member outside North America. SJD acts as European sponsor for consortium trials, starting with BCC018 in high risk neuroblastoma.</t>
+        </is>
+      </c>
+      <c r="H172" s="12" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="I172" s="12" t="inlineStr"/>
+      <c r="J172" s="12" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="K172" s="12" t="inlineStr">
+        <is>
+          <t>SJD announcement and Penn State Health News of November 2025 (consortium of more than 55 children's hospitals and research institutions; borderline as a consortium, like the Cancer Core Europe record). SJD news item dated 24 November 2025.</t>
+        </is>
+      </c>
+      <c r="L172" s="14" t="inlineStr">
+        <is>
+          <t>SJD Barcelona Children's Hospital, 2025-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B173" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C173" s="13" t="inlineStr">
+        <is>
+          <t>University of Illinois Chicago (College of Applied Health Sciences)</t>
+        </is>
+      </c>
+      <c r="D173" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E173" s="12" t="inlineStr">
+        <is>
+          <t>TecnoCampus School of Health Sciences (Universitat Pompeu Fabra)</t>
+        </is>
+      </c>
+      <c r="F173" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G173" s="12" t="inlineStr">
+        <is>
+          <t>UIC's College of Applied Health Sciences and the TecnoCampus School of Health Sciences signed a letter of intent in October 2025 to set up an educational collaboration. It covers faculty and student exchanges, visiting professors and joint research in kinesiology, nutrition and rehabilitation sciences.</t>
+        </is>
+      </c>
+      <c r="H173" s="12" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="I173" s="12" t="inlineStr"/>
+      <c r="J173" s="12" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="K173" s="12" t="inlineStr">
+        <is>
+          <t>A UIC College of Applied Health Sciences news story of 20 October 2025 reports that Dean Carlos Crespo and TecnoCampus general director Josep Lluis Checa signed the letter of intent on 6 October 2025 in Barcelona. UIC is the University of Illinois's academic health enterprise and includes a medical school, but this tie runs through the allied health college.</t>
+        </is>
+      </c>
+      <c r="L173" s="14" t="inlineStr">
+        <is>
+          <t>University of Illinois Chicago, College of Applied Health Sciences, 2025-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B174" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C174" s="13" t="inlineStr">
+        <is>
+          <t>University of Kansas Medical Center</t>
+        </is>
+      </c>
+      <c r="D174" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E174" s="12" t="inlineStr">
+        <is>
+          <t>Universitat Internacional de Catalunya (UIC Barcelona) Faculty of Medicine and Health Sciences</t>
+        </is>
+      </c>
+      <c r="F174" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G174" s="12" t="inlineStr">
+        <is>
+          <t>The University of Kansas Medical Center is one of UIC Barcelona's North American exchange partners for medicine. KUMC sends medical, nursing and health professions students to Barcelona for clinical rotations.</t>
+        </is>
+      </c>
+      <c r="H174" s="12" t="inlineStr"/>
+      <c r="I174" s="12" t="inlineStr"/>
+      <c r="J174" s="12" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="K174" s="12" t="inlineStr">
+        <is>
+          <t>UIC Barcelona's medicine brochures in English and Spanish, created 16 February 2026, list the University of Kansas Medical Center among three North American exchange agreements. The January 2024 edition lists it as well. KUMC's Office of International Programs lists UIC Barcelona as a Spain rotation site for M1 and M4 medical students, nursing and health professions students, two students per cycle. The same page also lists M4 rotations at the University of Navarra in Pamplona and Madrid and a summer program at the Universidad de Santiago de Compostela.</t>
+        </is>
+      </c>
+      <c r="L174" s="14" t="inlineStr">
+        <is>
+          <t>UIC Barcelona, 2026-02-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B175" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C175" s="13" t="inlineStr">
+        <is>
+          <t>ABC Medical Center (Centro Médico ABC)</t>
+        </is>
+      </c>
+      <c r="D175" s="12" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E175" s="12" t="inlineStr">
+        <is>
+          <t>Hospital Sant Joan de Déu Barcelona (SJD Barcelona Children's Hospital)</t>
+        </is>
+      </c>
+      <c r="F175" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G175" s="12" t="inlineStr">
+        <is>
+          <t>SJD Barcelona Children's Hospital and ABC Medical Center in Mexico City signed a collaboration agreement in August 2025 for joint training of health professionals, pediatric oncology research and second opinions on highly complex pediatric cases.</t>
+        </is>
+      </c>
+      <c r="H175" s="12" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="I175" s="12" t="inlineStr"/>
+      <c r="J175" s="12" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="K175" s="12" t="inlineStr">
+        <is>
+          <t>SJD announced the agreement on 29 August 2025.</t>
+        </is>
+      </c>
+      <c r="L175" s="14" t="inlineStr">
+        <is>
+          <t>SJD Barcelona Children's Hospital, 2025-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B176" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C176" s="13" t="inlineStr">
+        <is>
+          <t>Aier Eye Hospital Group</t>
+        </is>
+      </c>
+      <c r="D176" s="12" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E176" s="12" t="inlineStr">
+        <is>
+          <t>Clínica Baviera</t>
+        </is>
+      </c>
+      <c r="F176" s="12" t="inlineStr">
+        <is>
+          <t>Ownership or management</t>
+        </is>
+      </c>
+      <c r="G176" s="12" t="inlineStr">
+        <is>
+          <t>Chinese eye hospital group Aier took control of Clínica Baviera, the Madrid listed ophthalmology clinic chain, through a 2017 takeover bid. Aier remains the majority shareholder with about 73 to 75 percent after selling part of its stake in April 2025 (reported figures vary).</t>
+        </is>
+      </c>
+      <c r="H176" s="12" t="inlineStr">
+        <is>
+          <t>2017-08</t>
+        </is>
+      </c>
+      <c r="I176" s="12" t="inlineStr"/>
+      <c r="J176" s="12" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="K176" s="12" t="inlineStr">
+        <is>
+          <t>Alimarket reported in 2017 that Aier Eye Hospital took control of Clínica Baviera with 86.8% after its bid. Alantra reported in April 2025 that Aier, the majority shareholder, and the founders' vehicle placed 8% of the shares, leaving Aier with about 74.8%. Later reports through Clínica Baviera's first-half 2026 results of 29 July 2026 give Aier between 73 and 75 percent.</t>
+        </is>
+      </c>
+      <c r="L176" s="14" t="inlineStr">
+        <is>
+          <t>Alimarket, 2017</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B177" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C177" s="13" t="inlineStr">
+        <is>
+          <t>Bupa</t>
+        </is>
+      </c>
+      <c r="D177" s="12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E177" s="12" t="inlineStr">
+        <is>
+          <t>Sanitas (Sanitas hospitals)</t>
+        </is>
+      </c>
+      <c r="F177" s="12" t="inlineStr">
+        <is>
+          <t>Ownership or management</t>
+        </is>
+      </c>
+      <c r="G177" s="12" t="inlineStr">
+        <is>
+          <t>British healthcare group Bupa owns Sanitas, which runs private hospitals in Spain including Hospital Universitario Sanitas La Moraleja, La Zarzuela, CIMA in Barcelona and the new Blua Sanitas Valdebebas, alongside its health insurance and aged care businesses. A public private partnership hospital contract held by Sanitas ended in 2024.</t>
+        </is>
+      </c>
+      <c r="H177" s="12" t="inlineStr">
+        <is>
+          <t>1989</t>
+        </is>
+      </c>
+      <c r="I177" s="12" t="inlineStr"/>
+      <c r="J177" s="12" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="K177" s="12" t="inlineStr">
+        <is>
+          <t>Bupa's full year 2025 results of 5 March 2026 report strong customer growth in its Spanish hospitals business, the opening of Hospital Blua Sanitas Valdebebas, and the end in 2024 of a PPP contract in that business.</t>
+        </is>
+      </c>
+      <c r="L177" s="14" t="inlineStr">
+        <is>
+          <t>Bupa, 2026-03-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B178" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C178" s="13" t="inlineStr">
+        <is>
+          <t>Burjeel Cancer Institute (Burjeel Holdings)</t>
+        </is>
+      </c>
+      <c r="D178" s="12" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="E178" s="12" t="inlineStr">
+        <is>
+          <t>Hospital Sant Joan de Déu Barcelona (SJD Barcelona Children's Hospital)</t>
+        </is>
+      </c>
+      <c r="F178" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G178" s="12" t="inlineStr">
+        <is>
+          <t>SJD Barcelona Children's Hospital and the Burjeel Cancer Institute in Abu Dhabi signed a memorandum of understanding in June 2025 on pediatric oncology and rare diseases. It covers joint management of complex cases, remote appointments and second opinions with SJD specialists, and expert visits.</t>
+        </is>
+      </c>
+      <c r="H178" s="12" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="I178" s="12" t="inlineStr"/>
+      <c r="J178" s="12" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="K178" s="12" t="inlineStr">
+        <is>
+          <t>SJD announced the memorandum on 9 June 2025.</t>
+        </is>
+      </c>
+      <c r="L178" s="14" t="inlineStr">
+        <is>
+          <t>SJD Barcelona Children's Hospital, 2025-06-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B179" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C179" s="13" t="inlineStr">
+        <is>
+          <t>Cancer Core Europe (Gustave Roussy, DKFZ and NCT Heidelberg, Netherlands Cancer Institute, Karolinska Institutet, Cancer Research UK Cambridge Centre, Istituto Nazionale dei Tumori Milan)</t>
+        </is>
+      </c>
+      <c r="D179" s="12" t="inlineStr">
+        <is>
+          <t>Multiple (France, Germany, Netherlands, Sweden, United Kingdom, Italy)</t>
+        </is>
+      </c>
+      <c r="E179" s="12" t="inlineStr">
+        <is>
+          <t>Vall d'Hebron Institute of Oncology (VHIO)</t>
+        </is>
+      </c>
+      <c r="F179" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G179" s="12" t="inlineStr">
+        <is>
+          <t>VHIO is a founding member of Cancer Core Europe, a standing consortium of seven European comprehensive cancer centres that runs joint translational research, clinical trial and training programmes. VHIO director Josep Tabernero has chaired the consortium since 2023.</t>
+        </is>
+      </c>
+      <c r="H179" s="12" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="I179" s="12" t="inlineStr"/>
+      <c r="J179" s="12" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="K179" s="12" t="inlineStr">
+        <is>
+          <t>VHIO announced on 18 October 2023 that Josep Tabernero took the chair of Cancer Core Europe. Karolinska Institutet's page for the consortium's 10th annual meeting in Stockholm on 23 and 24 March 2026 lists all seven members, including VHIO, and VHIO speakers.</t>
+        </is>
+      </c>
+      <c r="L179" s="14" t="inlineStr">
+        <is>
+          <t>Vall d'Hebron Institute of Oncology, 2023-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B180" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C180" s="13" t="inlineStr">
+        <is>
+          <t>Clariane (formerly Korian)</t>
+        </is>
+      </c>
+      <c r="D180" s="12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="E180" s="12" t="inlineStr">
+        <is>
+          <t>Clariane España (Ita Salud Mental, Grupo 5, Iterias)</t>
+        </is>
+      </c>
+      <c r="F180" s="12" t="inlineStr">
+        <is>
+          <t>Ownership or management</t>
+        </is>
+      </c>
+      <c r="G180" s="12" t="inlineStr">
+        <is>
+          <t>French care group Clariane owns Ita Salud Mental, bought in 2021, and Grupo 5, bought in 2023, giving it what Clariane calls the largest network of mental health facilities in the Iberian Peninsula with outpatient and inpatient psychiatric care, as well as the Seniors nursing homes. It opened the new Iterias psychotherapy brand in Barcelona in October 2025.</t>
+        </is>
+      </c>
+      <c r="H180" s="12" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="I180" s="12" t="inlineStr"/>
+      <c r="J180" s="12" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="K180" s="12" t="inlineStr">
+        <is>
+          <t>Korian announced on 11 January 2023 that it had closed the Grupo 5 acquisition, adding to Ita Salud acquired in 2021. Clariane launched Iterias in Spain on 21 October 2025, and its Spain page reports EUR 267 million of Spanish revenue and 164 facilities as of 31 December 2025.</t>
+        </is>
+      </c>
+      <c r="L180" s="14" t="inlineStr">
+        <is>
+          <t>Business Wire, 2023-01-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B181" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C181" s="13" t="inlineStr">
+        <is>
+          <t>Fresenius Helios (Helios Health)</t>
+        </is>
+      </c>
+      <c r="D181" s="12" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E181" s="12" t="inlineStr">
+        <is>
+          <t>Quirónsalud</t>
+        </is>
+      </c>
+      <c r="F181" s="12" t="inlineStr">
+        <is>
+          <t>Ownership or management</t>
+        </is>
+      </c>
+      <c r="G181" s="12" t="inlineStr">
+        <is>
+          <t>Fresenius Helios, the hospital arm of the German Fresenius group, has owned Quirónsalud, the largest private hospital group in Spain, since early 2017. Quirónsalud lists 57 hospitals in Spain on its website.</t>
+        </is>
+      </c>
+      <c r="H181" s="12" t="inlineStr">
+        <is>
+          <t>2017-01</t>
+        </is>
+      </c>
+      <c r="I181" s="12" t="inlineStr"/>
+      <c r="J181" s="12" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="K181" s="12" t="inlineStr">
+        <is>
+          <t>Quirónsalud announced the integration with Helios on 5 September 2016. Fresenius reported on 25 February 2026 that Helios Spain grew revenue 7% to EUR 5,429 million in 2025 and had the strongest performance in the group.</t>
+        </is>
+      </c>
+      <c r="L181" s="14" t="inlineStr">
+        <is>
+          <t>Quirónsalud, 2016-09-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B182" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C182" s="13" t="inlineStr">
+        <is>
+          <t>GenesisCare</t>
+        </is>
+      </c>
+      <c r="D182" s="12" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="E182" s="12" t="inlineStr">
+        <is>
+          <t>GenesisCare España (IMOncology and Oncosur radiotherapy centres)</t>
+        </is>
+      </c>
+      <c r="F182" s="12" t="inlineStr">
+        <is>
+          <t>Ownership or management</t>
+        </is>
+      </c>
+      <c r="G182" s="12" t="inlineStr">
+        <is>
+          <t>Australian cancer care provider GenesisCare entered Spain in 2016 by buying IMOncology and Oncosur and ran 18 oncology and radiotherapy centres and units, several inside Vithas and other private hospitals. In July 2026 it agreed to sell the Spanish business to Vithas; the sale awaits approval by the competition authority (CNMC), so the ownership tie continues.</t>
+        </is>
+      </c>
+      <c r="H182" s="12" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="I182" s="12" t="inlineStr"/>
+      <c r="J182" s="12" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="K182" s="12" t="inlineStr">
+        <is>
+          <t>Alimarket reported on 22 July 2026 that Vithas closed the purchase of GenesisCare's Spanish business, with 18 centres and EUR 39.1 million revenue in 2025, subject to CNMC authorisation; no clearance was found by October 2026.</t>
+        </is>
+      </c>
+      <c r="L182" s="14" t="inlineStr">
+        <is>
+          <t>Alimarket, 2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B183" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C183" s="13" t="inlineStr">
+        <is>
+          <t>Grupo Médico Joya (Hospitales Joya)</t>
+        </is>
+      </c>
+      <c r="D183" s="12" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="E183" s="12" t="inlineStr">
+        <is>
+          <t>HM Hospitales</t>
+        </is>
+      </c>
+      <c r="F183" s="12" t="inlineStr">
+        <is>
+          <t>Clinical affiliation</t>
+        </is>
+      </c>
+      <c r="G183" s="12" t="inlineStr">
+        <is>
+          <t>HM Hospitales and Mexican private hospital group Hospitales Joya signed a strategic framework agreement in September 2026 to support continuity of care for patients moving between Spain and Mexico. It also covers reciprocal rotations, fellowships and staff exchanges, links with HM's CIOCC, CIEC and CINAC centres, and sharing of clinical and management practice.</t>
+        </is>
+      </c>
+      <c r="H183" s="12" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="I183" s="12" t="inlineStr"/>
+      <c r="J183" s="12" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="K183" s="12" t="inlineStr">
+        <is>
+          <t>Alimarket reported on 11 September 2026 that the agreement was signed the previous Thursday at the Mexican Embassy in Spain by the chairs and chief executives of both groups.</t>
+        </is>
+      </c>
+      <c r="L183" s="14" t="inlineStr">
+        <is>
+          <t>Alimarket, 2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B184" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C184" s="13" t="inlineStr">
+        <is>
+          <t>Sun Yat-sen University Cancer Center</t>
+        </is>
+      </c>
+      <c r="D184" s="12" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E184" s="12" t="inlineStr">
+        <is>
+          <t>Hospital Sant Joan de Déu Barcelona (SJD Barcelona Children's Hospital)</t>
+        </is>
+      </c>
+      <c r="F184" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G184" s="12" t="inlineStr">
+        <is>
+          <t>SJD Barcelona Children's Hospital and Sun Yat-sen University Cancer Center in Guangzhou signed a strategic agreement in pediatric oncology in 2025, including a cross border virtual consultation system and joint work on cell immunotherapy and rare tumour guidelines. The two co-organised the China Pediatric Oncology Frontier Forum in November 2025.</t>
+        </is>
+      </c>
+      <c r="H184" s="12" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="I184" s="12" t="inlineStr"/>
+      <c r="J184" s="12" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="K184" s="12" t="inlineStr">
+        <is>
+          <t>SJD announced the agreement on 2 June 2025 and reported on 12 December 2025 that it co-organised the 2025 China Pediatric Oncology Frontier Forum hosted by the cancer center in Guangzhou in late November 2025.</t>
+        </is>
+      </c>
+      <c r="L184" s="14" t="inlineStr">
+        <is>
+          <t>SJD Barcelona Children's Hospital, 2025-06-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B185" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C185" s="13" t="inlineStr">
+        <is>
+          <t>Vivalto Santé</t>
+        </is>
+      </c>
+      <c r="D185" s="12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="E185" s="12" t="inlineStr">
+        <is>
+          <t>Ribera (Ribera Salud group)</t>
+        </is>
+      </c>
+      <c r="F185" s="12" t="inlineStr">
+        <is>
+          <t>Ownership or management</t>
+        </is>
+      </c>
+      <c r="G185" s="12" t="inlineStr">
+        <is>
+          <t>French private hospital group Vivalto Santé bought Ribera, which runs public concession and private hospitals in Spain, from Centene in November 2022 and is its main shareholder. Ribera signed to buy the HCB Hospitales group in Benidorm and Dénia in February 2026 and completed the purchase in October 2026, after the competition authority cleared it in September.</t>
+        </is>
+      </c>
+      <c r="H185" s="12" t="inlineStr">
+        <is>
+          <t>2022-11</t>
+        </is>
+      </c>
+      <c r="I185" s="12" t="inlineStr"/>
+      <c r="J185" s="12" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="K185" s="12" t="inlineStr">
+        <is>
+          <t>Centene announced completion of the sale of Ribera Salud and its other Spanish and central European businesses to Vivalto Santé on 17 November 2022. Ribera's release of 18 February 2026 on the HCB acquisition names Vivalto Santé as its main shareholder; Alimarket reported on 1 October 2026 that the CNMC cleared the deal on 21 September 2026. economia3 reported on 6 October 2026 that Ribera had completed the acquisition.</t>
+        </is>
+      </c>
+      <c r="L185" s="14" t="inlineStr">
+        <is>
+          <t>Becker's Healthcare, 2022-11-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B186" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C186" s="13" t="inlineStr">
+        <is>
+          <t>Johns Hopkins Proton Therapy Center (Johns Hopkins Medicine)</t>
+        </is>
+      </c>
+      <c r="D186" s="12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E186" s="12" t="inlineStr">
+        <is>
+          <t>Clínica Universidad de Navarra (Cancer Center) and Facultad de Medicina, Universidad de Navarra</t>
+        </is>
+      </c>
+      <c r="F186" s="12" t="inlineStr">
+        <is>
+          <t>Training and education</t>
+        </is>
+      </c>
+      <c r="G186" s="12" t="inlineStr">
+        <is>
+          <t>The Clínica Universidad de Navarra signed a collaboration agreement with the Johns Hopkins Proton Therapy Center in Washington in October 2023 to promote training and research in proton therapy for professionals in Spain's national health system.</t>
+        </is>
+      </c>
+      <c r="H186" s="12" t="inlineStr">
+        <is>
+          <t>2023-10</t>
+        </is>
+      </c>
+      <c r="I186" s="12" t="inlineStr"/>
+      <c r="J186" s="12" t="inlineStr">
+        <is>
+          <t>2023-10</t>
+        </is>
+      </c>
+      <c r="K186" s="12" t="inlineStr">
+        <is>
+          <t>CUN Cancer Center news item of 9 October 2023 announces the agreement; no later dated activity with Johns Hopkins found (CUN's 2025 and 2026 proton therapy courses do not name Johns Hopkins). Rule: latest evidence 2021 to September 2024 means Unclear.</t>
+        </is>
+      </c>
+      <c r="L186" s="14" t="inlineStr">
+        <is>
+          <t>Cancer Center Clínica Universidad de Navarra, 2023-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="15" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="B187" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C187" s="13" t="inlineStr">
+        <is>
+          <t>Hospital de Amor (Barretos Cancer Hospital)</t>
+        </is>
+      </c>
+      <c r="D187" s="12" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E187" s="12" t="inlineStr">
+        <is>
+          <t>Hospital Sant Joan de Déu Barcelona (SJD Barcelona Children's Hospital)</t>
+        </is>
+      </c>
+      <c r="F187" s="12" t="inlineStr">
+        <is>
+          <t>Research collaboration</t>
+        </is>
+      </c>
+      <c r="G187" s="12" t="inlineStr">
+        <is>
+          <t>SJD Barcelona Children's Hospital and Hospital de Amor in Barretos, Brazil, signed an agreement in 2021 to share knowledge in pediatric oncology protocols, training and research. No later activity was found.</t>
+        </is>
+      </c>
+      <c r="H187" s="12" t="inlineStr">
+        <is>
+          <t>2021-07</t>
+        </is>
+      </c>
+      <c r="I187" s="12" t="inlineStr"/>
+      <c r="J187" s="12" t="inlineStr">
+        <is>
+          <t>2021-07</t>
+        </is>
+      </c>
+      <c r="K187" s="12" t="inlineStr">
+        <is>
+          <t>SJD announced the agreement on 13 July 2021; no later public evidence of activity was found.</t>
+        </is>
+      </c>
+      <c r="L187" s="14" t="inlineStr">
+        <is>
+          <t>SJD Barcelona Children's Hospital, 2021-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="16" t="inlineStr">
+        <is>
+          <t>Ended</t>
+        </is>
+      </c>
+      <c r="B188" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="C188" s="13" t="inlineStr">
+        <is>
+          <t>Fresenius Helios (Helios Health)</t>
+        </is>
+      </c>
+      <c r="D188" s="12" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E188" s="12" t="inlineStr">
+        <is>
+          <t>Eugin Group (fertility clinics)</t>
+        </is>
+      </c>
+      <c r="F188" s="12" t="inlineStr">
+        <is>
+          <t>Ownership or management</t>
+        </is>
+      </c>
+      <c r="G188" s="12" t="inlineStr">
+        <is>
+          <t>Fresenius Helios bought the Barcelona based Eugin fertility clinic group from NMC Health's administrators in a deal signed in December 2020 and sold it to IVI RMA and GED Capital in January 2024. Helios kept the fertility units inside Quirónsalud hospitals.</t>
+        </is>
+      </c>
+      <c r="H188" s="12" t="inlineStr">
+        <is>
+          <t>2020-12</t>
+        </is>
+      </c>
+      <c r="I188" s="12" t="inlineStr">
+        <is>
+          <t>2024-01</t>
+        </is>
+      </c>
+      <c r="J188" s="12" t="inlineStr">
+        <is>
+          <t>2024-01</t>
+        </is>
+      </c>
+      <c r="K188" s="12" t="inlineStr">
+        <is>
+          <t>Fresenius announced the Eugin acquisition on 21 December 2020 and announced completion of the divestment to IVI RMA and GED Capital on 31 January 2024.</t>
+        </is>
+      </c>
+      <c r="L188" s="14" t="inlineStr">
+        <is>
+          <t>Fresenius, 2020-12-21</t>
         </is>
       </c>
     </row>
@@ -10391,10 +11721,33 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L163" r:id="rId162"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L164" r:id="rId163"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L165" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L166" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L167" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L168" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L169" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L170" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L171" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L172" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L173" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L174" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L175" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L176" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L177" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L178" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L179" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L180" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L181" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L182" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L183" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L184" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L185" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L186" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L187" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L188" r:id="rId187"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId165"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId188"/>
   </tableParts>
 </worksheet>
 </file>
@@ -10405,7 +11758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E328"/>
+  <dimension ref="A1:E382"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -19212,6 +20565,1444 @@
       <c r="E328" s="5" t="inlineStr">
         <is>
           <t>https://uathospital.ng/nigeria-china-signs-letter-of-intent-to-improve-health-sector/</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="5" t="inlineStr">
+        <is>
+          <t>Cleveland Clinic</t>
+        </is>
+      </c>
+      <c r="B329" s="5" t="inlineStr">
+        <is>
+          <t>Vall d'Hebron University Hospital (Advanced Clinical Simulation Centre)</t>
+        </is>
+      </c>
+      <c r="C329" s="5" t="inlineStr">
+        <is>
+          <t>Vall d'Hebron Vall d'Hebron and Cleveland Clinic sign an agreement to strengthen educational collaboration in the field of simulation</t>
+        </is>
+      </c>
+      <c r="D329" s="5" t="inlineStr">
+        <is>
+          <t>2025-02-07</t>
+        </is>
+      </c>
+      <c r="E329" s="5" t="inlineStr">
+        <is>
+          <t>https://www.vallhebron.com/en/news/news/vall-dhebron-and-cleveland-clinic-sign-agreement-strengthen-educational-collaboration-field-simulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="5" t="inlineStr">
+        <is>
+          <t>Cleveland Clinic</t>
+        </is>
+      </c>
+      <c r="B330" s="5" t="inlineStr">
+        <is>
+          <t>Vall d'Hebron University Hospital (Advanced Clinical Simulation Centre)</t>
+        </is>
+      </c>
+      <c r="C330" s="5" t="inlineStr">
+        <is>
+          <t>Vall d'Hebron Report 2025</t>
+        </is>
+      </c>
+      <c r="D330" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E330" s="5" t="inlineStr">
+        <is>
+          <t>https://hospital.vallhebron.com/en/about-us/corporate-documentation/report-2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="5" t="inlineStr">
+        <is>
+          <t>George Washington University (School of Medicine and Health Sciences)</t>
+        </is>
+      </c>
+      <c r="B331" s="5" t="inlineStr">
+        <is>
+          <t>Universidad Autonoma de Madrid (Faculty of Medicine)</t>
+        </is>
+      </c>
+      <c r="C331" s="5" t="inlineStr">
+        <is>
+          <t>Universidad Autonoma de Madrid, Facultad de Medicina Convocatoria de ayudas 2026-2027 para practicas clinicas en George Washington University</t>
+        </is>
+      </c>
+      <c r="D331" s="5" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="E331" s="5" t="inlineStr">
+        <is>
+          <t>https://www.uam.es/medicina/estudios/practicas-externas/convocatoria-george-washington-university</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="5" t="inlineStr">
+        <is>
+          <t>Harvard Medical School (Harvard University)</t>
+        </is>
+      </c>
+      <c r="B332" s="5" t="inlineStr">
+        <is>
+          <t>Universidad Complutense de Madrid (Faculty of Medicine; Hospital Clinico San Carlos, Hospital 12 de Octubre, Hospital Gregorio Maranon)</t>
+        </is>
+      </c>
+      <c r="C332" s="5" t="inlineStr">
+        <is>
+          <t>Universidad Complutense de Madrid, Facultad de Medicina Clinical rotation at Complutense Medical School (CMS) 2025-26: elective description</t>
+        </is>
+      </c>
+      <c r="D332" s="5" t="inlineStr">
+        <is>
+          <t>2025-10-28</t>
+        </is>
+      </c>
+      <c r="E332" s="5" t="inlineStr">
+        <is>
+          <t>https://medicina.ucm.es/file/elective-description-clinical-rotations-hms-cms-2025-2026-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="5" t="inlineStr">
+        <is>
+          <t>Harvard Medical School (Harvard University)</t>
+        </is>
+      </c>
+      <c r="B333" s="5" t="inlineStr">
+        <is>
+          <t>Universidad Complutense de Madrid (Faculty of Medicine; Hospital Clinico San Carlos, Hospital 12 de Octubre, Hospital Gregorio Maranon)</t>
+        </is>
+      </c>
+      <c r="C333" s="5" t="inlineStr">
+        <is>
+          <t>Alberto Martin Siete estudiantes de Medicina realizaran una estancia de un mes en Harvard</t>
+        </is>
+      </c>
+      <c r="D333" s="5" t="inlineStr">
+        <is>
+          <t>2020-01-30</t>
+        </is>
+      </c>
+      <c r="E333" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ucm.es/tribunacomplutense/264/art3995.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="5" t="inlineStr">
+        <is>
+          <t>Harvard Medical School (Harvard University)</t>
+        </is>
+      </c>
+      <c r="B334" s="5" t="inlineStr">
+        <is>
+          <t>Universidad Complutense de Madrid (Faculty of Medicine; Hospital Clinico San Carlos, Hospital 12 de Octubre, Hospital Gregorio Maranon)</t>
+        </is>
+      </c>
+      <c r="C334" s="5" t="inlineStr">
+        <is>
+          <t>Universidad Complutense de Madrid, Facultad de Medicina Convocatoria Becas Harvard Medical School 2022-2023</t>
+        </is>
+      </c>
+      <c r="D334" s="5" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="E334" s="5" t="inlineStr">
+        <is>
+          <t>https://medicina.ucm.es/data/cont/media/www/805/Convocatoria%20Harvard%202022%20-%2023%20EV-1.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="5" t="inlineStr">
+        <is>
+          <t>Johns Hopkins University (Bloomberg School of Public Health)</t>
+        </is>
+      </c>
+      <c r="B335" s="5" t="inlineStr">
+        <is>
+          <t>Universitat Pompeu Fabra (JHU-UPF Public Policy Center), with the Agencia de Salut Publica de Barcelona</t>
+        </is>
+      </c>
+      <c r="C335" s="5" t="inlineStr">
+        <is>
+          <t>JHU-UPF Public Policy Center Annual report: academic year 2024-2025: critical knowledge for decision-making</t>
+        </is>
+      </c>
+      <c r="D335" s="5" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="E335" s="5" t="inlineStr">
+        <is>
+          <t>https://repositori.upf.edu/items/3552909c-eb4b-47bd-91c3-47699ba09b59/full</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="5" t="inlineStr">
+        <is>
+          <t>Johns Hopkins University (Bloomberg School of Public Health)</t>
+        </is>
+      </c>
+      <c r="B336" s="5" t="inlineStr">
+        <is>
+          <t>Universitat Pompeu Fabra (JHU-UPF Public Policy Center), with the Agencia de Salut Publica de Barcelona</t>
+        </is>
+      </c>
+      <c r="C336" s="5" t="inlineStr">
+        <is>
+          <t>JHU-UPF Public Policy Center Hopkins Fall Institute</t>
+        </is>
+      </c>
+      <c r="D336" s="5" t="inlineStr"/>
+      <c r="E336" s="5" t="inlineStr">
+        <is>
+          <t>https://www.upf.edu/web/jhu-ppc/hopkins-fall-institute</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="5" t="inlineStr">
+        <is>
+          <t>Johns Hopkins University (Bloomberg School of Public Health)</t>
+        </is>
+      </c>
+      <c r="B337" s="5" t="inlineStr">
+        <is>
+          <t>Universitat Pompeu Fabra (JHU-UPF Public Policy Center), with the Agencia de Salut Publica de Barcelona</t>
+        </is>
+      </c>
+      <c r="C337" s="5" t="inlineStr">
+        <is>
+          <t>Johns Hopkins Bloomberg School of Public Health Fall Institute in Health Policy and Management</t>
+        </is>
+      </c>
+      <c r="D337" s="5" t="inlineStr"/>
+      <c r="E337" s="5" t="inlineStr">
+        <is>
+          <t>https://publichealth.jhu.edu/academics/fall-institute-in-health-policy-and-management</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="5" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center</t>
+        </is>
+      </c>
+      <c r="B338" s="5" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center Madrid (operated by Grupo Hospiten)</t>
+        </is>
+      </c>
+      <c r="C338" s="5" t="inlineStr">
+        <is>
+          <t>Hospiten MD Anderson Cancer Center Madrid - Hospiten, recognised among the world's leading cancer hospitals by Newsweek and Statista</t>
+        </is>
+      </c>
+      <c r="D338" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="E338" s="5" t="inlineStr">
+        <is>
+          <t>https://hospiten.com/en/news/md-anderson-cancer-center-madrid-hospiten-reconocido-los-mejores-hospitales-oncologicos</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="5" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center</t>
+        </is>
+      </c>
+      <c r="B339" s="5" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center Madrid (operated by Grupo Hospiten)</t>
+        </is>
+      </c>
+      <c r="C339" s="5" t="inlineStr">
+        <is>
+          <t>Hospiten MD Anderson Cancer Center Madrid Hospiten, recognized by Forbes among the three best oncology hospitals in Spain</t>
+        </is>
+      </c>
+      <c r="D339" s="5" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="E339" s="5" t="inlineStr">
+        <is>
+          <t>https://hospiten.com/en/news/md-anderson-cancer-center-madrid-hospiten-recognized-by-forbes</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="5" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center</t>
+        </is>
+      </c>
+      <c r="B340" s="5" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center Madrid (operated by Grupo Hospiten)</t>
+        </is>
+      </c>
+      <c r="C340" s="5" t="inlineStr">
+        <is>
+          <t>Hospiten Grupo Hospiten adquiere el 39,98% de las acciones de MD Anderson Cancer Center Madrid</t>
+        </is>
+      </c>
+      <c r="D340" s="5" t="inlineStr">
+        <is>
+          <t>2013-01-10</t>
+        </is>
+      </c>
+      <c r="E340" s="5" t="inlineStr">
+        <is>
+          <t>https://hospiten.com/noticias/grupo-hospiten-compra-a-cartera-industrial-rea-su-participacion-en-el-md-anderson-cancer-center-madrid-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="5" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center</t>
+        </is>
+      </c>
+      <c r="B341" s="5" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center Madrid (operated by Grupo Hospiten)</t>
+        </is>
+      </c>
+      <c r="C341" s="5" t="inlineStr">
+        <is>
+          <t>MD Anderson Cancer Center Chapter 22: Sister Institutions (John Mendelsohn oral history)</t>
+        </is>
+      </c>
+      <c r="D341" s="5" t="inlineStr"/>
+      <c r="E341" s="5" t="inlineStr">
+        <is>
+          <t>https://openworks.mdanderson.org/mchv_interviewchapters/1438/</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="5" t="inlineStr">
+        <is>
+          <t>Mount Sinai Health System (Icahn School of Medicine, Mount Sinai Fuster Heart Hospital)</t>
+        </is>
+      </c>
+      <c r="B342" s="5" t="inlineStr">
+        <is>
+          <t>Centro Nacional de Investigaciones Cardiovasculares Carlos III (CNIC)</t>
+        </is>
+      </c>
+      <c r="C342" s="5" t="inlineStr">
+        <is>
+          <t>Mount Sinai Health System Beta blockers, the standard treatment after a heart attack, may offer no benefit for heart attack patients and women can have worse outcomes</t>
+        </is>
+      </c>
+      <c r="D342" s="5" t="inlineStr">
+        <is>
+          <t>2025-08-30</t>
+        </is>
+      </c>
+      <c r="E342" s="5" t="inlineStr">
+        <is>
+          <t>https://www.eurekalert.org/news-releases/1096364</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="5" t="inlineStr">
+        <is>
+          <t>Mount Sinai Health System (Icahn School of Medicine, Mount Sinai Fuster Heart Hospital)</t>
+        </is>
+      </c>
+      <c r="B343" s="5" t="inlineStr">
+        <is>
+          <t>Centro Nacional de Investigaciones Cardiovasculares Carlos III (CNIC)</t>
+        </is>
+      </c>
+      <c r="C343" s="5" t="inlineStr">
+        <is>
+          <t>Mount Sinai Health System Presence of subclinical atherosclerosis is marker of mortality and its progression increases risk of death</t>
+        </is>
+      </c>
+      <c r="D343" s="5" t="inlineStr">
+        <is>
+          <t>2024-09-30</t>
+        </is>
+      </c>
+      <c r="E343" s="5" t="inlineStr">
+        <is>
+          <t>https://www.eurekalert.org/news-releases/1059621</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="5" t="inlineStr">
+        <is>
+          <t>Mount Sinai Health System (Icahn School of Medicine, Mount Sinai Fuster Heart Hospital)</t>
+        </is>
+      </c>
+      <c r="B344" s="5" t="inlineStr">
+        <is>
+          <t>Centro Nacional de Investigaciones Cardiovasculares Carlos III (CNIC)</t>
+        </is>
+      </c>
+      <c r="C344" s="5" t="inlineStr">
+        <is>
+          <t>CNIC Shared learning between two giants of cardiovascular research</t>
+        </is>
+      </c>
+      <c r="D344" s="5" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="E344" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cnic.es/en/node/821</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="5" t="inlineStr">
+        <is>
+          <t>Penn State College of Medicine and Penn State Health (Beat Childhood Cancer Research Consortium)</t>
+        </is>
+      </c>
+      <c r="B345" s="5" t="inlineStr">
+        <is>
+          <t>Hospital Sant Joan de Déu Barcelona (Pediatric Cancer Center Barcelona)</t>
+        </is>
+      </c>
+      <c r="C345" s="5" t="inlineStr">
+        <is>
+          <t>SJD Barcelona Children's Hospital The SJD Barcelona Children's Hospital will be the first member of the Beat Childhood Cancer Consortium based outside of North America</t>
+        </is>
+      </c>
+      <c r="D345" s="5" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="E345" s="5" t="inlineStr">
+        <is>
+          <t>https://www.sjdhospitalbarcelona.org/en/news/sjd-barcelona-childrens-hospital-will-be-first-member-beat-childhood-cancer-consortium-based-outside-north-america</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="5" t="inlineStr">
+        <is>
+          <t>Penn State College of Medicine and Penn State Health (Beat Childhood Cancer Research Consortium)</t>
+        </is>
+      </c>
+      <c r="B346" s="5" t="inlineStr">
+        <is>
+          <t>Hospital Sant Joan de Déu Barcelona (Pediatric Cancer Center Barcelona)</t>
+        </is>
+      </c>
+      <c r="C346" s="5" t="inlineStr">
+        <is>
+          <t>Penn State Health News Penn State's Beat Childhood Cancer Research Consortium welcomes SJD Pediatric Cancer Center Barcelona</t>
+        </is>
+      </c>
+      <c r="D346" s="5" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="E346" s="5" t="inlineStr">
+        <is>
+          <t>https://pennstatehealthnews.org/2025/11/penn-states-beat-childhood-cancer-research-consortium-welcomes-sjd-pediatric-cancer-center-barcelona/</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="5" t="inlineStr">
+        <is>
+          <t>University of Illinois Chicago (College of Applied Health Sciences)</t>
+        </is>
+      </c>
+      <c r="B347" s="5" t="inlineStr">
+        <is>
+          <t>TecnoCampus School of Health Sciences (Universitat Pompeu Fabra)</t>
+        </is>
+      </c>
+      <c r="C347" s="5" t="inlineStr">
+        <is>
+          <t>Emily Parenti-Lopez AHS dean formalizes international collaboration between UIC and Spanish university</t>
+        </is>
+      </c>
+      <c r="D347" s="5" t="inlineStr">
+        <is>
+          <t>2025-10-20</t>
+        </is>
+      </c>
+      <c r="E347" s="5" t="inlineStr">
+        <is>
+          <t>https://ahs.uic.edu/news-stories/ahs-dean-formalizes-international-collaboration-between-uic-and-spanish-university</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="5" t="inlineStr">
+        <is>
+          <t>University of Kansas Medical Center</t>
+        </is>
+      </c>
+      <c r="B348" s="5" t="inlineStr">
+        <is>
+          <t>Universitat Internacional de Catalunya (UIC Barcelona) Faculty of Medicine and Health Sciences</t>
+        </is>
+      </c>
+      <c r="C348" s="5" t="inlineStr">
+        <is>
+          <t>Universitat Internacional de Catalunya Medicine degree brochure (English)</t>
+        </is>
+      </c>
+      <c r="D348" s="5" t="inlineStr">
+        <is>
+          <t>2026-02-16</t>
+        </is>
+      </c>
+      <c r="E348" s="5" t="inlineStr">
+        <is>
+          <t>https://www.uic.es/sites/default/files/folleto-medicina-eng.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="5" t="inlineStr">
+        <is>
+          <t>University of Kansas Medical Center</t>
+        </is>
+      </c>
+      <c r="B349" s="5" t="inlineStr">
+        <is>
+          <t>Universitat Internacional de Catalunya (UIC Barcelona) Faculty of Medicine and Health Sciences</t>
+        </is>
+      </c>
+      <c r="C349" s="5" t="inlineStr">
+        <is>
+          <t>University of Kansas Medical Center, Office of International Programs International Educational Experiences: Spain</t>
+        </is>
+      </c>
+      <c r="D349" s="5" t="inlineStr"/>
+      <c r="E349" s="5" t="inlineStr">
+        <is>
+          <t>https://www.kumc.edu/academic-and-student-affairs/departments/office-of-international-programs/outbound-programs/international-educational-experiences/program-locations/spain.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="5" t="inlineStr">
+        <is>
+          <t>ABC Medical Center (Centro Médico ABC)</t>
+        </is>
+      </c>
+      <c r="B350" s="5" t="inlineStr">
+        <is>
+          <t>Hospital Sant Joan de Déu Barcelona (SJD Barcelona Children's Hospital)</t>
+        </is>
+      </c>
+      <c r="C350" s="5" t="inlineStr">
+        <is>
+          <t>Hospital Sant Joan de Déu Barcelona The SJD Barcelona Children's Hospital and the ABC Medical Center in Mexico collaborate to advance pediatric oncology</t>
+        </is>
+      </c>
+      <c r="D350" s="5" t="inlineStr">
+        <is>
+          <t>2025-08-29</t>
+        </is>
+      </c>
+      <c r="E350" s="5" t="inlineStr">
+        <is>
+          <t>https://www.sjdhospitalbarcelona.org/en/news/sjd-barcelona-childrens-hospital-abc-medical-center-mexico-collaborate-advance-pediatric-oncology</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="5" t="inlineStr">
+        <is>
+          <t>Aier Eye Hospital Group</t>
+        </is>
+      </c>
+      <c r="B351" s="5" t="inlineStr">
+        <is>
+          <t>Clínica Baviera</t>
+        </is>
+      </c>
+      <c r="C351" s="5" t="inlineStr">
+        <is>
+          <t>Alimarket Sanidad La china Aier Eye Hospital toma el control de Clínica Baviera</t>
+        </is>
+      </c>
+      <c r="D351" s="5" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="E351" s="5" t="inlineStr">
+        <is>
+          <t>https://www.alimarket.es/sanidad/noticia/239028/la-china-aier-eye-hospital-toma-el-control-de-clinica-baviera</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="5" t="inlineStr">
+        <is>
+          <t>Aier Eye Hospital Group</t>
+        </is>
+      </c>
+      <c r="B352" s="5" t="inlineStr">
+        <is>
+          <t>Clínica Baviera</t>
+        </is>
+      </c>
+      <c r="C352" s="5" t="inlineStr">
+        <is>
+          <t>Alantra Alantra Acts as Global Coordinator in the c.EUR42.4mn Placement of Clinica Baviera's Shares</t>
+        </is>
+      </c>
+      <c r="D352" s="5" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="E352" s="5" t="inlineStr">
+        <is>
+          <t>https://www.alantra.com/ib-transaction/clinica-baviera-accelerated-bookbuilding/</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="5" t="inlineStr">
+        <is>
+          <t>Aier Eye Hospital Group</t>
+        </is>
+      </c>
+      <c r="B353" s="5" t="inlineStr">
+        <is>
+          <t>Clínica Baviera</t>
+        </is>
+      </c>
+      <c r="C353" s="5" t="inlineStr">
+        <is>
+          <t>elEconomista Los dueños de Clínica Baviera venden un 8% de la compañía por 42,4 millones</t>
+        </is>
+      </c>
+      <c r="D353" s="5" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="E353" s="5" t="inlineStr">
+        <is>
+          <t>https://www.eleconomista.es/salud-bienestar/noticias/13301420/04/25/los-duenos-de-clinica-baviera-venden-un-8-de-la-compania-por-424-millones.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="5" t="inlineStr">
+        <is>
+          <t>Aier Eye Hospital Group</t>
+        </is>
+      </c>
+      <c r="B354" s="5" t="inlineStr">
+        <is>
+          <t>Clínica Baviera</t>
+        </is>
+      </c>
+      <c r="C354" s="5" t="inlineStr">
+        <is>
+          <t>Clínica Baviera Aier Eye Hospital (shareholder page)</t>
+        </is>
+      </c>
+      <c r="D354" s="5" t="inlineStr"/>
+      <c r="E354" s="5" t="inlineStr">
+        <is>
+          <t>https://grupobaviera.es/accionistas-inversores/en/aier-eye-hospital/</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="5" t="inlineStr">
+        <is>
+          <t>Bupa</t>
+        </is>
+      </c>
+      <c r="B355" s="5" t="inlineStr">
+        <is>
+          <t>Sanitas (Sanitas hospitals)</t>
+        </is>
+      </c>
+      <c r="C355" s="5" t="inlineStr">
+        <is>
+          <t>Bupa Bupa Group full year financial results 2025</t>
+        </is>
+      </c>
+      <c r="D355" s="5" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="E355" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bupa.com/news-and-press/press-releases/2026/bupa-group-full-year-financial-results-2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="5" t="inlineStr">
+        <is>
+          <t>Bupa</t>
+        </is>
+      </c>
+      <c r="B356" s="5" t="inlineStr">
+        <is>
+          <t>Sanitas (Sanitas hospitals)</t>
+        </is>
+      </c>
+      <c r="C356" s="5" t="inlineStr">
+        <is>
+          <t>Bupa Results announcement and financial statement FY2025</t>
+        </is>
+      </c>
+      <c r="D356" s="5" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="E356" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bupa.com/~/media/files/b/bupa-v5/documents/financials/results-centre/2025/bupa-group-results-and-financial-statement-fy2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="5" t="inlineStr">
+        <is>
+          <t>Bupa</t>
+        </is>
+      </c>
+      <c r="B357" s="5" t="inlineStr">
+        <is>
+          <t>Sanitas (Sanitas hospitals)</t>
+        </is>
+      </c>
+      <c r="C357" s="5" t="inlineStr">
+        <is>
+          <t>Sanitas Sanitas 2026 executive summary</t>
+        </is>
+      </c>
+      <c r="D357" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="E357" s="5" t="inlineStr">
+        <is>
+          <t>https://informeanual.sanitas.es/wp-content/uploads/2026/07/Sanitas_2026_resumen-ejecutivo_EN.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="5" t="inlineStr">
+        <is>
+          <t>Burjeel Cancer Institute (Burjeel Holdings)</t>
+        </is>
+      </c>
+      <c r="B358" s="5" t="inlineStr">
+        <is>
+          <t>Hospital Sant Joan de Déu Barcelona (SJD Barcelona Children's Hospital)</t>
+        </is>
+      </c>
+      <c r="C358" s="5" t="inlineStr">
+        <is>
+          <t>Hospital Sant Joan de Déu Barcelona New international partnership between the SJD Barcelona Children's Hospital and the Burjeel Cancer Institute</t>
+        </is>
+      </c>
+      <c r="D358" s="5" t="inlineStr">
+        <is>
+          <t>2025-06-09</t>
+        </is>
+      </c>
+      <c r="E358" s="5" t="inlineStr">
+        <is>
+          <t>https://www.sjdhospitalbarcelona.org/en/news/new-international-partnership-between-sjd-barcelona-childrens-hospital-burjeel-cancer-institute</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="5" t="inlineStr">
+        <is>
+          <t>Cancer Core Europe (Gustave Roussy, DKFZ and NCT Heidelberg, Netherlands Cancer Institute, Karolinska Institutet, Cancer Research UK Cambridge Centre, Istituto Nazionale dei Tumori Milan)</t>
+        </is>
+      </c>
+      <c r="B359" s="5" t="inlineStr">
+        <is>
+          <t>Vall d'Hebron Institute of Oncology (VHIO)</t>
+        </is>
+      </c>
+      <c r="C359" s="5" t="inlineStr">
+        <is>
+          <t>VHIO Dr. Josep Tabernero, director of VHIO, chairman of the European consortium Cancer Core Europe</t>
+        </is>
+      </c>
+      <c r="D359" s="5" t="inlineStr">
+        <is>
+          <t>2023-10-18</t>
+        </is>
+      </c>
+      <c r="E359" s="5" t="inlineStr">
+        <is>
+          <t>https://vhio.net/2023/10/18/dr-josep-tabernero-director-of-vhio-assumes-the-presidency-of-the-european-project-cancer-core-europe</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="5" t="inlineStr">
+        <is>
+          <t>Cancer Core Europe (Gustave Roussy, DKFZ and NCT Heidelberg, Netherlands Cancer Institute, Karolinska Institutet, Cancer Research UK Cambridge Centre, Istituto Nazionale dei Tumori Milan)</t>
+        </is>
+      </c>
+      <c r="B360" s="5" t="inlineStr">
+        <is>
+          <t>Vall d'Hebron Institute of Oncology (VHIO)</t>
+        </is>
+      </c>
+      <c r="C360" s="5" t="inlineStr">
+        <is>
+          <t>Karolinska Institutet About Cancer Core Europe (CCE Annual Meeting and Karolinska CCC Days 2026)</t>
+        </is>
+      </c>
+      <c r="D360" s="5" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="E360" s="5" t="inlineStr">
+        <is>
+          <t>https://ki.se/en/cancer-research-ki/collaborations/cce-annual-meeting-karolinska-ccc-days-2026/about-cancer-core-europe</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="5" t="inlineStr">
+        <is>
+          <t>Clariane (formerly Korian)</t>
+        </is>
+      </c>
+      <c r="B361" s="5" t="inlineStr">
+        <is>
+          <t>Clariane España (Ita Salud Mental, Grupo 5, Iterias)</t>
+        </is>
+      </c>
+      <c r="C361" s="5" t="inlineStr">
+        <is>
+          <t>Korian Korian Closes the Acquisition of Grupo 5 Reinforcing Korian Position in Mental Health in Spain</t>
+        </is>
+      </c>
+      <c r="D361" s="5" t="inlineStr">
+        <is>
+          <t>2023-01-11</t>
+        </is>
+      </c>
+      <c r="E361" s="5" t="inlineStr">
+        <is>
+          <t>https://www.businesswire.com/news/home/20230111005688/en/Korian-Closes-the-Acquisition-of-Grupo-5-Reinforcing-Korian-Position-in-Mental-Health-in-Spain</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="5" t="inlineStr">
+        <is>
+          <t>Clariane (formerly Korian)</t>
+        </is>
+      </c>
+      <c r="B362" s="5" t="inlineStr">
+        <is>
+          <t>Clariane España (Ita Salud Mental, Grupo 5, Iterias)</t>
+        </is>
+      </c>
+      <c r="C362" s="5" t="inlineStr">
+        <is>
+          <t>Clariane Clariane launches Iterias in Spain, a new brand dedicated to psychotherapy for all</t>
+        </is>
+      </c>
+      <c r="D362" s="5" t="inlineStr">
+        <is>
+          <t>2025-10-21</t>
+        </is>
+      </c>
+      <c r="E362" s="5" t="inlineStr">
+        <is>
+          <t>https://www.clariane.com/en/press-room/press-releases/clariane-launches-iterias-in-spain-a-new-brand-dedicated-to-psychotherapy</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="5" t="inlineStr">
+        <is>
+          <t>Clariane (formerly Korian)</t>
+        </is>
+      </c>
+      <c r="B363" s="5" t="inlineStr">
+        <is>
+          <t>Clariane España (Ita Salud Mental, Grupo 5, Iterias)</t>
+        </is>
+      </c>
+      <c r="C363" s="5" t="inlineStr">
+        <is>
+          <t>Clariane Clariane in Spain</t>
+        </is>
+      </c>
+      <c r="D363" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E363" s="5" t="inlineStr">
+        <is>
+          <t>https://clariane.com/en/our-locations/clariane-in-spain</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="5" t="inlineStr">
+        <is>
+          <t>Fresenius Helios (Helios Health)</t>
+        </is>
+      </c>
+      <c r="B364" s="5" t="inlineStr">
+        <is>
+          <t>Quirónsalud</t>
+        </is>
+      </c>
+      <c r="C364" s="5" t="inlineStr">
+        <is>
+          <t>Quirónsalud Quirónsalud y Helios crean un grupo sanitario hispano-alemán, el mayor de Europa y uno de los mayores del mundo</t>
+        </is>
+      </c>
+      <c r="D364" s="5" t="inlineStr">
+        <is>
+          <t>2016-09-05</t>
+        </is>
+      </c>
+      <c r="E364" s="5" t="inlineStr">
+        <is>
+          <t>https://www.quironsalud.com/en/communication/news/quironsalud-helios-crean-grupo-sanitario-hispano-alem-25d03</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="5" t="inlineStr">
+        <is>
+          <t>Fresenius Helios (Helios Health)</t>
+        </is>
+      </c>
+      <c r="B365" s="5" t="inlineStr">
+        <is>
+          <t>Quirónsalud</t>
+        </is>
+      </c>
+      <c r="C365" s="5" t="inlineStr">
+        <is>
+          <t>Fresenius SE &amp; Co. KGaA #FutureFresenius: REJUVENATE in action (Q4 and FY 2025 results)</t>
+        </is>
+      </c>
+      <c r="D365" s="5" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="E365" s="5" t="inlineStr">
+        <is>
+          <t>https://www.fresenius.com/press-release-q4-2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="5" t="inlineStr">
+        <is>
+          <t>Fresenius Helios (Helios Health)</t>
+        </is>
+      </c>
+      <c r="B366" s="5" t="inlineStr">
+        <is>
+          <t>Quirónsalud</t>
+        </is>
+      </c>
+      <c r="C366" s="5" t="inlineStr">
+        <is>
+          <t>Fresenius SE &amp; Co. KGaA Fresenius Press Release Q4 and FY 2025</t>
+        </is>
+      </c>
+      <c r="D366" s="5" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="E366" s="5" t="inlineStr">
+        <is>
+          <t>https://www.fresenius.com/sites/default/files/2026-02/20260225_fse_presserelease_q4_2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="5" t="inlineStr">
+        <is>
+          <t>Fresenius Helios (Helios Health)</t>
+        </is>
+      </c>
+      <c r="B367" s="5" t="inlineStr">
+        <is>
+          <t>Quirónsalud</t>
+        </is>
+      </c>
+      <c r="C367" s="5" t="inlineStr">
+        <is>
+          <t>Quirónsalud Quirónsalud corporate site</t>
+        </is>
+      </c>
+      <c r="D367" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E367" s="5" t="inlineStr">
+        <is>
+          <t>https://www.quironsalud.com/en</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="5" t="inlineStr">
+        <is>
+          <t>GenesisCare</t>
+        </is>
+      </c>
+      <c r="B368" s="5" t="inlineStr">
+        <is>
+          <t>GenesisCare España (IMOncology and Oncosur radiotherapy centres)</t>
+        </is>
+      </c>
+      <c r="C368" s="5" t="inlineStr">
+        <is>
+          <t>Alimarket Sanidad El grupo australiano GenesisCare entra en España con la compra del 100% de IMOncology</t>
+        </is>
+      </c>
+      <c r="D368" s="5" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="E368" s="5" t="inlineStr">
+        <is>
+          <t>https://www.alimarket.es/noticia/214426/el-grupo-australiano-genesiscare-entra-en-espana-con-la-compra-del-100--de--imoncology</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="5" t="inlineStr">
+        <is>
+          <t>GenesisCare</t>
+        </is>
+      </c>
+      <c r="B369" s="5" t="inlineStr">
+        <is>
+          <t>GenesisCare España (IMOncology and Oncosur radiotherapy centres)</t>
+        </is>
+      </c>
+      <c r="C369" s="5" t="inlineStr">
+        <is>
+          <t>Eva de Frutos Vithas cierra la compra de GenesisCare España</t>
+        </is>
+      </c>
+      <c r="D369" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="E369" s="5" t="inlineStr">
+        <is>
+          <t>https://www.alimarket.es/sanidad/noticia/429416/vithas-cierra-la-compra-de-genesiscare-espana</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="5" t="inlineStr">
+        <is>
+          <t>GenesisCare</t>
+        </is>
+      </c>
+      <c r="B370" s="5" t="inlineStr">
+        <is>
+          <t>GenesisCare España (IMOncology and Oncosur radiotherapy centres)</t>
+        </is>
+      </c>
+      <c r="C370" s="5" t="inlineStr">
+        <is>
+          <t>El Español Invertia Vithas adquiere GenesisCare para reforzar su red asistencial oncológica</t>
+        </is>
+      </c>
+      <c r="D370" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="E370" s="5" t="inlineStr">
+        <is>
+          <t>https://www.elespanol.com/invertia/observatorios/sanidad/20260721/vithas-adquiere-genesiscare-reforzar-red-asistencial-oncologica-nuevos-centros-hospitalarios/1003744328844_0.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Médico Joya (Hospitales Joya)</t>
+        </is>
+      </c>
+      <c r="B371" s="5" t="inlineStr">
+        <is>
+          <t>HM Hospitales</t>
+        </is>
+      </c>
+      <c r="C371" s="5" t="inlineStr">
+        <is>
+          <t>Alimarket Sanidad HM Hospitales y Grupo Médico Joya sellan una alianza estratégica para impulsar la continuidad asistencial entre España y México</t>
+        </is>
+      </c>
+      <c r="D371" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E371" s="5" t="inlineStr">
+        <is>
+          <t>https://www.alimarket.es/sanidad/noticia/430873/hm-hospitales-y-grupo-medico-joya-sellan-una-alianza-estrategica-para-impulsar-la-continuidad-asistencial-entre-espana-y-mexico</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="5" t="inlineStr">
+        <is>
+          <t>Sun Yat-sen University Cancer Center</t>
+        </is>
+      </c>
+      <c r="B372" s="5" t="inlineStr">
+        <is>
+          <t>Hospital Sant Joan de Déu Barcelona (SJD Barcelona Children's Hospital)</t>
+        </is>
+      </c>
+      <c r="C372" s="5" t="inlineStr">
+        <is>
+          <t>Hospital Sant Joan de Déu Barcelona The SJD Barcelona Children's Hospital signs an agreement with the Sun Yat-sen University Cancer Center to help further research in pediatric oncology</t>
+        </is>
+      </c>
+      <c r="D372" s="5" t="inlineStr">
+        <is>
+          <t>2025-06-02</t>
+        </is>
+      </c>
+      <c r="E372" s="5" t="inlineStr">
+        <is>
+          <t>https://www.sjdhospitalbarcelona.org/en/news/sjd-barcelona-childrens-hospital-signs-agreement-sun-yat-sen-university-cancer-center-help-further-research-pediatric-oncology</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="5" t="inlineStr">
+        <is>
+          <t>Sun Yat-sen University Cancer Center</t>
+        </is>
+      </c>
+      <c r="B373" s="5" t="inlineStr">
+        <is>
+          <t>Hospital Sant Joan de Déu Barcelona (SJD Barcelona Children's Hospital)</t>
+        </is>
+      </c>
+      <c r="C373" s="5" t="inlineStr">
+        <is>
+          <t>Hospital Sant Joan de Déu Barcelona SJD Barcelona Children's Hospital experts were invited to the 2025 China Pediatric Oncology Frontier Forum</t>
+        </is>
+      </c>
+      <c r="D373" s="5" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="E373" s="5" t="inlineStr">
+        <is>
+          <t>https://www.sjdhospitalbarcelona.org/en/news/sjd-barcelona-childrens-hospital-experts-were-invited-2025-china-pediatric-oncology-frontier-forum</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="5" t="inlineStr">
+        <is>
+          <t>Vivalto Santé</t>
+        </is>
+      </c>
+      <c r="B374" s="5" t="inlineStr">
+        <is>
+          <t>Ribera (Ribera Salud group)</t>
+        </is>
+      </c>
+      <c r="C374" s="5" t="inlineStr">
+        <is>
+          <t>Becker's Payer Issues Centene completes sale of Spanish, central European businesses</t>
+        </is>
+      </c>
+      <c r="D374" s="5" t="inlineStr">
+        <is>
+          <t>2022-11-17</t>
+        </is>
+      </c>
+      <c r="E374" s="5" t="inlineStr">
+        <is>
+          <t>https://www.beckerspayer.com/m-and-a/centene-completes-sale-of-spanish-central-european-businesses.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="5" t="inlineStr">
+        <is>
+          <t>Vivalto Santé</t>
+        </is>
+      </c>
+      <c r="B375" s="5" t="inlineStr">
+        <is>
+          <t>Ribera (Ribera Salud group)</t>
+        </is>
+      </c>
+      <c r="C375" s="5" t="inlineStr">
+        <is>
+          <t>Vivalto Santé Vivalto Santé entame un fort développement en Europe</t>
+        </is>
+      </c>
+      <c r="D375" s="5" t="inlineStr">
+        <is>
+          <t>2022-11-17</t>
+        </is>
+      </c>
+      <c r="E375" s="5" t="inlineStr">
+        <is>
+          <t>https://www.vivalto-sante.com/wp-content/uploads/2022/11/2022-11-17-Vivalto-Sante-entame-un-fort-developpement-en-europe.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="5" t="inlineStr">
+        <is>
+          <t>Vivalto Santé</t>
+        </is>
+      </c>
+      <c r="B376" s="5" t="inlineStr">
+        <is>
+          <t>Ribera (Ribera Salud group)</t>
+        </is>
+      </c>
+      <c r="C376" s="5" t="inlineStr">
+        <is>
+          <t>Ribera Health Group Ribera signs the acquisition of the HCB Hospitals group and reinforces its growth in the Valencian Community</t>
+        </is>
+      </c>
+      <c r="D376" s="5" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="E376" s="5" t="inlineStr">
+        <is>
+          <t>https://www.riberasalud.com/en/ribera-firma-la-adquisicion-del-grupo-hcb-hospitales-y-refuerza-su-crecimiento-en-la-comunidad-valenciana/</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="5" t="inlineStr">
+        <is>
+          <t>Vivalto Santé</t>
+        </is>
+      </c>
+      <c r="B377" s="5" t="inlineStr">
+        <is>
+          <t>Ribera (Ribera Salud group)</t>
+        </is>
+      </c>
+      <c r="C377" s="5" t="inlineStr">
+        <is>
+          <t>Alimarket Sanidad La CNMC autoriza en primera fase y con compromisos la adquisición del Grupo HCB Hospitales por parte de Grupo Ribera</t>
+        </is>
+      </c>
+      <c r="D377" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E377" s="5" t="inlineStr">
+        <is>
+          <t>https://www.alimarket.es/sanidad/noticia/431931/la-cnmc-autoriza-en-primera-fase-y-con-compromisos-la-adquisicion-del-grupo-hcb-hospitales-por-parte-de-grupo-ribera</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="5" t="inlineStr">
+        <is>
+          <t>Vivalto Santé</t>
+        </is>
+      </c>
+      <c r="B378" s="5" t="inlineStr">
+        <is>
+          <t>Ribera (Ribera Salud group)</t>
+        </is>
+      </c>
+      <c r="C378" s="5" t="inlineStr">
+        <is>
+          <t>economia3 Ribera culmina la compra de HCB y refuerza su red sanitaria valenciana</t>
+        </is>
+      </c>
+      <c r="D378" s="5" t="inlineStr">
+        <is>
+          <t>6 October 2026</t>
+        </is>
+      </c>
+      <c r="E378" s="5" t="inlineStr">
+        <is>
+          <t>https://economia3.com/2026/10/06/762373-ribera-culmina-la-compra-de-hcb-y-refuerza-su-red-sanitaria-valenciana/</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="5" t="inlineStr">
+        <is>
+          <t>Johns Hopkins Proton Therapy Center (Johns Hopkins Medicine)</t>
+        </is>
+      </c>
+      <c r="B379" s="5" t="inlineStr">
+        <is>
+          <t>Clínica Universidad de Navarra (Cancer Center) and Facultad de Medicina, Universidad de Navarra</t>
+        </is>
+      </c>
+      <c r="C379" s="5" t="inlineStr">
+        <is>
+          <t>Clínica Universidad de Navarra La Clínica Universidad de Navarra y Johns Hopkins se alían para impulsar la formación en protonterapia en España</t>
+        </is>
+      </c>
+      <c r="D379" s="5" t="inlineStr">
+        <is>
+          <t>2023-10-09</t>
+        </is>
+      </c>
+      <c r="E379" s="5" t="inlineStr">
+        <is>
+          <t>https://cancercenter.cun.es/noticias/clinica-universidad-navarra-johns-hopkins-alian-impulsar-formacion-protonterapia-espana</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="5" t="inlineStr">
+        <is>
+          <t>Hospital de Amor (Barretos Cancer Hospital)</t>
+        </is>
+      </c>
+      <c r="B380" s="5" t="inlineStr">
+        <is>
+          <t>Hospital Sant Joan de Déu Barcelona (SJD Barcelona Children's Hospital)</t>
+        </is>
+      </c>
+      <c r="C380" s="5" t="inlineStr">
+        <is>
+          <t>Hospital Sant Joan de Déu Barcelona SJD Barcelona Children's Hospital and the Brazilian cancer hospital in Barretos sign a collaboration agreement</t>
+        </is>
+      </c>
+      <c r="D380" s="5" t="inlineStr">
+        <is>
+          <t>2021-07-13</t>
+        </is>
+      </c>
+      <c r="E380" s="5" t="inlineStr">
+        <is>
+          <t>https://www.sjdhospitalbarcelona.org/en/news/sjd-barcelona-childrens-hospital-brazilian-cancer-hospital-barretos-sign-collaboration-agreement</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="5" t="inlineStr">
+        <is>
+          <t>Fresenius Helios (Helios Health)</t>
+        </is>
+      </c>
+      <c r="B381" s="5" t="inlineStr">
+        <is>
+          <t>Eugin Group (fertility clinics)</t>
+        </is>
+      </c>
+      <c r="C381" s="5" t="inlineStr">
+        <is>
+          <t>Fresenius SE &amp; Co. KGaA Fresenius Helios acquires Eugin Group</t>
+        </is>
+      </c>
+      <c r="D381" s="5" t="inlineStr">
+        <is>
+          <t>2020-12-21</t>
+        </is>
+      </c>
+      <c r="E381" s="5" t="inlineStr">
+        <is>
+          <t>https://www.fresenius.com/sites/default/files/2021-11/FSE_Helios_Acquisition_Eugin_e.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="5" t="inlineStr">
+        <is>
+          <t>Fresenius Helios (Helios Health)</t>
+        </is>
+      </c>
+      <c r="B382" s="5" t="inlineStr">
+        <is>
+          <t>Eugin Group (fertility clinics)</t>
+        </is>
+      </c>
+      <c r="C382" s="5" t="inlineStr">
+        <is>
+          <t>Fresenius SE &amp; Co. KGaA Fresenius successfully completes divestment of fertility services group Eugin</t>
+        </is>
+      </c>
+      <c r="D382" s="5" t="inlineStr">
+        <is>
+          <t>2024-01-31</t>
+        </is>
+      </c>
+      <c r="E382" s="5" t="inlineStr">
+        <is>
+          <t>https://www.fresenius.com/sites/default/files/2024-01/20240131_FSE_Press_Release_ClosingEugin.pdf</t>
         </is>
       </c>
     </row>
@@ -19544,6 +22335,60 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E326" r:id="rId325"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E327" r:id="rId326"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E328" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E329" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E330" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E331" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E332" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E333" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E334" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E335" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E336" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E337" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E338" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E339" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E340" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E341" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E342" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E343" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E344" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E345" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E346" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E347" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E348" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E349" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E350" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E351" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E352" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E353" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E354" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E355" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E356" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E357" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E358" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E359" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E360" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E361" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E362" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E363" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E364" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E365" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E366" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E367" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E368" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E369" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E370" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E371" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E372" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E373" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E374" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E375" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E376" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E377" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E378" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E379" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E380" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E381" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E382" r:id="rId381"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>